<commit_message>
chore(holomap): maj gabarit — ponts abaissés à 1 m (calque Surélevé)
L'auteur a abaissé l'altitude des 3 ponts (2 m -> 1 m) et décalé un pont d'une
rangée. Le lecteur runtime reprend la maj automatiquement ; rendu vérifié (tablier
juste au-dessus de l'eau). TestHoloXlsx : altitude assertée « faible (1-4 m) »
plutôt qu'une valeur exacte, pour rester valide quand l'auteur ajuste.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Carte Holo/carte_holomap.xlsx
+++ b/Carte Holo/carte_holomap.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\benja\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Projets\IdleEvolution\Carte Holo\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{2726FBA3-6C90-4C7D-9586-5B15ED7C3D08}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{88F874DD-C4C0-4240-B0E9-950199932A78}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -21,7 +21,6 @@
     <sheet name="Ouvrages d'art" sheetId="6" r:id="rId6"/>
   </sheets>
   <calcPr calcId="191029"/>
-  <fileRecoveryPr repairLoad="1"/>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <xcalcf:calcFeatures>
@@ -1328,23 +1327,6 @@
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="9" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="10" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="9" borderId="11" xfId="0" applyFill="1" applyBorder="1"/>
@@ -1398,6 +1380,23 @@
     <xf numFmtId="0" fontId="0" fillId="8" borderId="45" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="9" borderId="46" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="9" borderId="20" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1709,11 +1708,11 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="A1" s="30" t="s">
+      <c r="A1" s="85" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="31"/>
-      <c r="C1" s="31"/>
+      <c r="B1" s="84"/>
+      <c r="C1" s="84"/>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
@@ -1771,11 +1770,11 @@
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A9" s="32" t="s">
+      <c r="A9" s="86" t="s">
         <v>13</v>
       </c>
-      <c r="B9" s="31"/>
-      <c r="C9" s="31"/>
+      <c r="B9" s="84"/>
+      <c r="C9" s="84"/>
     </row>
   </sheetData>
   <mergeCells count="2">
@@ -2286,10 +2285,10 @@
       <c r="AP6" s="7"/>
       <c r="AQ6" s="7"/>
       <c r="AR6" s="7"/>
-      <c r="AS6" s="39"/>
-      <c r="AT6" s="39"/>
-      <c r="AU6" s="39"/>
-      <c r="AV6" s="39"/>
+      <c r="AS6" s="30"/>
+      <c r="AT6" s="30"/>
+      <c r="AU6" s="30"/>
+      <c r="AV6" s="30"/>
       <c r="AW6" s="7"/>
       <c r="AX6" s="7"/>
       <c r="AY6" s="7"/>
@@ -2350,12 +2349,12 @@
       <c r="AO7" s="7"/>
       <c r="AP7" s="7"/>
       <c r="AQ7" s="7"/>
-      <c r="AR7" s="40"/>
-      <c r="AS7" s="41"/>
-      <c r="AT7" s="42"/>
-      <c r="AU7" s="42"/>
-      <c r="AV7" s="43"/>
-      <c r="AW7" s="44"/>
+      <c r="AR7" s="31"/>
+      <c r="AS7" s="32"/>
+      <c r="AT7" s="33"/>
+      <c r="AU7" s="33"/>
+      <c r="AV7" s="34"/>
+      <c r="AW7" s="35"/>
       <c r="AX7" s="7"/>
       <c r="AY7" s="7"/>
       <c r="AZ7" s="7"/>
@@ -2415,14 +2414,14 @@
       <c r="AO8" s="7"/>
       <c r="AP8" s="7"/>
       <c r="AQ8" s="7"/>
-      <c r="AR8" s="40"/>
-      <c r="AS8" s="45"/>
+      <c r="AR8" s="31"/>
+      <c r="AS8" s="36"/>
       <c r="AT8" s="15" t="s">
         <v>135</v>
       </c>
       <c r="AU8" s="15"/>
-      <c r="AV8" s="46"/>
-      <c r="AW8" s="44"/>
+      <c r="AV8" s="37"/>
+      <c r="AW8" s="35"/>
       <c r="AX8" s="7"/>
       <c r="AY8" s="7"/>
       <c r="AZ8" s="7"/>
@@ -2482,12 +2481,12 @@
       <c r="AO9" s="15"/>
       <c r="AP9" s="15"/>
       <c r="AQ9" s="15"/>
-      <c r="AR9" s="47"/>
-      <c r="AS9" s="45"/>
+      <c r="AR9" s="38"/>
+      <c r="AS9" s="36"/>
       <c r="AT9" s="15"/>
       <c r="AU9" s="15"/>
-      <c r="AV9" s="46"/>
-      <c r="AW9" s="44"/>
+      <c r="AV9" s="37"/>
+      <c r="AW9" s="35"/>
       <c r="AX9" s="7"/>
       <c r="AY9" s="7"/>
       <c r="AZ9" s="7"/>
@@ -2547,12 +2546,12 @@
       <c r="AO10" s="7"/>
       <c r="AP10" s="7"/>
       <c r="AQ10" s="7"/>
-      <c r="AR10" s="40"/>
-      <c r="AS10" s="48"/>
-      <c r="AT10" s="49"/>
-      <c r="AU10" s="49"/>
-      <c r="AV10" s="50"/>
-      <c r="AW10" s="44"/>
+      <c r="AR10" s="31"/>
+      <c r="AS10" s="39"/>
+      <c r="AT10" s="40"/>
+      <c r="AU10" s="40"/>
+      <c r="AV10" s="41"/>
+      <c r="AW10" s="35"/>
       <c r="AX10" s="7"/>
       <c r="AY10" s="7"/>
       <c r="AZ10" s="7"/>
@@ -2613,10 +2612,10 @@
       <c r="AP11" s="7"/>
       <c r="AQ11" s="7"/>
       <c r="AR11" s="7"/>
-      <c r="AS11" s="51"/>
-      <c r="AT11" s="51"/>
-      <c r="AU11" s="51"/>
-      <c r="AV11" s="51"/>
+      <c r="AS11" s="42"/>
+      <c r="AT11" s="42"/>
+      <c r="AU11" s="42"/>
+      <c r="AV11" s="42"/>
       <c r="AW11" s="7"/>
       <c r="AX11" s="7"/>
       <c r="AY11" s="7"/>
@@ -3436,10 +3435,10 @@
       <c r="T24" s="14"/>
       <c r="U24" s="14"/>
       <c r="V24" s="14"/>
-      <c r="W24" s="52"/>
-      <c r="X24" s="52"/>
-      <c r="Y24" s="52"/>
-      <c r="Z24" s="52"/>
+      <c r="W24" s="43"/>
+      <c r="X24" s="43"/>
+      <c r="Y24" s="43"/>
+      <c r="Z24" s="43"/>
       <c r="AA24" s="14"/>
       <c r="AB24" s="14"/>
       <c r="AC24" s="14"/>
@@ -3500,12 +3499,12 @@
       <c r="S25" s="12"/>
       <c r="T25" s="12"/>
       <c r="U25" s="12"/>
-      <c r="V25" s="53"/>
-      <c r="W25" s="54"/>
-      <c r="X25" s="55"/>
-      <c r="Y25" s="56"/>
-      <c r="Z25" s="57"/>
-      <c r="AA25" s="57"/>
+      <c r="V25" s="44"/>
+      <c r="W25" s="45"/>
+      <c r="X25" s="46"/>
+      <c r="Y25" s="47"/>
+      <c r="Z25" s="48"/>
+      <c r="AA25" s="48"/>
       <c r="AB25" s="16"/>
       <c r="AC25" s="16"/>
       <c r="AD25" s="14"/>
@@ -3557,20 +3556,20 @@
       <c r="K26" s="7"/>
       <c r="L26" s="7"/>
       <c r="M26" s="14"/>
-      <c r="N26" s="52"/>
-      <c r="O26" s="52"/>
+      <c r="N26" s="43"/>
+      <c r="O26" s="43"/>
       <c r="P26" s="14"/>
       <c r="Q26" s="14"/>
       <c r="R26" s="12"/>
       <c r="S26" s="12"/>
       <c r="T26" s="16"/>
       <c r="U26" s="16"/>
-      <c r="V26" s="58"/>
-      <c r="W26" s="59"/>
+      <c r="V26" s="49"/>
+      <c r="W26" s="50"/>
       <c r="X26" s="16"/>
-      <c r="Y26" s="60"/>
-      <c r="Z26" s="57"/>
-      <c r="AA26" s="57"/>
+      <c r="Y26" s="51"/>
+      <c r="Z26" s="48"/>
+      <c r="AA26" s="48"/>
       <c r="AB26" s="16"/>
       <c r="AC26" s="16"/>
       <c r="AD26" s="14"/>
@@ -3621,21 +3620,21 @@
       <c r="J27" s="7"/>
       <c r="K27" s="7"/>
       <c r="L27" s="7"/>
-      <c r="M27" s="61"/>
-      <c r="N27" s="62"/>
-      <c r="O27" s="63"/>
-      <c r="P27" s="64"/>
+      <c r="M27" s="52"/>
+      <c r="N27" s="53"/>
+      <c r="O27" s="54"/>
+      <c r="P27" s="55"/>
       <c r="Q27" s="14"/>
       <c r="R27" s="16"/>
       <c r="S27" s="16"/>
       <c r="T27" s="16"/>
       <c r="U27" s="12"/>
-      <c r="V27" s="58"/>
-      <c r="W27" s="65"/>
-      <c r="X27" s="66"/>
-      <c r="Y27" s="67"/>
-      <c r="Z27" s="57"/>
-      <c r="AA27" s="64"/>
+      <c r="V27" s="49"/>
+      <c r="W27" s="56"/>
+      <c r="X27" s="57"/>
+      <c r="Y27" s="58"/>
+      <c r="Z27" s="48"/>
+      <c r="AA27" s="55"/>
       <c r="AB27" s="14"/>
       <c r="AC27" s="14"/>
       <c r="AD27" s="14"/>
@@ -3686,27 +3685,27 @@
       <c r="J28" s="7"/>
       <c r="K28" s="7"/>
       <c r="L28" s="14"/>
-      <c r="M28" s="68"/>
-      <c r="N28" s="69"/>
-      <c r="O28" s="70"/>
-      <c r="P28" s="64"/>
+      <c r="M28" s="59"/>
+      <c r="N28" s="60"/>
+      <c r="O28" s="61"/>
+      <c r="P28" s="55"/>
       <c r="Q28" s="14"/>
       <c r="R28" s="12"/>
       <c r="S28" s="12"/>
       <c r="T28" s="16"/>
       <c r="U28" s="12"/>
       <c r="V28" s="12"/>
-      <c r="W28" s="71"/>
-      <c r="X28" s="71"/>
-      <c r="Y28" s="71"/>
-      <c r="Z28" s="71"/>
+      <c r="W28" s="62"/>
+      <c r="X28" s="62"/>
+      <c r="Y28" s="62"/>
+      <c r="Z28" s="62"/>
       <c r="AA28" s="14"/>
       <c r="AB28" s="14"/>
-      <c r="AC28" s="52"/>
-      <c r="AD28" s="52"/>
-      <c r="AE28" s="52"/>
-      <c r="AF28" s="52"/>
-      <c r="AG28" s="52"/>
+      <c r="AC28" s="43"/>
+      <c r="AD28" s="43"/>
+      <c r="AE28" s="43"/>
+      <c r="AF28" s="43"/>
+      <c r="AG28" s="43"/>
       <c r="AH28" s="14"/>
       <c r="AI28" s="14"/>
       <c r="AJ28" s="7"/>
@@ -3750,11 +3749,11 @@
       <c r="I29" s="7"/>
       <c r="J29" s="7"/>
       <c r="K29" s="7"/>
-      <c r="L29" s="61"/>
-      <c r="M29" s="72"/>
-      <c r="N29" s="73"/>
-      <c r="O29" s="74"/>
-      <c r="P29" s="64"/>
+      <c r="L29" s="52"/>
+      <c r="M29" s="63"/>
+      <c r="N29" s="64"/>
+      <c r="O29" s="65"/>
+      <c r="P29" s="55"/>
       <c r="Q29" s="14"/>
       <c r="R29" s="12"/>
       <c r="S29" s="12"/>
@@ -3766,13 +3765,13 @@
       <c r="Y29" s="16"/>
       <c r="Z29" s="16"/>
       <c r="AA29" s="14"/>
-      <c r="AB29" s="75"/>
-      <c r="AC29" s="76"/>
-      <c r="AD29" s="77"/>
-      <c r="AE29" s="77"/>
-      <c r="AF29" s="77"/>
-      <c r="AG29" s="78"/>
-      <c r="AH29" s="64"/>
+      <c r="AB29" s="66"/>
+      <c r="AC29" s="67"/>
+      <c r="AD29" s="68"/>
+      <c r="AE29" s="68"/>
+      <c r="AF29" s="68"/>
+      <c r="AG29" s="69"/>
+      <c r="AH29" s="55"/>
       <c r="AI29" s="14"/>
       <c r="AJ29" s="7"/>
       <c r="AK29" s="7"/>
@@ -3816,9 +3815,9 @@
       <c r="J30" s="7"/>
       <c r="K30" s="7"/>
       <c r="L30" s="14"/>
-      <c r="M30" s="79"/>
-      <c r="N30" s="79"/>
-      <c r="O30" s="79"/>
+      <c r="M30" s="70"/>
+      <c r="N30" s="70"/>
+      <c r="O30" s="70"/>
       <c r="P30" s="14"/>
       <c r="Q30" s="14"/>
       <c r="R30" s="12"/>
@@ -3831,13 +3830,13 @@
       <c r="Y30" s="16"/>
       <c r="Z30" s="16"/>
       <c r="AA30" s="14"/>
-      <c r="AB30" s="75"/>
-      <c r="AC30" s="80"/>
+      <c r="AB30" s="66"/>
+      <c r="AC30" s="71"/>
       <c r="AD30" s="12"/>
       <c r="AE30" s="12"/>
       <c r="AF30" s="12"/>
-      <c r="AG30" s="81"/>
-      <c r="AH30" s="64"/>
+      <c r="AG30" s="72"/>
+      <c r="AH30" s="55"/>
       <c r="AI30" s="14"/>
       <c r="AJ30" s="7"/>
       <c r="AK30" s="7"/>
@@ -3896,15 +3895,15 @@
       <c r="Y31" s="16"/>
       <c r="Z31" s="16"/>
       <c r="AA31" s="14"/>
-      <c r="AB31" s="75"/>
-      <c r="AC31" s="80"/>
+      <c r="AB31" s="66"/>
+      <c r="AC31" s="71"/>
       <c r="AD31" s="12"/>
       <c r="AE31" s="12" t="s">
         <v>136</v>
       </c>
       <c r="AF31" s="12"/>
-      <c r="AG31" s="81"/>
-      <c r="AH31" s="64"/>
+      <c r="AG31" s="72"/>
+      <c r="AH31" s="55"/>
       <c r="AI31" s="14"/>
       <c r="AJ31" s="16"/>
       <c r="AK31" s="16"/>
@@ -3963,13 +3962,13 @@
       <c r="Y32" s="16"/>
       <c r="Z32" s="16"/>
       <c r="AA32" s="14"/>
-      <c r="AB32" s="75"/>
-      <c r="AC32" s="80"/>
+      <c r="AB32" s="66"/>
+      <c r="AC32" s="71"/>
       <c r="AD32" s="12"/>
       <c r="AE32" s="12"/>
       <c r="AF32" s="12"/>
-      <c r="AG32" s="81"/>
-      <c r="AH32" s="64"/>
+      <c r="AG32" s="72"/>
+      <c r="AH32" s="55"/>
       <c r="AI32" s="14"/>
       <c r="AJ32" s="16"/>
       <c r="AK32" s="16"/>
@@ -4028,13 +4027,13 @@
       <c r="Y33" s="16"/>
       <c r="Z33" s="16"/>
       <c r="AA33" s="14"/>
-      <c r="AB33" s="75"/>
-      <c r="AC33" s="82"/>
-      <c r="AD33" s="83"/>
-      <c r="AE33" s="83"/>
-      <c r="AF33" s="83"/>
-      <c r="AG33" s="84"/>
-      <c r="AH33" s="64"/>
+      <c r="AB33" s="66"/>
+      <c r="AC33" s="73"/>
+      <c r="AD33" s="74"/>
+      <c r="AE33" s="74"/>
+      <c r="AF33" s="74"/>
+      <c r="AG33" s="75"/>
+      <c r="AH33" s="55"/>
       <c r="AI33" s="14"/>
       <c r="AJ33" s="16"/>
       <c r="AK33" s="16"/>
@@ -4094,11 +4093,11 @@
       <c r="Z34" s="14"/>
       <c r="AA34" s="14"/>
       <c r="AB34" s="14"/>
-      <c r="AC34" s="79"/>
-      <c r="AD34" s="79"/>
-      <c r="AE34" s="79"/>
-      <c r="AF34" s="79"/>
-      <c r="AG34" s="79"/>
+      <c r="AC34" s="70"/>
+      <c r="AD34" s="70"/>
+      <c r="AE34" s="70"/>
+      <c r="AF34" s="70"/>
+      <c r="AG34" s="70"/>
       <c r="AH34" s="14"/>
       <c r="AI34" s="14"/>
       <c r="AJ34" s="14"/>
@@ -4159,12 +4158,12 @@
       <c r="Z35" s="14"/>
       <c r="AA35" s="14"/>
       <c r="AB35" s="14"/>
-      <c r="AC35" s="85"/>
-      <c r="AD35" s="85"/>
-      <c r="AE35" s="85"/>
-      <c r="AF35" s="85"/>
-      <c r="AG35" s="85"/>
-      <c r="AH35" s="85"/>
+      <c r="AC35" s="76"/>
+      <c r="AD35" s="76"/>
+      <c r="AE35" s="76"/>
+      <c r="AF35" s="76"/>
+      <c r="AG35" s="76"/>
+      <c r="AH35" s="76"/>
       <c r="AI35" s="14"/>
       <c r="AJ35" s="14"/>
       <c r="AK35" s="14"/>
@@ -4223,14 +4222,14 @@
       <c r="Y36" s="16"/>
       <c r="Z36" s="16"/>
       <c r="AA36" s="14"/>
-      <c r="AB36" s="86"/>
-      <c r="AC36" s="87"/>
-      <c r="AD36" s="88"/>
-      <c r="AE36" s="88"/>
-      <c r="AF36" s="88"/>
-      <c r="AG36" s="88"/>
-      <c r="AH36" s="78"/>
-      <c r="AI36" s="64"/>
+      <c r="AB36" s="77"/>
+      <c r="AC36" s="78"/>
+      <c r="AD36" s="79"/>
+      <c r="AE36" s="79"/>
+      <c r="AF36" s="79"/>
+      <c r="AG36" s="79"/>
+      <c r="AH36" s="69"/>
+      <c r="AI36" s="55"/>
       <c r="AJ36" s="16"/>
       <c r="AK36" s="16"/>
       <c r="AL36" s="16"/>
@@ -4288,16 +4287,16 @@
       <c r="Y37" s="16"/>
       <c r="Z37" s="16"/>
       <c r="AA37" s="14"/>
-      <c r="AB37" s="86"/>
-      <c r="AC37" s="89"/>
+      <c r="AB37" s="77"/>
+      <c r="AC37" s="80"/>
       <c r="AD37" s="12"/>
       <c r="AE37" s="12"/>
       <c r="AF37" s="12" t="s">
         <v>137</v>
       </c>
       <c r="AG37" s="12"/>
-      <c r="AH37" s="81"/>
-      <c r="AI37" s="64"/>
+      <c r="AH37" s="72"/>
+      <c r="AI37" s="55"/>
       <c r="AJ37" s="16"/>
       <c r="AK37" s="16"/>
       <c r="AL37" s="16"/>
@@ -4356,13 +4355,13 @@
       <c r="Z38" s="16"/>
       <c r="AA38" s="14"/>
       <c r="AB38" s="14"/>
-      <c r="AC38" s="90"/>
-      <c r="AD38" s="89"/>
+      <c r="AC38" s="81"/>
+      <c r="AD38" s="80"/>
       <c r="AE38" s="12"/>
       <c r="AF38" s="12"/>
       <c r="AG38" s="12"/>
-      <c r="AH38" s="81"/>
-      <c r="AI38" s="64"/>
+      <c r="AH38" s="72"/>
+      <c r="AI38" s="55"/>
       <c r="AJ38" s="16"/>
       <c r="AK38" s="16"/>
       <c r="AL38" s="16"/>
@@ -4422,12 +4421,12 @@
       <c r="AA39" s="14"/>
       <c r="AB39" s="14"/>
       <c r="AC39" s="15"/>
-      <c r="AD39" s="90"/>
-      <c r="AE39" s="89"/>
+      <c r="AD39" s="81"/>
+      <c r="AE39" s="80"/>
       <c r="AF39" s="12"/>
       <c r="AG39" s="12"/>
-      <c r="AH39" s="81"/>
-      <c r="AI39" s="64"/>
+      <c r="AH39" s="72"/>
+      <c r="AI39" s="55"/>
       <c r="AJ39" s="7"/>
       <c r="AK39" s="7"/>
       <c r="AL39" s="7"/>
@@ -4488,11 +4487,11 @@
       <c r="AB40" s="14"/>
       <c r="AC40" s="12"/>
       <c r="AD40" s="15"/>
-      <c r="AE40" s="90"/>
-      <c r="AF40" s="89"/>
-      <c r="AG40" s="83"/>
-      <c r="AH40" s="84"/>
-      <c r="AI40" s="64"/>
+      <c r="AE40" s="81"/>
+      <c r="AF40" s="80"/>
+      <c r="AG40" s="74"/>
+      <c r="AH40" s="75"/>
+      <c r="AI40" s="55"/>
       <c r="AJ40" s="7"/>
       <c r="AK40" s="7"/>
       <c r="AL40" s="7"/>
@@ -4555,8 +4554,8 @@
       <c r="AD41" s="15"/>
       <c r="AE41" s="15"/>
       <c r="AF41" s="15"/>
-      <c r="AG41" s="91"/>
-      <c r="AH41" s="91"/>
+      <c r="AG41" s="82"/>
+      <c r="AH41" s="82"/>
       <c r="AI41" s="14"/>
       <c r="AJ41" s="14"/>
       <c r="AK41" s="14"/>
@@ -8188,7 +8187,7 @@
       <c r="U34" s="8"/>
       <c r="V34" s="11"/>
       <c r="W34" s="11">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="X34" s="11"/>
       <c r="Y34" s="8"/>
@@ -8513,9 +8512,11 @@
       <c r="S39" s="8"/>
       <c r="T39" s="8"/>
       <c r="U39" s="8"/>
-      <c r="V39" s="8"/>
-      <c r="W39" s="8"/>
-      <c r="X39" s="8"/>
+      <c r="V39" s="11"/>
+      <c r="W39" s="11">
+        <v>1</v>
+      </c>
+      <c r="X39" s="11"/>
       <c r="Y39" s="8"/>
       <c r="Z39" s="8"/>
       <c r="AA39" s="8"/>
@@ -8578,11 +8579,9 @@
       <c r="S40" s="8"/>
       <c r="T40" s="8"/>
       <c r="U40" s="8"/>
-      <c r="V40" s="11"/>
-      <c r="W40" s="11">
-        <v>2</v>
-      </c>
-      <c r="X40" s="11"/>
+      <c r="V40" s="8"/>
+      <c r="W40" s="8"/>
+      <c r="X40" s="8"/>
       <c r="Y40" s="8"/>
       <c r="Z40" s="8"/>
       <c r="AA40" s="8"/>
@@ -8979,7 +8978,7 @@
       <c r="AB46" s="8"/>
       <c r="AC46" s="11"/>
       <c r="AD46" s="11">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="AE46" s="11"/>
       <c r="AF46" s="8"/>
@@ -9989,50 +9988,50 @@
       <c r="BI61" s="8"/>
     </row>
     <row r="63" spans="1:61" x14ac:dyDescent="0.25">
-      <c r="A63" s="33" t="s">
+      <c r="A63" s="83" t="s">
         <v>15</v>
       </c>
-      <c r="B63" s="31"/>
-      <c r="C63" s="31"/>
-      <c r="D63" s="31"/>
-      <c r="E63" s="31"/>
-      <c r="F63" s="31"/>
-      <c r="G63" s="31"/>
-      <c r="H63" s="31"/>
-      <c r="I63" s="31"/>
-      <c r="J63" s="31"/>
-      <c r="K63" s="31"/>
-      <c r="L63" s="31"/>
-      <c r="M63" s="31"/>
-      <c r="N63" s="31"/>
-      <c r="O63" s="31"/>
-      <c r="P63" s="31"/>
-      <c r="Q63" s="31"/>
-      <c r="R63" s="31"/>
-      <c r="S63" s="31"/>
-      <c r="T63" s="31"/>
+      <c r="B63" s="84"/>
+      <c r="C63" s="84"/>
+      <c r="D63" s="84"/>
+      <c r="E63" s="84"/>
+      <c r="F63" s="84"/>
+      <c r="G63" s="84"/>
+      <c r="H63" s="84"/>
+      <c r="I63" s="84"/>
+      <c r="J63" s="84"/>
+      <c r="K63" s="84"/>
+      <c r="L63" s="84"/>
+      <c r="M63" s="84"/>
+      <c r="N63" s="84"/>
+      <c r="O63" s="84"/>
+      <c r="P63" s="84"/>
+      <c r="Q63" s="84"/>
+      <c r="R63" s="84"/>
+      <c r="S63" s="84"/>
+      <c r="T63" s="84"/>
     </row>
     <row r="64" spans="1:61" ht="81.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A64" s="31"/>
-      <c r="B64" s="31"/>
-      <c r="C64" s="31"/>
-      <c r="D64" s="31"/>
-      <c r="E64" s="31"/>
-      <c r="F64" s="31"/>
-      <c r="G64" s="31"/>
-      <c r="H64" s="31"/>
-      <c r="I64" s="31"/>
-      <c r="J64" s="31"/>
-      <c r="K64" s="31"/>
-      <c r="L64" s="31"/>
-      <c r="M64" s="31"/>
-      <c r="N64" s="31"/>
-      <c r="O64" s="31"/>
-      <c r="P64" s="31"/>
-      <c r="Q64" s="31"/>
-      <c r="R64" s="31"/>
-      <c r="S64" s="31"/>
-      <c r="T64" s="31"/>
+      <c r="A64" s="84"/>
+      <c r="B64" s="84"/>
+      <c r="C64" s="84"/>
+      <c r="D64" s="84"/>
+      <c r="E64" s="84"/>
+      <c r="F64" s="84"/>
+      <c r="G64" s="84"/>
+      <c r="H64" s="84"/>
+      <c r="I64" s="84"/>
+      <c r="J64" s="84"/>
+      <c r="K64" s="84"/>
+      <c r="L64" s="84"/>
+      <c r="M64" s="84"/>
+      <c r="N64" s="84"/>
+      <c r="O64" s="84"/>
+      <c r="P64" s="84"/>
+      <c r="Q64" s="84"/>
+      <c r="R64" s="84"/>
+      <c r="S64" s="84"/>
+      <c r="T64" s="84"/>
     </row>
     <row r="66" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B66" s="9"/>
@@ -10065,26 +10064,26 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:4" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="A1" s="30" t="s">
+      <c r="A1" s="85" t="s">
         <v>16</v>
       </c>
-      <c r="B1" s="31"/>
-      <c r="C1" s="31"/>
-      <c r="D1" s="31"/>
+      <c r="B1" s="84"/>
+      <c r="C1" s="84"/>
+      <c r="D1" s="84"/>
     </row>
     <row r="3" spans="1:4" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="36" t="s">
+      <c r="A3" s="90" t="s">
         <v>17</v>
       </c>
-      <c r="B3" s="31"/>
-      <c r="C3" s="31"/>
-      <c r="D3" s="31"/>
+      <c r="B3" s="84"/>
+      <c r="C3" s="84"/>
+      <c r="D3" s="84"/>
     </row>
     <row r="4" spans="1:4" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="31"/>
-      <c r="B4" s="31"/>
-      <c r="C4" s="31"/>
-      <c r="D4" s="31"/>
+      <c r="A4" s="84"/>
+      <c r="B4" s="84"/>
+      <c r="C4" s="84"/>
+      <c r="D4" s="84"/>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A6" s="1" t="s">
@@ -10101,12 +10100,12 @@
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A7" s="37" t="s">
+      <c r="A7" s="89" t="s">
         <v>22</v>
       </c>
-      <c r="B7" s="31"/>
-      <c r="C7" s="31"/>
-      <c r="D7" s="31"/>
+      <c r="B7" s="84"/>
+      <c r="C7" s="84"/>
+      <c r="D7" s="84"/>
     </row>
     <row r="8" spans="1:4" ht="24" x14ac:dyDescent="0.25">
       <c r="A8" s="12"/>
@@ -10169,20 +10168,20 @@
       </c>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A13" s="34" t="s">
+      <c r="A13" s="91" t="s">
         <v>34</v>
       </c>
-      <c r="B13" s="31"/>
-      <c r="C13" s="31"/>
-      <c r="D13" s="31"/>
+      <c r="B13" s="84"/>
+      <c r="C13" s="84"/>
+      <c r="D13" s="84"/>
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A15" s="37" t="s">
+      <c r="A15" s="89" t="s">
         <v>35</v>
       </c>
-      <c r="B15" s="31"/>
-      <c r="C15" s="31"/>
-      <c r="D15" s="31"/>
+      <c r="B15" s="84"/>
+      <c r="C15" s="84"/>
+      <c r="D15" s="84"/>
     </row>
     <row r="16" spans="1:4" ht="24" x14ac:dyDescent="0.25">
       <c r="A16" s="17"/>
@@ -10257,346 +10256,350 @@
       </c>
     </row>
     <row r="22" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A22" s="34" t="s">
+      <c r="A22" s="91" t="s">
         <v>49</v>
       </c>
-      <c r="B22" s="31"/>
-      <c r="C22" s="31"/>
-      <c r="D22" s="31"/>
+      <c r="B22" s="84"/>
+      <c r="C22" s="84"/>
+      <c r="D22" s="84"/>
     </row>
     <row r="26" spans="1:4" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A26" s="38" t="s">
+      <c r="A26" s="88" t="s">
         <v>50</v>
       </c>
-      <c r="B26" s="31"/>
-      <c r="C26" s="31"/>
-      <c r="D26" s="31"/>
+      <c r="B26" s="84"/>
+      <c r="C26" s="84"/>
+      <c r="D26" s="84"/>
     </row>
     <row r="27" spans="1:4" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A27" s="35" t="s">
+      <c r="A27" s="87" t="s">
         <v>51</v>
       </c>
-      <c r="B27" s="31"/>
-      <c r="C27" s="31"/>
-      <c r="D27" s="31"/>
+      <c r="B27" s="84"/>
+      <c r="C27" s="84"/>
+      <c r="D27" s="84"/>
     </row>
     <row r="28" spans="1:4" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A28" s="35" t="s">
+      <c r="A28" s="87" t="s">
         <v>52</v>
       </c>
-      <c r="B28" s="31"/>
-      <c r="C28" s="31"/>
-      <c r="D28" s="31"/>
+      <c r="B28" s="84"/>
+      <c r="C28" s="84"/>
+      <c r="D28" s="84"/>
     </row>
     <row r="29" spans="1:4" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A29" s="35" t="s">
+      <c r="A29" s="87" t="s">
         <v>53</v>
       </c>
-      <c r="B29" s="31"/>
-      <c r="C29" s="31"/>
-      <c r="D29" s="31"/>
+      <c r="B29" s="84"/>
+      <c r="C29" s="84"/>
+      <c r="D29" s="84"/>
     </row>
     <row r="30" spans="1:4" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A30" s="35" t="s">
+      <c r="A30" s="87" t="s">
         <v>54</v>
       </c>
-      <c r="B30" s="31"/>
-      <c r="C30" s="31"/>
-      <c r="D30" s="31"/>
+      <c r="B30" s="84"/>
+      <c r="C30" s="84"/>
+      <c r="D30" s="84"/>
     </row>
     <row r="31" spans="1:4" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A31" s="35" t="s">
+      <c r="A31" s="87" t="s">
         <v>55</v>
       </c>
-      <c r="B31" s="31"/>
-      <c r="C31" s="31"/>
-      <c r="D31" s="31"/>
+      <c r="B31" s="84"/>
+      <c r="C31" s="84"/>
+      <c r="D31" s="84"/>
     </row>
     <row r="32" spans="1:4" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A32" s="35" t="s">
+      <c r="A32" s="87" t="s">
         <v>56</v>
       </c>
-      <c r="B32" s="31"/>
-      <c r="C32" s="31"/>
-      <c r="D32" s="31"/>
+      <c r="B32" s="84"/>
+      <c r="C32" s="84"/>
+      <c r="D32" s="84"/>
     </row>
     <row r="33" spans="1:4" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A33" s="35" t="s">
+      <c r="A33" s="87" t="s">
         <v>57</v>
       </c>
-      <c r="B33" s="31"/>
-      <c r="C33" s="31"/>
-      <c r="D33" s="31"/>
+      <c r="B33" s="84"/>
+      <c r="C33" s="84"/>
+      <c r="D33" s="84"/>
     </row>
     <row r="34" spans="1:4" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A34" s="35" t="s">
+      <c r="A34" s="87" t="s">
         <v>58</v>
       </c>
-      <c r="B34" s="31"/>
-      <c r="C34" s="31"/>
-      <c r="D34" s="31"/>
+      <c r="B34" s="84"/>
+      <c r="C34" s="84"/>
+      <c r="D34" s="84"/>
     </row>
     <row r="35" spans="1:4" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A35" s="35" t="s">
+      <c r="A35" s="87" t="s">
         <v>59</v>
       </c>
-      <c r="B35" s="31"/>
-      <c r="C35" s="31"/>
-      <c r="D35" s="31"/>
+      <c r="B35" s="84"/>
+      <c r="C35" s="84"/>
+      <c r="D35" s="84"/>
     </row>
     <row r="36" spans="1:4" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A36" s="35"/>
-      <c r="B36" s="31"/>
-      <c r="C36" s="31"/>
-      <c r="D36" s="31"/>
+      <c r="A36" s="87"/>
+      <c r="B36" s="84"/>
+      <c r="C36" s="84"/>
+      <c r="D36" s="84"/>
     </row>
     <row r="37" spans="1:4" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A37" s="38" t="s">
+      <c r="A37" s="88" t="s">
         <v>60</v>
       </c>
-      <c r="B37" s="31"/>
-      <c r="C37" s="31"/>
-      <c r="D37" s="31"/>
+      <c r="B37" s="84"/>
+      <c r="C37" s="84"/>
+      <c r="D37" s="84"/>
     </row>
     <row r="38" spans="1:4" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A38" s="35" t="s">
+      <c r="A38" s="87" t="s">
         <v>61</v>
       </c>
-      <c r="B38" s="31"/>
-      <c r="C38" s="31"/>
-      <c r="D38" s="31"/>
+      <c r="B38" s="84"/>
+      <c r="C38" s="84"/>
+      <c r="D38" s="84"/>
     </row>
     <row r="39" spans="1:4" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A39" s="35" t="s">
+      <c r="A39" s="87" t="s">
         <v>62</v>
       </c>
-      <c r="B39" s="31"/>
-      <c r="C39" s="31"/>
-      <c r="D39" s="31"/>
+      <c r="B39" s="84"/>
+      <c r="C39" s="84"/>
+      <c r="D39" s="84"/>
     </row>
     <row r="40" spans="1:4" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A40" s="35" t="s">
+      <c r="A40" s="87" t="s">
         <v>63</v>
       </c>
-      <c r="B40" s="31"/>
-      <c r="C40" s="31"/>
-      <c r="D40" s="31"/>
+      <c r="B40" s="84"/>
+      <c r="C40" s="84"/>
+      <c r="D40" s="84"/>
     </row>
     <row r="41" spans="1:4" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A41" s="35" t="s">
+      <c r="A41" s="87" t="s">
         <v>64</v>
       </c>
-      <c r="B41" s="31"/>
-      <c r="C41" s="31"/>
-      <c r="D41" s="31"/>
+      <c r="B41" s="84"/>
+      <c r="C41" s="84"/>
+      <c r="D41" s="84"/>
     </row>
     <row r="42" spans="1:4" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A42" s="35" t="s">
+      <c r="A42" s="87" t="s">
         <v>65</v>
       </c>
-      <c r="B42" s="31"/>
-      <c r="C42" s="31"/>
-      <c r="D42" s="31"/>
+      <c r="B42" s="84"/>
+      <c r="C42" s="84"/>
+      <c r="D42" s="84"/>
     </row>
     <row r="43" spans="1:4" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A43" s="35" t="s">
+      <c r="A43" s="87" t="s">
         <v>66</v>
       </c>
-      <c r="B43" s="31"/>
-      <c r="C43" s="31"/>
-      <c r="D43" s="31"/>
+      <c r="B43" s="84"/>
+      <c r="C43" s="84"/>
+      <c r="D43" s="84"/>
     </row>
     <row r="44" spans="1:4" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A44" s="35"/>
-      <c r="B44" s="31"/>
-      <c r="C44" s="31"/>
-      <c r="D44" s="31"/>
+      <c r="A44" s="87"/>
+      <c r="B44" s="84"/>
+      <c r="C44" s="84"/>
+      <c r="D44" s="84"/>
     </row>
     <row r="45" spans="1:4" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A45" s="38" t="s">
+      <c r="A45" s="88" t="s">
         <v>67</v>
       </c>
-      <c r="B45" s="31"/>
-      <c r="C45" s="31"/>
-      <c r="D45" s="31"/>
+      <c r="B45" s="84"/>
+      <c r="C45" s="84"/>
+      <c r="D45" s="84"/>
     </row>
     <row r="46" spans="1:4" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A46" s="35" t="s">
+      <c r="A46" s="87" t="s">
         <v>68</v>
       </c>
-      <c r="B46" s="31"/>
-      <c r="C46" s="31"/>
-      <c r="D46" s="31"/>
+      <c r="B46" s="84"/>
+      <c r="C46" s="84"/>
+      <c r="D46" s="84"/>
     </row>
     <row r="47" spans="1:4" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A47" s="35" t="s">
+      <c r="A47" s="87" t="s">
         <v>69</v>
       </c>
-      <c r="B47" s="31"/>
-      <c r="C47" s="31"/>
-      <c r="D47" s="31"/>
+      <c r="B47" s="84"/>
+      <c r="C47" s="84"/>
+      <c r="D47" s="84"/>
     </row>
     <row r="48" spans="1:4" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A48" s="35" t="s">
+      <c r="A48" s="87" t="s">
         <v>70</v>
       </c>
-      <c r="B48" s="31"/>
-      <c r="C48" s="31"/>
-      <c r="D48" s="31"/>
+      <c r="B48" s="84"/>
+      <c r="C48" s="84"/>
+      <c r="D48" s="84"/>
     </row>
     <row r="49" spans="1:4" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A49" s="35" t="s">
+      <c r="A49" s="87" t="s">
         <v>71</v>
       </c>
-      <c r="B49" s="31"/>
-      <c r="C49" s="31"/>
-      <c r="D49" s="31"/>
+      <c r="B49" s="84"/>
+      <c r="C49" s="84"/>
+      <c r="D49" s="84"/>
     </row>
     <row r="50" spans="1:4" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A50" s="35"/>
-      <c r="B50" s="31"/>
-      <c r="C50" s="31"/>
-      <c r="D50" s="31"/>
+      <c r="A50" s="87"/>
+      <c r="B50" s="84"/>
+      <c r="C50" s="84"/>
+      <c r="D50" s="84"/>
     </row>
     <row r="51" spans="1:4" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A51" s="38" t="s">
+      <c r="A51" s="88" t="s">
         <v>72</v>
       </c>
-      <c r="B51" s="31"/>
-      <c r="C51" s="31"/>
-      <c r="D51" s="31"/>
+      <c r="B51" s="84"/>
+      <c r="C51" s="84"/>
+      <c r="D51" s="84"/>
     </row>
     <row r="52" spans="1:4" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A52" s="35" t="s">
+      <c r="A52" s="87" t="s">
         <v>73</v>
       </c>
-      <c r="B52" s="31"/>
-      <c r="C52" s="31"/>
-      <c r="D52" s="31"/>
+      <c r="B52" s="84"/>
+      <c r="C52" s="84"/>
+      <c r="D52" s="84"/>
     </row>
     <row r="53" spans="1:4" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A53" s="35" t="s">
+      <c r="A53" s="87" t="s">
         <v>74</v>
       </c>
-      <c r="B53" s="31"/>
-      <c r="C53" s="31"/>
-      <c r="D53" s="31"/>
+      <c r="B53" s="84"/>
+      <c r="C53" s="84"/>
+      <c r="D53" s="84"/>
     </row>
     <row r="54" spans="1:4" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A54" s="35" t="s">
+      <c r="A54" s="87" t="s">
         <v>75</v>
       </c>
-      <c r="B54" s="31"/>
-      <c r="C54" s="31"/>
-      <c r="D54" s="31"/>
+      <c r="B54" s="84"/>
+      <c r="C54" s="84"/>
+      <c r="D54" s="84"/>
     </row>
     <row r="55" spans="1:4" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A55" s="35" t="s">
+      <c r="A55" s="87" t="s">
         <v>76</v>
       </c>
-      <c r="B55" s="31"/>
-      <c r="C55" s="31"/>
-      <c r="D55" s="31"/>
+      <c r="B55" s="84"/>
+      <c r="C55" s="84"/>
+      <c r="D55" s="84"/>
     </row>
     <row r="56" spans="1:4" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A56" s="35" t="s">
+      <c r="A56" s="87" t="s">
         <v>77</v>
       </c>
-      <c r="B56" s="31"/>
-      <c r="C56" s="31"/>
-      <c r="D56" s="31"/>
+      <c r="B56" s="84"/>
+      <c r="C56" s="84"/>
+      <c r="D56" s="84"/>
     </row>
     <row r="57" spans="1:4" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A57" s="35" t="s">
+      <c r="A57" s="87" t="s">
         <v>78</v>
       </c>
-      <c r="B57" s="31"/>
-      <c r="C57" s="31"/>
-      <c r="D57" s="31"/>
+      <c r="B57" s="84"/>
+      <c r="C57" s="84"/>
+      <c r="D57" s="84"/>
     </row>
     <row r="58" spans="1:4" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A58" s="35" t="s">
+      <c r="A58" s="87" t="s">
         <v>79</v>
       </c>
-      <c r="B58" s="31"/>
-      <c r="C58" s="31"/>
-      <c r="D58" s="31"/>
+      <c r="B58" s="84"/>
+      <c r="C58" s="84"/>
+      <c r="D58" s="84"/>
     </row>
     <row r="59" spans="1:4" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A59" s="35"/>
-      <c r="B59" s="31"/>
-      <c r="C59" s="31"/>
-      <c r="D59" s="31"/>
+      <c r="A59" s="87"/>
+      <c r="B59" s="84"/>
+      <c r="C59" s="84"/>
+      <c r="D59" s="84"/>
     </row>
     <row r="60" spans="1:4" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A60" s="38" t="s">
+      <c r="A60" s="88" t="s">
         <v>80</v>
       </c>
-      <c r="B60" s="31"/>
-      <c r="C60" s="31"/>
-      <c r="D60" s="31"/>
+      <c r="B60" s="84"/>
+      <c r="C60" s="84"/>
+      <c r="D60" s="84"/>
     </row>
     <row r="61" spans="1:4" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A61" s="35" t="s">
+      <c r="A61" s="87" t="s">
         <v>81</v>
       </c>
-      <c r="B61" s="31"/>
-      <c r="C61" s="31"/>
-      <c r="D61" s="31"/>
+      <c r="B61" s="84"/>
+      <c r="C61" s="84"/>
+      <c r="D61" s="84"/>
     </row>
     <row r="62" spans="1:4" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A62" s="35" t="s">
+      <c r="A62" s="87" t="s">
         <v>82</v>
       </c>
-      <c r="B62" s="31"/>
-      <c r="C62" s="31"/>
-      <c r="D62" s="31"/>
+      <c r="B62" s="84"/>
+      <c r="C62" s="84"/>
+      <c r="D62" s="84"/>
     </row>
     <row r="63" spans="1:4" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A63" s="35" t="s">
+      <c r="A63" s="87" t="s">
         <v>83</v>
       </c>
-      <c r="B63" s="31"/>
-      <c r="C63" s="31"/>
-      <c r="D63" s="31"/>
+      <c r="B63" s="84"/>
+      <c r="C63" s="84"/>
+      <c r="D63" s="84"/>
     </row>
     <row r="64" spans="1:4" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A64" s="35" t="s">
+      <c r="A64" s="87" t="s">
         <v>84</v>
       </c>
-      <c r="B64" s="31"/>
-      <c r="C64" s="31"/>
-      <c r="D64" s="31"/>
+      <c r="B64" s="84"/>
+      <c r="C64" s="84"/>
+      <c r="D64" s="84"/>
     </row>
     <row r="65" spans="1:4" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A65" s="35" t="s">
+      <c r="A65" s="87" t="s">
         <v>85</v>
       </c>
-      <c r="B65" s="31"/>
-      <c r="C65" s="31"/>
-      <c r="D65" s="31"/>
+      <c r="B65" s="84"/>
+      <c r="C65" s="84"/>
+      <c r="D65" s="84"/>
     </row>
     <row r="66" spans="1:4" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A66" s="35" t="s">
+      <c r="A66" s="87" t="s">
         <v>86</v>
       </c>
-      <c r="B66" s="31"/>
-      <c r="C66" s="31"/>
-      <c r="D66" s="31"/>
+      <c r="B66" s="84"/>
+      <c r="C66" s="84"/>
+      <c r="D66" s="84"/>
     </row>
   </sheetData>
   <mergeCells count="47">
-    <mergeCell ref="A65:D65"/>
-    <mergeCell ref="A41:D41"/>
-    <mergeCell ref="A46:D46"/>
-    <mergeCell ref="A66:D66"/>
-    <mergeCell ref="A37:D37"/>
-    <mergeCell ref="A56:D56"/>
-    <mergeCell ref="A50:D50"/>
-    <mergeCell ref="A55:D55"/>
-    <mergeCell ref="A57:D57"/>
-    <mergeCell ref="A47:D47"/>
-    <mergeCell ref="A42:D42"/>
+    <mergeCell ref="A62:D62"/>
+    <mergeCell ref="A38:D38"/>
+    <mergeCell ref="A29:D29"/>
+    <mergeCell ref="A52:D52"/>
+    <mergeCell ref="A43:D43"/>
+    <mergeCell ref="A28:D28"/>
+    <mergeCell ref="A13:D13"/>
+    <mergeCell ref="A44:D44"/>
+    <mergeCell ref="A40:D40"/>
+    <mergeCell ref="A31:D31"/>
+    <mergeCell ref="A34:D34"/>
+    <mergeCell ref="A30:D30"/>
+    <mergeCell ref="A39:D39"/>
+    <mergeCell ref="A22:D22"/>
+    <mergeCell ref="A35:D35"/>
     <mergeCell ref="A1:D1"/>
     <mergeCell ref="A45:D45"/>
     <mergeCell ref="A61:D61"/>
@@ -10609,30 +10612,26 @@
     <mergeCell ref="A3:D4"/>
     <mergeCell ref="A15:D15"/>
     <mergeCell ref="A59:D59"/>
-    <mergeCell ref="A64:D64"/>
     <mergeCell ref="A49:D49"/>
     <mergeCell ref="A51:D51"/>
     <mergeCell ref="A60:D60"/>
     <mergeCell ref="A36:D36"/>
+    <mergeCell ref="A65:D65"/>
+    <mergeCell ref="A41:D41"/>
+    <mergeCell ref="A46:D46"/>
+    <mergeCell ref="A66:D66"/>
+    <mergeCell ref="A37:D37"/>
+    <mergeCell ref="A56:D56"/>
+    <mergeCell ref="A50:D50"/>
+    <mergeCell ref="A55:D55"/>
+    <mergeCell ref="A57:D57"/>
+    <mergeCell ref="A47:D47"/>
+    <mergeCell ref="A42:D42"/>
+    <mergeCell ref="A64:D64"/>
     <mergeCell ref="A63:D63"/>
-    <mergeCell ref="A28:D28"/>
-    <mergeCell ref="A13:D13"/>
-    <mergeCell ref="A44:D44"/>
-    <mergeCell ref="A40:D40"/>
-    <mergeCell ref="A31:D31"/>
     <mergeCell ref="A58:D58"/>
-    <mergeCell ref="A34:D34"/>
     <mergeCell ref="A48:D48"/>
-    <mergeCell ref="A30:D30"/>
-    <mergeCell ref="A39:D39"/>
-    <mergeCell ref="A22:D22"/>
     <mergeCell ref="A53:D53"/>
-    <mergeCell ref="A35:D35"/>
-    <mergeCell ref="A62:D62"/>
-    <mergeCell ref="A38:D38"/>
-    <mergeCell ref="A29:D29"/>
-    <mergeCell ref="A52:D52"/>
-    <mergeCell ref="A43:D43"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -11198,42 +11197,42 @@
       <c r="J39" s="29"/>
     </row>
     <row r="41" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A41" s="33" t="s">
+      <c r="A41" s="83" t="s">
         <v>117</v>
       </c>
-      <c r="B41" s="31"/>
-      <c r="C41" s="31"/>
-      <c r="D41" s="31"/>
-      <c r="E41" s="31"/>
-      <c r="F41" s="31"/>
-      <c r="G41" s="31"/>
-      <c r="H41" s="31"/>
-      <c r="I41" s="31"/>
-      <c r="J41" s="31"/>
+      <c r="B41" s="84"/>
+      <c r="C41" s="84"/>
+      <c r="D41" s="84"/>
+      <c r="E41" s="84"/>
+      <c r="F41" s="84"/>
+      <c r="G41" s="84"/>
+      <c r="H41" s="84"/>
+      <c r="I41" s="84"/>
+      <c r="J41" s="84"/>
     </row>
     <row r="42" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A42" s="31"/>
-      <c r="B42" s="31"/>
-      <c r="C42" s="31"/>
-      <c r="D42" s="31"/>
-      <c r="E42" s="31"/>
-      <c r="F42" s="31"/>
-      <c r="G42" s="31"/>
-      <c r="H42" s="31"/>
-      <c r="I42" s="31"/>
-      <c r="J42" s="31"/>
+      <c r="A42" s="84"/>
+      <c r="B42" s="84"/>
+      <c r="C42" s="84"/>
+      <c r="D42" s="84"/>
+      <c r="E42" s="84"/>
+      <c r="F42" s="84"/>
+      <c r="G42" s="84"/>
+      <c r="H42" s="84"/>
+      <c r="I42" s="84"/>
+      <c r="J42" s="84"/>
     </row>
     <row r="43" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A43" s="31"/>
-      <c r="B43" s="31"/>
-      <c r="C43" s="31"/>
-      <c r="D43" s="31"/>
-      <c r="E43" s="31"/>
-      <c r="F43" s="31"/>
-      <c r="G43" s="31"/>
-      <c r="H43" s="31"/>
-      <c r="I43" s="31"/>
-      <c r="J43" s="31"/>
+      <c r="A43" s="84"/>
+      <c r="B43" s="84"/>
+      <c r="C43" s="84"/>
+      <c r="D43" s="84"/>
+      <c r="E43" s="84"/>
+      <c r="F43" s="84"/>
+      <c r="G43" s="84"/>
+      <c r="H43" s="84"/>
+      <c r="I43" s="84"/>
+      <c r="J43" s="84"/>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -11529,24 +11528,24 @@
       <c r="G24" s="29"/>
     </row>
     <row r="26" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A26" s="33" t="s">
+      <c r="A26" s="83" t="s">
         <v>134</v>
       </c>
-      <c r="B26" s="31"/>
-      <c r="C26" s="31"/>
-      <c r="D26" s="31"/>
-      <c r="E26" s="31"/>
-      <c r="F26" s="31"/>
-      <c r="G26" s="31"/>
+      <c r="B26" s="84"/>
+      <c r="C26" s="84"/>
+      <c r="D26" s="84"/>
+      <c r="E26" s="84"/>
+      <c r="F26" s="84"/>
+      <c r="G26" s="84"/>
     </row>
     <row r="27" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A27" s="31"/>
-      <c r="B27" s="31"/>
-      <c r="C27" s="31"/>
-      <c r="D27" s="31"/>
-      <c r="E27" s="31"/>
-      <c r="F27" s="31"/>
-      <c r="G27" s="31"/>
+      <c r="A27" s="84"/>
+      <c r="B27" s="84"/>
+      <c r="C27" s="84"/>
+      <c r="D27" s="84"/>
+      <c r="E27" s="84"/>
+      <c r="F27" s="84"/>
+      <c r="G27" s="84"/>
     </row>
   </sheetData>
   <mergeCells count="1">

</xml_diff>

<commit_message>
feat(holomap3d): voirie typee par largeur + circulation directionnelle
Les routes sont decomposees en BANDES rectangulaires (rangees/colonnes contigues
de meme emprise) -> chaque bande connait son axe et sa largeur :
- largeur 1 = departementale (1 voie/sens), 2 = nationale (2 voies/sens),
  4 = autoroute (3 voies/sens) (_n_voies).
- marquage au sol : MEDIANE vive (double trait) separant les 2 sens + lignes de
  voie pointillees (nb selon le type).
- trafic DIRECTIONNEL par voie : chaussee A en sens - (ambre), chaussee B en
  sens + (cyan) -> le sens de circulation se lit. Densite selon la longueur.
- lampadaires reposes sur les bords EXTERIEURS des bandes (propre quelle que soit
  la largeur), remplace l'ancien placement par run.
Remplace les axes neon + le trafic bidirectionnel sur centerline.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Carte Holo/carte_holomap.xlsx
+++ b/Carte Holo/carte_holomap.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Projets\IdleEvolution\Carte Holo\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{88F874DD-C4C0-4240-B0E9-950199932A78}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DF2FD20E-2915-4C20-AAE5-6B41F4C86D1A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Paramètres" sheetId="1" r:id="rId1"/>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="157" uniqueCount="138">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="159" uniqueCount="140">
   <si>
     <t>Paramètres globaux — HoloMap</t>
   </si>
@@ -452,6 +452,12 @@
   </si>
   <si>
     <t>12g</t>
+  </si>
+  <si>
+    <t>pont</t>
+  </si>
+  <si>
+    <t>10d</t>
   </si>
 </sst>
 </file>
@@ -604,7 +610,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="47">
+  <borders count="61">
     <border>
       <left/>
       <right/>
@@ -1272,11 +1278,187 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFD0D0D0"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFD0D0D0"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFD0D0D0"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFD0D0D0"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFD0D0D0"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFD0D0D0"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFD0D0D0"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFD0D0D0"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFD0D0D0"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFD0D0D0"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFD0D0D0"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFD0D0D0"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFD0D0D0"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color rgb="FFD0D0D0"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFD0D0D0"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color rgb="FFD0D0D0"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFD0D0D0"/>
+      </left>
+      <right/>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFD0D0D0"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFD0D0D0"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color rgb="FFD0D0D0"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFD0D0D0"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFD0D0D0"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFD0D0D0"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color rgb="FFD0D0D0"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="92">
+  <cellXfs count="107">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -1389,6 +1571,7 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
@@ -1396,7 +1579,21 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="47" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="48" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="49" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="50" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="51" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="52" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="53" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="54" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="55" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="56" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="9" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="57" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="58" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="59" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="60" xfId="0" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -3085,7 +3282,7 @@
       <c r="BH18" s="7"/>
       <c r="BI18" s="7"/>
     </row>
-    <row r="19" spans="1:61" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:61" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A19" s="6">
         <v>18</v>
       </c>
@@ -3111,14 +3308,14 @@
       <c r="U19" s="7"/>
       <c r="V19" s="7"/>
       <c r="W19" s="15"/>
-      <c r="X19" s="7"/>
-      <c r="Y19" s="7"/>
-      <c r="Z19" s="7"/>
-      <c r="AA19" s="7"/>
-      <c r="AB19" s="7"/>
-      <c r="AC19" s="7"/>
-      <c r="AD19" s="7"/>
-      <c r="AE19" s="7"/>
+      <c r="X19" s="14"/>
+      <c r="Y19" s="43"/>
+      <c r="Z19" s="43"/>
+      <c r="AA19" s="43"/>
+      <c r="AB19" s="43"/>
+      <c r="AC19" s="43"/>
+      <c r="AD19" s="43"/>
+      <c r="AE19" s="14"/>
       <c r="AF19" s="7"/>
       <c r="AG19" s="7"/>
       <c r="AH19" s="7"/>
@@ -3176,14 +3373,14 @@
       <c r="U20" s="7"/>
       <c r="V20" s="7"/>
       <c r="W20" s="15"/>
-      <c r="X20" s="7"/>
-      <c r="Y20" s="7"/>
-      <c r="Z20" s="7"/>
-      <c r="AA20" s="7"/>
-      <c r="AB20" s="7"/>
-      <c r="AC20" s="7"/>
-      <c r="AD20" s="7"/>
-      <c r="AE20" s="7"/>
+      <c r="X20" s="66"/>
+      <c r="Y20" s="93"/>
+      <c r="Z20" s="94"/>
+      <c r="AA20" s="94"/>
+      <c r="AB20" s="94"/>
+      <c r="AC20" s="99"/>
+      <c r="AD20" s="104"/>
+      <c r="AE20" s="55"/>
       <c r="AF20" s="7"/>
       <c r="AG20" s="7"/>
       <c r="AH20" s="7"/>
@@ -3241,14 +3438,16 @@
       <c r="U21" s="14"/>
       <c r="V21" s="14"/>
       <c r="W21" s="14"/>
-      <c r="X21" s="14"/>
-      <c r="Y21" s="14"/>
-      <c r="Z21" s="14"/>
-      <c r="AA21" s="14"/>
-      <c r="AB21" s="14"/>
-      <c r="AC21" s="14"/>
-      <c r="AD21" s="14"/>
-      <c r="AE21" s="14"/>
+      <c r="X21" s="66"/>
+      <c r="Y21" s="101"/>
+      <c r="Z21" s="102"/>
+      <c r="AA21" s="102" t="s">
+        <v>139</v>
+      </c>
+      <c r="AB21" s="102"/>
+      <c r="AC21" s="103"/>
+      <c r="AD21" s="105"/>
+      <c r="AE21" s="55"/>
       <c r="AF21" s="7"/>
       <c r="AG21" s="7"/>
       <c r="AH21" s="7"/>
@@ -3300,20 +3499,30 @@
       <c r="O22" s="7"/>
       <c r="P22" s="14"/>
       <c r="Q22" s="14"/>
-      <c r="R22" s="12"/>
-      <c r="S22" s="12"/>
-      <c r="T22" s="12"/>
-      <c r="U22" s="12"/>
-      <c r="V22" s="12"/>
+      <c r="R22" s="12">
+        <v>6</v>
+      </c>
+      <c r="S22" s="12">
+        <v>4</v>
+      </c>
+      <c r="T22" s="12">
+        <v>8</v>
+      </c>
+      <c r="U22" s="12">
+        <v>9</v>
+      </c>
+      <c r="V22" s="12">
+        <v>4</v>
+      </c>
       <c r="W22" s="15"/>
-      <c r="X22" s="14"/>
-      <c r="Y22" s="12"/>
-      <c r="Z22" s="12"/>
-      <c r="AA22" s="12"/>
-      <c r="AB22" s="12"/>
-      <c r="AC22" s="12"/>
-      <c r="AD22" s="14"/>
-      <c r="AE22" s="14"/>
+      <c r="X22" s="66"/>
+      <c r="Y22" s="100"/>
+      <c r="Z22" s="79"/>
+      <c r="AA22" s="79"/>
+      <c r="AB22" s="79"/>
+      <c r="AC22" s="97"/>
+      <c r="AD22" s="105"/>
+      <c r="AE22" s="55"/>
       <c r="AF22" s="7"/>
       <c r="AG22" s="7"/>
       <c r="AH22" s="7"/>
@@ -3345,7 +3554,7 @@
       <c r="BH22" s="7"/>
       <c r="BI22" s="7"/>
     </row>
-    <row r="23" spans="1:61" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:61" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A23" s="6">
         <v>22</v>
       </c>
@@ -3365,20 +3574,30 @@
       <c r="O23" s="14"/>
       <c r="P23" s="14"/>
       <c r="Q23" s="14"/>
-      <c r="R23" s="12"/>
-      <c r="S23" s="12"/>
-      <c r="T23" s="12"/>
-      <c r="U23" s="12"/>
-      <c r="V23" s="12"/>
+      <c r="R23" s="12">
+        <v>6</v>
+      </c>
+      <c r="S23" s="12">
+        <v>7</v>
+      </c>
+      <c r="T23" s="12">
+        <v>8</v>
+      </c>
+      <c r="U23" s="12">
+        <v>9</v>
+      </c>
+      <c r="V23" s="12">
+        <v>5</v>
+      </c>
       <c r="W23" s="15"/>
-      <c r="X23" s="14"/>
-      <c r="Y23" s="12"/>
-      <c r="Z23" s="12"/>
-      <c r="AA23" s="12"/>
-      <c r="AB23" s="12"/>
-      <c r="AC23" s="12"/>
-      <c r="AD23" s="14"/>
-      <c r="AE23" s="14"/>
+      <c r="X23" s="66"/>
+      <c r="Y23" s="95"/>
+      <c r="Z23" s="96"/>
+      <c r="AA23" s="96"/>
+      <c r="AB23" s="96"/>
+      <c r="AC23" s="98"/>
+      <c r="AD23" s="106"/>
+      <c r="AE23" s="55"/>
       <c r="AF23" s="7"/>
       <c r="AG23" s="7"/>
       <c r="AH23" s="7"/>
@@ -3437,11 +3656,11 @@
       <c r="V24" s="14"/>
       <c r="W24" s="43"/>
       <c r="X24" s="43"/>
-      <c r="Y24" s="43"/>
-      <c r="Z24" s="43"/>
-      <c r="AA24" s="14"/>
-      <c r="AB24" s="14"/>
-      <c r="AC24" s="14"/>
+      <c r="Y24" s="92"/>
+      <c r="Z24" s="92"/>
+      <c r="AA24" s="70"/>
+      <c r="AB24" s="70"/>
+      <c r="AC24" s="70"/>
       <c r="AD24" s="14"/>
       <c r="AE24" s="14"/>
       <c r="AF24" s="7"/>
@@ -10042,7 +10261,9 @@
     </row>
     <row r="67" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B67" s="11"/>
-      <c r="C67" s="10"/>
+      <c r="C67" s="10" t="s">
+        <v>138</v>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -10072,7 +10293,7 @@
       <c r="D1" s="84"/>
     </row>
     <row r="3" spans="1:4" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="90" t="s">
+      <c r="A3" s="91" t="s">
         <v>17</v>
       </c>
       <c r="B3" s="84"/>
@@ -10100,7 +10321,7 @@
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A7" s="89" t="s">
+      <c r="A7" s="90" t="s">
         <v>22</v>
       </c>
       <c r="B7" s="84"/>
@@ -10168,7 +10389,7 @@
       </c>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A13" s="91" t="s">
+      <c r="A13" s="88" t="s">
         <v>34</v>
       </c>
       <c r="B13" s="84"/>
@@ -10176,7 +10397,7 @@
       <c r="D13" s="84"/>
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A15" s="89" t="s">
+      <c r="A15" s="90" t="s">
         <v>35</v>
       </c>
       <c r="B15" s="84"/>
@@ -10256,7 +10477,7 @@
       </c>
     </row>
     <row r="22" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A22" s="91" t="s">
+      <c r="A22" s="88" t="s">
         <v>49</v>
       </c>
       <c r="B22" s="84"/>
@@ -10264,14 +10485,14 @@
       <c r="D22" s="84"/>
     </row>
     <row r="26" spans="1:4" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A26" s="88" t="s">
+      <c r="A26" s="89" t="s">
         <v>50</v>
       </c>
       <c r="B26" s="84"/>
       <c r="C26" s="84"/>
       <c r="D26" s="84"/>
     </row>
-    <row r="27" spans="1:4" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:4" ht="31.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A27" s="87" t="s">
         <v>51</v>
       </c>
@@ -10279,7 +10500,7 @@
       <c r="C27" s="84"/>
       <c r="D27" s="84"/>
     </row>
-    <row r="28" spans="1:4" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:4" ht="30.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A28" s="87" t="s">
         <v>52</v>
       </c>
@@ -10287,7 +10508,7 @@
       <c r="C28" s="84"/>
       <c r="D28" s="84"/>
     </row>
-    <row r="29" spans="1:4" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:4" ht="32.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A29" s="87" t="s">
         <v>53</v>
       </c>
@@ -10295,7 +10516,7 @@
       <c r="C29" s="84"/>
       <c r="D29" s="84"/>
     </row>
-    <row r="30" spans="1:4" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:4" ht="34.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A30" s="87" t="s">
         <v>54</v>
       </c>
@@ -10303,7 +10524,7 @@
       <c r="C30" s="84"/>
       <c r="D30" s="84"/>
     </row>
-    <row r="31" spans="1:4" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:4" ht="29.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A31" s="87" t="s">
         <v>55</v>
       </c>
@@ -10311,7 +10532,7 @@
       <c r="C31" s="84"/>
       <c r="D31" s="84"/>
     </row>
-    <row r="32" spans="1:4" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:4" ht="35.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A32" s="87" t="s">
         <v>56</v>
       </c>
@@ -10319,7 +10540,7 @@
       <c r="C32" s="84"/>
       <c r="D32" s="84"/>
     </row>
-    <row r="33" spans="1:4" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:4" ht="30.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A33" s="87" t="s">
         <v>57</v>
       </c>
@@ -10327,7 +10548,7 @@
       <c r="C33" s="84"/>
       <c r="D33" s="84"/>
     </row>
-    <row r="34" spans="1:4" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:4" ht="30.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A34" s="87" t="s">
         <v>58</v>
       </c>
@@ -10335,7 +10556,7 @@
       <c r="C34" s="84"/>
       <c r="D34" s="84"/>
     </row>
-    <row r="35" spans="1:4" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:4" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A35" s="87" t="s">
         <v>59</v>
       </c>
@@ -10350,7 +10571,7 @@
       <c r="D36" s="84"/>
     </row>
     <row r="37" spans="1:4" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A37" s="88" t="s">
+      <c r="A37" s="89" t="s">
         <v>60</v>
       </c>
       <c r="B37" s="84"/>
@@ -10412,14 +10633,14 @@
       <c r="D44" s="84"/>
     </row>
     <row r="45" spans="1:4" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A45" s="88" t="s">
+      <c r="A45" s="89" t="s">
         <v>67</v>
       </c>
       <c r="B45" s="84"/>
       <c r="C45" s="84"/>
       <c r="D45" s="84"/>
     </row>
-    <row r="46" spans="1:4" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:4" ht="37.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A46" s="87" t="s">
         <v>68</v>
       </c>
@@ -10427,7 +10648,7 @@
       <c r="C46" s="84"/>
       <c r="D46" s="84"/>
     </row>
-    <row r="47" spans="1:4" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:4" ht="30.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A47" s="87" t="s">
         <v>69</v>
       </c>
@@ -10435,7 +10656,7 @@
       <c r="C47" s="84"/>
       <c r="D47" s="84"/>
     </row>
-    <row r="48" spans="1:4" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:4" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A48" s="87" t="s">
         <v>70</v>
       </c>
@@ -10443,7 +10664,7 @@
       <c r="C48" s="84"/>
       <c r="D48" s="84"/>
     </row>
-    <row r="49" spans="1:4" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:4" ht="48" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A49" s="87" t="s">
         <v>71</v>
       </c>
@@ -10458,7 +10679,7 @@
       <c r="D50" s="84"/>
     </row>
     <row r="51" spans="1:4" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A51" s="88" t="s">
+      <c r="A51" s="89" t="s">
         <v>72</v>
       </c>
       <c r="B51" s="84"/>
@@ -10481,7 +10702,7 @@
       <c r="C53" s="84"/>
       <c r="D53" s="84"/>
     </row>
-    <row r="54" spans="1:4" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:4" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A54" s="87" t="s">
         <v>75</v>
       </c>
@@ -10528,7 +10749,7 @@
       <c r="D59" s="84"/>
     </row>
     <row r="60" spans="1:4" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A60" s="88" t="s">
+      <c r="A60" s="89" t="s">
         <v>80</v>
       </c>
       <c r="B60" s="84"/>
@@ -10585,21 +10806,22 @@
     </row>
   </sheetData>
   <mergeCells count="47">
-    <mergeCell ref="A62:D62"/>
-    <mergeCell ref="A38:D38"/>
-    <mergeCell ref="A29:D29"/>
-    <mergeCell ref="A52:D52"/>
-    <mergeCell ref="A43:D43"/>
-    <mergeCell ref="A28:D28"/>
-    <mergeCell ref="A13:D13"/>
-    <mergeCell ref="A44:D44"/>
-    <mergeCell ref="A40:D40"/>
-    <mergeCell ref="A31:D31"/>
-    <mergeCell ref="A34:D34"/>
-    <mergeCell ref="A30:D30"/>
-    <mergeCell ref="A39:D39"/>
-    <mergeCell ref="A22:D22"/>
-    <mergeCell ref="A35:D35"/>
+    <mergeCell ref="A65:D65"/>
+    <mergeCell ref="A41:D41"/>
+    <mergeCell ref="A46:D46"/>
+    <mergeCell ref="A66:D66"/>
+    <mergeCell ref="A37:D37"/>
+    <mergeCell ref="A56:D56"/>
+    <mergeCell ref="A50:D50"/>
+    <mergeCell ref="A55:D55"/>
+    <mergeCell ref="A57:D57"/>
+    <mergeCell ref="A47:D47"/>
+    <mergeCell ref="A42:D42"/>
+    <mergeCell ref="A64:D64"/>
+    <mergeCell ref="A63:D63"/>
+    <mergeCell ref="A58:D58"/>
+    <mergeCell ref="A48:D48"/>
+    <mergeCell ref="A53:D53"/>
     <mergeCell ref="A1:D1"/>
     <mergeCell ref="A45:D45"/>
     <mergeCell ref="A61:D61"/>
@@ -10616,22 +10838,21 @@
     <mergeCell ref="A51:D51"/>
     <mergeCell ref="A60:D60"/>
     <mergeCell ref="A36:D36"/>
-    <mergeCell ref="A65:D65"/>
-    <mergeCell ref="A41:D41"/>
-    <mergeCell ref="A46:D46"/>
-    <mergeCell ref="A66:D66"/>
-    <mergeCell ref="A37:D37"/>
-    <mergeCell ref="A56:D56"/>
-    <mergeCell ref="A50:D50"/>
-    <mergeCell ref="A55:D55"/>
-    <mergeCell ref="A57:D57"/>
-    <mergeCell ref="A47:D47"/>
-    <mergeCell ref="A42:D42"/>
-    <mergeCell ref="A64:D64"/>
-    <mergeCell ref="A63:D63"/>
-    <mergeCell ref="A58:D58"/>
-    <mergeCell ref="A48:D48"/>
-    <mergeCell ref="A53:D53"/>
+    <mergeCell ref="A28:D28"/>
+    <mergeCell ref="A13:D13"/>
+    <mergeCell ref="A44:D44"/>
+    <mergeCell ref="A40:D40"/>
+    <mergeCell ref="A31:D31"/>
+    <mergeCell ref="A34:D34"/>
+    <mergeCell ref="A30:D30"/>
+    <mergeCell ref="A39:D39"/>
+    <mergeCell ref="A22:D22"/>
+    <mergeCell ref="A35:D35"/>
+    <mergeCell ref="A62:D62"/>
+    <mergeCell ref="A38:D38"/>
+    <mergeCell ref="A29:D29"/>
+    <mergeCell ref="A52:D52"/>
+    <mergeCell ref="A43:D43"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
feat(holomap3d): feux tricolores + toits/enseignes + brume d'horizon
#1 Feux tricolores (HoloTraffic) : carrefours = composantes connexes de cases
   d'intersection ; un carrefour « controle » (approches sur les 2 axes, >=3
   cotes) alterne vert H / vert V / tout-rouge. Une voiture qui arrive a la ligne
   d'arret n'entre que si son axe est au vert -> elle s'arrete au rouge. Feux
   dessines (barres vert/rouge/ambre) dans l'ImmediateMesh. Test : toujours fluide
   (412 m) et zero croisement.
#3 Toits & enseignes : antennes/citernes sur les batiments-boite, BALISES rouges
   clignotantes au sommet des hautes/grandes tours (alpha pulse), bannieres
   holographiques sur quelques facades.
#6 Brume & horizon : jupe cylindrique a degrade (bleu-cyan -> transparent) +
   nappe de brume au sol + fond bleu nuit -> la ville se decolle du noir.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Carte Holo/carte_holomap.xlsx
+++ b/Carte Holo/carte_holomap.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Projets\IdleEvolution\Carte Holo\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DF2FD20E-2915-4C20-AAE5-6B41F4C86D1A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{86574EEE-621B-4EC8-A5C0-37F04E5E8BC2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -542,7 +542,7 @@
       <name val="Arial"/>
     </font>
   </fonts>
-  <fills count="14">
+  <fills count="15">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -609,8 +609,14 @@
         <fgColor rgb="FF9AA0A6"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFD2B48C"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="61">
+  <borders count="66">
     <border>
       <left/>
       <right/>
@@ -1279,6 +1285,21 @@
       <diagonal/>
     </border>
     <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
       <left style="thin">
         <color rgb="FFD0D0D0"/>
       </left>
@@ -1320,6 +1341,21 @@
       <diagonal/>
     </border>
     <border>
+      <left style="thin">
+        <color rgb="FFD0D0D0"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFD0D0D0"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
       <left style="medium">
         <color indexed="64"/>
       </left>
@@ -1340,6 +1376,21 @@
       </left>
       <right style="thin">
         <color rgb="FFD0D0D0"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFD0D0D0"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFD0D0D0"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
       </right>
       <top style="thin">
         <color rgb="FFD0D0D0"/>
@@ -1454,11 +1505,41 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFD0D0D0"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFD0D0D0"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFD0D0D0"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFD0D0D0"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFD0D0D0"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFD0D0D0"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="107">
+  <cellXfs count="118">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -1579,27 +1660,43 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="47" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="8" borderId="48" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="48" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="8" borderId="49" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="8" borderId="50" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="8" borderId="51" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="8" borderId="52" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="8" borderId="53" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="8" borderId="54" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="8" borderId="55" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="8" borderId="56" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="8" borderId="9" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="8" borderId="57" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="8" borderId="58" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="8" borderId="59" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="9" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="8" borderId="60" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="61" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="62" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="63" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="47" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="14" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="14" borderId="2" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="14" borderId="49" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="14" borderId="50" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="14" borderId="51" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="14" borderId="64" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="14" borderId="65" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="14" borderId="52" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="14" borderId="53" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="14" borderId="54" xfId="0" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
+  <colors>
+    <mruColors>
+      <color rgb="FFD2B48C"/>
+    </mruColors>
+  </colors>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
       <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
@@ -3412,7 +3509,7 @@
       <c r="BH20" s="7"/>
       <c r="BI20" s="7"/>
     </row>
-    <row r="21" spans="1:61" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:61" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A21" s="6">
         <v>20</v>
       </c>
@@ -3432,11 +3529,11 @@
       <c r="O21" s="7"/>
       <c r="P21" s="14"/>
       <c r="Q21" s="14"/>
-      <c r="R21" s="14"/>
-      <c r="S21" s="14"/>
-      <c r="T21" s="14"/>
-      <c r="U21" s="14"/>
-      <c r="V21" s="14"/>
+      <c r="R21" s="43"/>
+      <c r="S21" s="43"/>
+      <c r="T21" s="43"/>
+      <c r="U21" s="43"/>
+      <c r="V21" s="43"/>
       <c r="W21" s="14"/>
       <c r="X21" s="66"/>
       <c r="Y21" s="101"/>
@@ -3479,7 +3576,7 @@
       <c r="BH21" s="7"/>
       <c r="BI21" s="7"/>
     </row>
-    <row r="22" spans="1:61" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:61" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A22" s="6">
         <v>21</v>
       </c>
@@ -3498,23 +3595,23 @@
       <c r="N22" s="7"/>
       <c r="O22" s="7"/>
       <c r="P22" s="14"/>
-      <c r="Q22" s="14"/>
-      <c r="R22" s="12">
+      <c r="Q22" s="66"/>
+      <c r="R22" s="107">
         <v>6</v>
       </c>
-      <c r="S22" s="12">
+      <c r="S22" s="107">
         <v>4</v>
       </c>
-      <c r="T22" s="12">
+      <c r="T22" s="107">
         <v>8</v>
       </c>
-      <c r="U22" s="12">
+      <c r="U22" s="107">
         <v>9</v>
       </c>
-      <c r="V22" s="12">
+      <c r="V22" s="107">
         <v>4</v>
       </c>
-      <c r="W22" s="15"/>
+      <c r="W22" s="108"/>
       <c r="X22" s="66"/>
       <c r="Y22" s="100"/>
       <c r="Z22" s="79"/>
@@ -3573,23 +3670,23 @@
       <c r="N23" s="14"/>
       <c r="O23" s="14"/>
       <c r="P23" s="14"/>
-      <c r="Q23" s="14"/>
-      <c r="R23" s="12">
+      <c r="Q23" s="66"/>
+      <c r="R23" s="107">
         <v>6</v>
       </c>
-      <c r="S23" s="12">
+      <c r="S23" s="107">
         <v>7</v>
       </c>
-      <c r="T23" s="12">
+      <c r="T23" s="107">
         <v>8</v>
       </c>
-      <c r="U23" s="12">
+      <c r="U23" s="107">
         <v>9</v>
       </c>
-      <c r="V23" s="12">
+      <c r="V23" s="107">
         <v>5</v>
       </c>
-      <c r="W23" s="15"/>
+      <c r="W23" s="108"/>
       <c r="X23" s="66"/>
       <c r="Y23" s="95"/>
       <c r="Z23" s="96"/>
@@ -3649,11 +3746,11 @@
       <c r="O24" s="12"/>
       <c r="P24" s="14"/>
       <c r="Q24" s="14"/>
-      <c r="R24" s="14"/>
-      <c r="S24" s="14"/>
-      <c r="T24" s="14"/>
-      <c r="U24" s="14"/>
-      <c r="V24" s="14"/>
+      <c r="R24" s="70"/>
+      <c r="S24" s="70"/>
+      <c r="T24" s="70"/>
+      <c r="U24" s="70"/>
+      <c r="V24" s="70"/>
       <c r="W24" s="43"/>
       <c r="X24" s="43"/>
       <c r="Y24" s="92"/>
@@ -4337,8 +4434,8 @@
       <c r="AY34" s="14"/>
       <c r="AZ34" s="14"/>
       <c r="BA34" s="14"/>
-      <c r="BB34" s="7"/>
-      <c r="BC34" s="7"/>
+      <c r="BB34" s="14"/>
+      <c r="BC34" s="14"/>
       <c r="BD34" s="7"/>
       <c r="BE34" s="7"/>
       <c r="BF34" s="7"/>
@@ -4393,17 +4490,17 @@
       <c r="AP35" s="14"/>
       <c r="AQ35" s="14"/>
       <c r="AR35" s="14"/>
-      <c r="AS35" s="14"/>
-      <c r="AT35" s="14"/>
-      <c r="AU35" s="14"/>
-      <c r="AV35" s="14"/>
-      <c r="AW35" s="14"/>
-      <c r="AX35" s="14"/>
-      <c r="AY35" s="14"/>
-      <c r="AZ35" s="14"/>
-      <c r="BA35" s="14"/>
-      <c r="BB35" s="7"/>
-      <c r="BC35" s="7"/>
+      <c r="AS35" s="43"/>
+      <c r="AT35" s="43"/>
+      <c r="AU35" s="43"/>
+      <c r="AV35" s="43"/>
+      <c r="AW35" s="43"/>
+      <c r="AX35" s="43"/>
+      <c r="AY35" s="43"/>
+      <c r="AZ35" s="43"/>
+      <c r="BA35" s="43"/>
+      <c r="BB35" s="14"/>
+      <c r="BC35" s="14"/>
       <c r="BD35" s="7"/>
       <c r="BE35" s="7"/>
       <c r="BF35" s="7"/>
@@ -4457,18 +4554,18 @@
       <c r="AO36" s="7"/>
       <c r="AP36" s="7"/>
       <c r="AQ36" s="7"/>
-      <c r="AR36" s="14"/>
-      <c r="AS36" s="7"/>
-      <c r="AT36" s="7"/>
-      <c r="AU36" s="7"/>
-      <c r="AV36" s="7"/>
-      <c r="AW36" s="7"/>
-      <c r="AX36" s="7"/>
-      <c r="AY36" s="7"/>
-      <c r="AZ36" s="7"/>
-      <c r="BA36" s="7"/>
-      <c r="BB36" s="7"/>
-      <c r="BC36" s="7"/>
+      <c r="AR36" s="66"/>
+      <c r="AS36" s="110"/>
+      <c r="AT36" s="111"/>
+      <c r="AU36" s="111"/>
+      <c r="AV36" s="111"/>
+      <c r="AW36" s="111"/>
+      <c r="AX36" s="111"/>
+      <c r="AY36" s="111"/>
+      <c r="AZ36" s="111"/>
+      <c r="BA36" s="112"/>
+      <c r="BB36" s="55"/>
+      <c r="BC36" s="14"/>
       <c r="BD36" s="7"/>
       <c r="BE36" s="7"/>
       <c r="BF36" s="7"/>
@@ -4524,18 +4621,18 @@
       <c r="AO37" s="7"/>
       <c r="AP37" s="7"/>
       <c r="AQ37" s="7"/>
-      <c r="AR37" s="14"/>
-      <c r="AS37" s="7"/>
-      <c r="AT37" s="7"/>
-      <c r="AU37" s="7"/>
-      <c r="AV37" s="7"/>
-      <c r="AW37" s="7"/>
-      <c r="AX37" s="7"/>
-      <c r="AY37" s="7"/>
-      <c r="AZ37" s="7"/>
-      <c r="BA37" s="7"/>
-      <c r="BB37" s="7"/>
-      <c r="BC37" s="7"/>
+      <c r="AR37" s="66"/>
+      <c r="AS37" s="113"/>
+      <c r="AT37" s="109"/>
+      <c r="AU37" s="109"/>
+      <c r="AV37" s="109"/>
+      <c r="AW37" s="109"/>
+      <c r="AX37" s="109"/>
+      <c r="AY37" s="109"/>
+      <c r="AZ37" s="109"/>
+      <c r="BA37" s="114"/>
+      <c r="BB37" s="55"/>
+      <c r="BC37" s="14"/>
       <c r="BD37" s="7"/>
       <c r="BE37" s="7"/>
       <c r="BF37" s="7"/>
@@ -4589,18 +4686,18 @@
       <c r="AO38" s="7"/>
       <c r="AP38" s="7"/>
       <c r="AQ38" s="7"/>
-      <c r="AR38" s="14"/>
-      <c r="AS38" s="7"/>
-      <c r="AT38" s="7"/>
-      <c r="AU38" s="7"/>
-      <c r="AV38" s="7"/>
-      <c r="AW38" s="7"/>
-      <c r="AX38" s="7"/>
-      <c r="AY38" s="7"/>
-      <c r="AZ38" s="7"/>
-      <c r="BA38" s="7"/>
-      <c r="BB38" s="7"/>
-      <c r="BC38" s="7"/>
+      <c r="AR38" s="66"/>
+      <c r="AS38" s="113"/>
+      <c r="AT38" s="109"/>
+      <c r="AU38" s="109"/>
+      <c r="AV38" s="109"/>
+      <c r="AW38" s="109"/>
+      <c r="AX38" s="109"/>
+      <c r="AY38" s="109"/>
+      <c r="AZ38" s="109"/>
+      <c r="BA38" s="114"/>
+      <c r="BB38" s="55"/>
+      <c r="BC38" s="14"/>
       <c r="BD38" s="7"/>
       <c r="BE38" s="7"/>
       <c r="BF38" s="7"/>
@@ -4654,18 +4751,18 @@
       <c r="AO39" s="7"/>
       <c r="AP39" s="7"/>
       <c r="AQ39" s="7"/>
-      <c r="AR39" s="14"/>
-      <c r="AS39" s="7"/>
-      <c r="AT39" s="7"/>
-      <c r="AU39" s="7"/>
-      <c r="AV39" s="7"/>
-      <c r="AW39" s="7"/>
-      <c r="AX39" s="7"/>
-      <c r="AY39" s="7"/>
-      <c r="AZ39" s="7"/>
-      <c r="BA39" s="7"/>
-      <c r="BB39" s="7"/>
-      <c r="BC39" s="7"/>
+      <c r="AR39" s="66"/>
+      <c r="AS39" s="113"/>
+      <c r="AT39" s="109"/>
+      <c r="AU39" s="109"/>
+      <c r="AV39" s="109"/>
+      <c r="AW39" s="109"/>
+      <c r="AX39" s="109"/>
+      <c r="AY39" s="109"/>
+      <c r="AZ39" s="109"/>
+      <c r="BA39" s="114"/>
+      <c r="BB39" s="55"/>
+      <c r="BC39" s="14"/>
       <c r="BD39" s="7"/>
       <c r="BE39" s="7"/>
       <c r="BF39" s="7"/>
@@ -4719,18 +4816,18 @@
       <c r="AO40" s="7"/>
       <c r="AP40" s="7"/>
       <c r="AQ40" s="7"/>
-      <c r="AR40" s="14"/>
-      <c r="AS40" s="7"/>
-      <c r="AT40" s="7"/>
-      <c r="AU40" s="7"/>
-      <c r="AV40" s="7"/>
-      <c r="AW40" s="7"/>
-      <c r="AX40" s="7"/>
-      <c r="AY40" s="7"/>
-      <c r="AZ40" s="7"/>
-      <c r="BA40" s="7"/>
-      <c r="BB40" s="7"/>
-      <c r="BC40" s="7"/>
+      <c r="AR40" s="66"/>
+      <c r="AS40" s="113"/>
+      <c r="AT40" s="109"/>
+      <c r="AU40" s="109"/>
+      <c r="AV40" s="109"/>
+      <c r="AW40" s="109"/>
+      <c r="AX40" s="109"/>
+      <c r="AY40" s="109"/>
+      <c r="AZ40" s="109"/>
+      <c r="BA40" s="114"/>
+      <c r="BB40" s="55"/>
+      <c r="BC40" s="14"/>
       <c r="BD40" s="7"/>
       <c r="BE40" s="7"/>
       <c r="BF40" s="7"/>
@@ -4784,18 +4881,18 @@
       <c r="AO41" s="7"/>
       <c r="AP41" s="7"/>
       <c r="AQ41" s="7"/>
-      <c r="AR41" s="14"/>
-      <c r="AS41" s="7"/>
-      <c r="AT41" s="7"/>
-      <c r="AU41" s="7"/>
-      <c r="AV41" s="7"/>
-      <c r="AW41" s="7"/>
-      <c r="AX41" s="7"/>
-      <c r="AY41" s="7"/>
-      <c r="AZ41" s="7"/>
-      <c r="BA41" s="7"/>
-      <c r="BB41" s="7"/>
-      <c r="BC41" s="7"/>
+      <c r="AR41" s="66"/>
+      <c r="AS41" s="113"/>
+      <c r="AT41" s="109"/>
+      <c r="AU41" s="109"/>
+      <c r="AV41" s="109"/>
+      <c r="AW41" s="109"/>
+      <c r="AX41" s="109"/>
+      <c r="AY41" s="109"/>
+      <c r="AZ41" s="109"/>
+      <c r="BA41" s="114"/>
+      <c r="BB41" s="55"/>
+      <c r="BC41" s="14"/>
       <c r="BD41" s="7"/>
       <c r="BE41" s="7"/>
       <c r="BF41" s="7"/>
@@ -4803,7 +4900,7 @@
       <c r="BH41" s="7"/>
       <c r="BI41" s="7"/>
     </row>
-    <row r="42" spans="1:61" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:61" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A42" s="6">
         <v>41</v>
       </c>
@@ -4841,7 +4938,7 @@
       <c r="AG42" s="12"/>
       <c r="AH42" s="12"/>
       <c r="AI42" s="14"/>
-      <c r="AJ42" s="14"/>
+      <c r="AJ42" s="15"/>
       <c r="AK42" s="15"/>
       <c r="AL42" s="14"/>
       <c r="AM42" s="14"/>
@@ -4849,18 +4946,18 @@
       <c r="AO42" s="7"/>
       <c r="AP42" s="7"/>
       <c r="AQ42" s="7"/>
-      <c r="AR42" s="14"/>
-      <c r="AS42" s="7"/>
-      <c r="AT42" s="7"/>
-      <c r="AU42" s="7"/>
-      <c r="AV42" s="7"/>
-      <c r="AW42" s="7"/>
-      <c r="AX42" s="7"/>
-      <c r="AY42" s="7"/>
-      <c r="AZ42" s="7"/>
-      <c r="BA42" s="7"/>
-      <c r="BB42" s="7"/>
-      <c r="BC42" s="7"/>
+      <c r="AR42" s="66"/>
+      <c r="AS42" s="115"/>
+      <c r="AT42" s="116"/>
+      <c r="AU42" s="116"/>
+      <c r="AV42" s="116"/>
+      <c r="AW42" s="116"/>
+      <c r="AX42" s="116"/>
+      <c r="AY42" s="116"/>
+      <c r="AZ42" s="116"/>
+      <c r="BA42" s="117"/>
+      <c r="BB42" s="55"/>
+      <c r="BC42" s="14"/>
       <c r="BD42" s="7"/>
       <c r="BE42" s="7"/>
       <c r="BF42" s="7"/>
@@ -4915,15 +5012,15 @@
       <c r="AP43" s="15"/>
       <c r="AQ43" s="15"/>
       <c r="AR43" s="14"/>
-      <c r="AS43" s="14"/>
-      <c r="AT43" s="14"/>
-      <c r="AU43" s="14"/>
-      <c r="AV43" s="14"/>
-      <c r="AW43" s="14"/>
-      <c r="AX43" s="14"/>
-      <c r="AY43" s="14"/>
-      <c r="AZ43" s="14"/>
-      <c r="BA43" s="14"/>
+      <c r="AS43" s="70"/>
+      <c r="AT43" s="70"/>
+      <c r="AU43" s="70"/>
+      <c r="AV43" s="70"/>
+      <c r="AW43" s="70"/>
+      <c r="AX43" s="70"/>
+      <c r="AY43" s="70"/>
+      <c r="AZ43" s="70"/>
+      <c r="BA43" s="70"/>
       <c r="BB43" s="14"/>
       <c r="BC43" s="14"/>
       <c r="BD43" s="7"/>
@@ -4973,8 +5070,8 @@
       <c r="AI44" s="15"/>
       <c r="AJ44" s="15"/>
       <c r="AK44" s="15"/>
-      <c r="AL44" s="7"/>
-      <c r="AM44" s="7"/>
+      <c r="AL44" s="12"/>
+      <c r="AM44" s="12"/>
       <c r="AN44" s="14"/>
       <c r="AO44" s="15"/>
       <c r="AP44" s="15"/>
@@ -5036,13 +5133,13 @@
       <c r="AG45" s="15"/>
       <c r="AH45" s="15"/>
       <c r="AI45" s="15"/>
-      <c r="AJ45" s="7"/>
-      <c r="AK45" s="7"/>
-      <c r="AL45" s="7"/>
-      <c r="AM45" s="7"/>
+      <c r="AJ45" s="12"/>
+      <c r="AK45" s="12"/>
+      <c r="AL45" s="12"/>
+      <c r="AM45" s="12"/>
       <c r="AN45" s="14"/>
-      <c r="AO45" s="14"/>
-      <c r="AP45" s="14"/>
+      <c r="AO45" s="15"/>
+      <c r="AP45" s="15"/>
       <c r="AQ45" s="15"/>
       <c r="AR45" s="14"/>
       <c r="AS45" s="14"/>
@@ -5101,14 +5198,14 @@
       <c r="AG46" s="14"/>
       <c r="AH46" s="14"/>
       <c r="AI46" s="14"/>
-      <c r="AJ46" s="7"/>
-      <c r="AK46" s="7"/>
-      <c r="AL46" s="7"/>
-      <c r="AM46" s="7"/>
-      <c r="AN46" s="7"/>
-      <c r="AO46" s="7"/>
+      <c r="AJ46" s="14"/>
+      <c r="AK46" s="14"/>
+      <c r="AL46" s="14"/>
+      <c r="AM46" s="14"/>
+      <c r="AN46" s="14"/>
+      <c r="AO46" s="14"/>
       <c r="AP46" s="14"/>
-      <c r="AQ46" s="15"/>
+      <c r="AQ46" s="14"/>
       <c r="AR46" s="14"/>
       <c r="AS46" s="14"/>
       <c r="AT46" s="15"/>
@@ -5157,21 +5254,21 @@
       <c r="X47" s="7"/>
       <c r="Y47" s="7"/>
       <c r="Z47" s="7"/>
-      <c r="AA47" s="7"/>
-      <c r="AB47" s="7"/>
-      <c r="AC47" s="7"/>
+      <c r="AA47" s="14"/>
+      <c r="AB47" s="14"/>
+      <c r="AC47" s="14"/>
       <c r="AD47" s="15"/>
-      <c r="AE47" s="7"/>
-      <c r="AF47" s="7"/>
-      <c r="AG47" s="7"/>
-      <c r="AH47" s="7"/>
-      <c r="AI47" s="7"/>
-      <c r="AJ47" s="7"/>
-      <c r="AK47" s="7"/>
-      <c r="AL47" s="7"/>
-      <c r="AM47" s="7"/>
-      <c r="AN47" s="7"/>
-      <c r="AO47" s="7"/>
+      <c r="AE47" s="14"/>
+      <c r="AF47" s="14"/>
+      <c r="AG47" s="14"/>
+      <c r="AH47" s="14"/>
+      <c r="AI47" s="14"/>
+      <c r="AJ47" s="14"/>
+      <c r="AK47" s="14"/>
+      <c r="AL47" s="14"/>
+      <c r="AM47" s="14"/>
+      <c r="AN47" s="14"/>
+      <c r="AO47" s="14"/>
       <c r="AP47" s="14"/>
       <c r="AQ47" s="14"/>
       <c r="AR47" s="14"/>

</xml_diff>

<commit_message>
feat(holomap3d): vrai STADE de baseball (gradins + projecteurs + tableau)
Remplace le terrain plat par un stade complet, construit sur des ELLIPSES
ajustees a la bbox -> remplit n'importe quel RATIO de bloc (corrige l'impression
de "taille max" liee a l'ancien min(w,h)). Composants :
- terrain : gazon (territoire bon) + closure/warning track + losange + bases +
  monticule, marbre cote +Z, champ ouvert vers -Z ;
- GRADINS en bol : anneaux elliptiques montants (kf -> bord) + coutures radiales ;
- PROJECTEURS : mats au sommet du bol + bancs lumineux (glow) ;
- TABLEAU d'affichage au centre du champ (ecran cyan).

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Carte Holo/carte_holomap.xlsx
+++ b/Carte Holo/carte_holomap.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Projets\IdleEvolution\Carte Holo\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{86574EEE-621B-4EC8-A5C0-37F04E5E8BC2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{20049AA6-2974-49E6-8853-8A1AAABC2769}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -616,7 +616,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="66">
+  <borders count="68">
     <border>
       <left/>
       <right/>
@@ -1248,43 +1248,6 @@
       <diagonal/>
     </border>
     <border>
-      <left/>
-      <right style="thin">
-        <color rgb="FFD0D0D0"/>
-      </right>
-      <top/>
-      <bottom style="thin">
-        <color rgb="FFD0D0D0"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="thin">
-        <color rgb="FFD0D0D0"/>
-      </right>
-      <top style="thin">
-        <color rgb="FFD0D0D0"/>
-      </top>
-      <bottom style="medium">
-        <color theme="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FFD0D0D0"/>
-      </left>
-      <right style="medium">
-        <color theme="1"/>
-      </right>
-      <top/>
-      <bottom style="thin">
-        <color rgb="FFD0D0D0"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
       <left style="medium">
         <color indexed="64"/>
       </left>
@@ -1535,11 +1498,60 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="118">
+  <cellXfs count="119">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -1636,12 +1648,7 @@
     <xf numFmtId="0" fontId="0" fillId="8" borderId="41" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="8" borderId="42" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="8" borderId="43" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="42" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="40" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="8" borderId="44" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="8" borderId="20" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="8" borderId="45" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="46" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="9" borderId="20" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
@@ -1660,32 +1667,38 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="48" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="45" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="46" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="47" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="8" borderId="49" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="8" borderId="50" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="8" borderId="52" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="8" borderId="53" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="54" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="8" borderId="55" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="8" borderId="56" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="9" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="8" borderId="57" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="8" borderId="58" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="8" borderId="59" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="8" borderId="9" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="8" borderId="60" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="8" borderId="61" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="8" borderId="62" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="8" borderId="63" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="8" borderId="47" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="44" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="9" borderId="14" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="14" borderId="2" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="14" borderId="46" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="14" borderId="47" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="14" borderId="48" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="14" borderId="61" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="14" borderId="62" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="14" borderId="49" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="14" borderId="50" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="14" borderId="51" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="14" borderId="64" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="14" borderId="65" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="14" borderId="52" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="14" borderId="53" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="14" borderId="54" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="0" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="63" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="64" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="65" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="66" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="67" xfId="0" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -2002,11 +2015,11 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="A1" s="85" t="s">
+      <c r="A1" s="80" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="84"/>
-      <c r="C1" s="84"/>
+      <c r="B1" s="79"/>
+      <c r="C1" s="79"/>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
@@ -2064,11 +2077,11 @@
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A9" s="86" t="s">
+      <c r="A9" s="81" t="s">
         <v>13</v>
       </c>
-      <c r="B9" s="84"/>
-      <c r="C9" s="84"/>
+      <c r="B9" s="79"/>
+      <c r="C9" s="79"/>
     </row>
   </sheetData>
   <mergeCells count="2">
@@ -3471,12 +3484,12 @@
       <c r="V20" s="7"/>
       <c r="W20" s="15"/>
       <c r="X20" s="66"/>
-      <c r="Y20" s="93"/>
-      <c r="Z20" s="94"/>
-      <c r="AA20" s="94"/>
-      <c r="AB20" s="94"/>
-      <c r="AC20" s="99"/>
-      <c r="AD20" s="104"/>
+      <c r="Y20" s="88"/>
+      <c r="Z20" s="89"/>
+      <c r="AA20" s="89"/>
+      <c r="AB20" s="89"/>
+      <c r="AC20" s="94"/>
+      <c r="AD20" s="99"/>
       <c r="AE20" s="55"/>
       <c r="AF20" s="7"/>
       <c r="AG20" s="7"/>
@@ -3536,14 +3549,14 @@
       <c r="V21" s="43"/>
       <c r="W21" s="14"/>
       <c r="X21" s="66"/>
-      <c r="Y21" s="101"/>
-      <c r="Z21" s="102"/>
-      <c r="AA21" s="102" t="s">
+      <c r="Y21" s="96"/>
+      <c r="Z21" s="97"/>
+      <c r="AA21" s="97" t="s">
         <v>139</v>
       </c>
-      <c r="AB21" s="102"/>
-      <c r="AC21" s="103"/>
-      <c r="AD21" s="105"/>
+      <c r="AB21" s="97"/>
+      <c r="AC21" s="98"/>
+      <c r="AD21" s="100"/>
       <c r="AE21" s="55"/>
       <c r="AF21" s="7"/>
       <c r="AG21" s="7"/>
@@ -3596,29 +3609,29 @@
       <c r="O22" s="7"/>
       <c r="P22" s="14"/>
       <c r="Q22" s="66"/>
-      <c r="R22" s="107">
+      <c r="R22" s="102">
         <v>6</v>
       </c>
-      <c r="S22" s="107">
+      <c r="S22" s="102">
         <v>4</v>
       </c>
-      <c r="T22" s="107">
+      <c r="T22" s="102">
         <v>8</v>
       </c>
-      <c r="U22" s="107">
+      <c r="U22" s="102">
         <v>9</v>
       </c>
-      <c r="V22" s="107">
+      <c r="V22" s="102">
         <v>4</v>
       </c>
-      <c r="W22" s="108"/>
+      <c r="W22" s="103"/>
       <c r="X22" s="66"/>
-      <c r="Y22" s="100"/>
-      <c r="Z22" s="79"/>
-      <c r="AA22" s="79"/>
-      <c r="AB22" s="79"/>
-      <c r="AC22" s="97"/>
-      <c r="AD22" s="105"/>
+      <c r="Y22" s="95"/>
+      <c r="Z22" s="76"/>
+      <c r="AA22" s="76"/>
+      <c r="AB22" s="76"/>
+      <c r="AC22" s="92"/>
+      <c r="AD22" s="100"/>
       <c r="AE22" s="55"/>
       <c r="AF22" s="7"/>
       <c r="AG22" s="7"/>
@@ -3671,29 +3684,29 @@
       <c r="O23" s="14"/>
       <c r="P23" s="14"/>
       <c r="Q23" s="66"/>
-      <c r="R23" s="107">
+      <c r="R23" s="102">
         <v>6</v>
       </c>
-      <c r="S23" s="107">
+      <c r="S23" s="102">
         <v>7</v>
       </c>
-      <c r="T23" s="107">
+      <c r="T23" s="102">
         <v>8</v>
       </c>
-      <c r="U23" s="107">
+      <c r="U23" s="102">
         <v>9</v>
       </c>
-      <c r="V23" s="107">
+      <c r="V23" s="102">
         <v>5</v>
       </c>
-      <c r="W23" s="108"/>
+      <c r="W23" s="103"/>
       <c r="X23" s="66"/>
-      <c r="Y23" s="95"/>
-      <c r="Z23" s="96"/>
-      <c r="AA23" s="96"/>
-      <c r="AB23" s="96"/>
-      <c r="AC23" s="98"/>
-      <c r="AD23" s="106"/>
+      <c r="Y23" s="90"/>
+      <c r="Z23" s="91"/>
+      <c r="AA23" s="91"/>
+      <c r="AB23" s="91"/>
+      <c r="AC23" s="93"/>
+      <c r="AD23" s="101"/>
       <c r="AE23" s="55"/>
       <c r="AF23" s="7"/>
       <c r="AG23" s="7"/>
@@ -3753,8 +3766,8 @@
       <c r="V24" s="70"/>
       <c r="W24" s="43"/>
       <c r="X24" s="43"/>
-      <c r="Y24" s="92"/>
-      <c r="Z24" s="92"/>
+      <c r="Y24" s="87"/>
+      <c r="Z24" s="87"/>
       <c r="AA24" s="70"/>
       <c r="AB24" s="70"/>
       <c r="AC24" s="70"/>
@@ -4474,12 +4487,12 @@
       <c r="Z35" s="14"/>
       <c r="AA35" s="14"/>
       <c r="AB35" s="14"/>
-      <c r="AC35" s="76"/>
-      <c r="AD35" s="76"/>
-      <c r="AE35" s="76"/>
-      <c r="AF35" s="76"/>
-      <c r="AG35" s="76"/>
-      <c r="AH35" s="76"/>
+      <c r="AC35" s="43"/>
+      <c r="AD35" s="43"/>
+      <c r="AE35" s="43"/>
+      <c r="AF35" s="43"/>
+      <c r="AG35" s="43"/>
+      <c r="AH35" s="43"/>
       <c r="AI35" s="14"/>
       <c r="AJ35" s="14"/>
       <c r="AK35" s="14"/>
@@ -4538,13 +4551,13 @@
       <c r="Y36" s="16"/>
       <c r="Z36" s="16"/>
       <c r="AA36" s="14"/>
-      <c r="AB36" s="77"/>
-      <c r="AC36" s="78"/>
-      <c r="AD36" s="79"/>
-      <c r="AE36" s="79"/>
-      <c r="AF36" s="79"/>
-      <c r="AG36" s="79"/>
-      <c r="AH36" s="69"/>
+      <c r="AB36" s="66"/>
+      <c r="AC36" s="114"/>
+      <c r="AD36" s="115"/>
+      <c r="AE36" s="115"/>
+      <c r="AF36" s="115"/>
+      <c r="AG36" s="115"/>
+      <c r="AH36" s="99"/>
       <c r="AI36" s="55"/>
       <c r="AJ36" s="16"/>
       <c r="AK36" s="16"/>
@@ -4555,15 +4568,15 @@
       <c r="AP36" s="7"/>
       <c r="AQ36" s="7"/>
       <c r="AR36" s="66"/>
-      <c r="AS36" s="110"/>
-      <c r="AT36" s="111"/>
-      <c r="AU36" s="111"/>
-      <c r="AV36" s="111"/>
-      <c r="AW36" s="111"/>
-      <c r="AX36" s="111"/>
-      <c r="AY36" s="111"/>
-      <c r="AZ36" s="111"/>
-      <c r="BA36" s="112"/>
+      <c r="AS36" s="105"/>
+      <c r="AT36" s="106"/>
+      <c r="AU36" s="106"/>
+      <c r="AV36" s="106"/>
+      <c r="AW36" s="106"/>
+      <c r="AX36" s="106"/>
+      <c r="AY36" s="106"/>
+      <c r="AZ36" s="106"/>
+      <c r="BA36" s="107"/>
       <c r="BB36" s="55"/>
       <c r="BC36" s="14"/>
       <c r="BD36" s="7"/>
@@ -4573,7 +4586,7 @@
       <c r="BH36" s="7"/>
       <c r="BI36" s="7"/>
     </row>
-    <row r="37" spans="1:61" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:61" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A37" s="6">
         <v>36</v>
       </c>
@@ -4603,15 +4616,15 @@
       <c r="Y37" s="16"/>
       <c r="Z37" s="16"/>
       <c r="AA37" s="14"/>
-      <c r="AB37" s="77"/>
-      <c r="AC37" s="80"/>
-      <c r="AD37" s="12"/>
-      <c r="AE37" s="12"/>
-      <c r="AF37" s="12" t="s">
+      <c r="AB37" s="66"/>
+      <c r="AC37" s="116"/>
+      <c r="AD37" s="113"/>
+      <c r="AE37" s="113"/>
+      <c r="AF37" s="113" t="s">
         <v>137</v>
       </c>
-      <c r="AG37" s="12"/>
-      <c r="AH37" s="72"/>
+      <c r="AG37" s="113"/>
+      <c r="AH37" s="100"/>
       <c r="AI37" s="55"/>
       <c r="AJ37" s="16"/>
       <c r="AK37" s="16"/>
@@ -4622,15 +4635,15 @@
       <c r="AP37" s="7"/>
       <c r="AQ37" s="7"/>
       <c r="AR37" s="66"/>
-      <c r="AS37" s="113"/>
-      <c r="AT37" s="109"/>
-      <c r="AU37" s="109"/>
-      <c r="AV37" s="109"/>
-      <c r="AW37" s="109"/>
-      <c r="AX37" s="109"/>
-      <c r="AY37" s="109"/>
-      <c r="AZ37" s="109"/>
-      <c r="BA37" s="114"/>
+      <c r="AS37" s="108"/>
+      <c r="AT37" s="104"/>
+      <c r="AU37" s="104"/>
+      <c r="AV37" s="104"/>
+      <c r="AW37" s="104"/>
+      <c r="AX37" s="104"/>
+      <c r="AY37" s="104"/>
+      <c r="AZ37" s="104"/>
+      <c r="BA37" s="109"/>
       <c r="BB37" s="55"/>
       <c r="BC37" s="14"/>
       <c r="BD37" s="7"/>
@@ -4640,7 +4653,7 @@
       <c r="BH37" s="7"/>
       <c r="BI37" s="7"/>
     </row>
-    <row r="38" spans="1:61" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:61" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A38" s="6">
         <v>37</v>
       </c>
@@ -4670,13 +4683,13 @@
       <c r="Y38" s="16"/>
       <c r="Z38" s="16"/>
       <c r="AA38" s="14"/>
-      <c r="AB38" s="14"/>
-      <c r="AC38" s="81"/>
-      <c r="AD38" s="80"/>
-      <c r="AE38" s="12"/>
-      <c r="AF38" s="12"/>
-      <c r="AG38" s="12"/>
-      <c r="AH38" s="72"/>
+      <c r="AB38" s="66"/>
+      <c r="AC38" s="116"/>
+      <c r="AD38" s="113"/>
+      <c r="AE38" s="113"/>
+      <c r="AF38" s="113"/>
+      <c r="AG38" s="113"/>
+      <c r="AH38" s="100"/>
       <c r="AI38" s="55"/>
       <c r="AJ38" s="16"/>
       <c r="AK38" s="16"/>
@@ -4687,15 +4700,15 @@
       <c r="AP38" s="7"/>
       <c r="AQ38" s="7"/>
       <c r="AR38" s="66"/>
-      <c r="AS38" s="113"/>
-      <c r="AT38" s="109"/>
-      <c r="AU38" s="109"/>
-      <c r="AV38" s="109"/>
-      <c r="AW38" s="109"/>
-      <c r="AX38" s="109"/>
-      <c r="AY38" s="109"/>
-      <c r="AZ38" s="109"/>
-      <c r="BA38" s="114"/>
+      <c r="AS38" s="108"/>
+      <c r="AT38" s="104"/>
+      <c r="AU38" s="104"/>
+      <c r="AV38" s="104"/>
+      <c r="AW38" s="104"/>
+      <c r="AX38" s="104"/>
+      <c r="AY38" s="104"/>
+      <c r="AZ38" s="104"/>
+      <c r="BA38" s="109"/>
       <c r="BB38" s="55"/>
       <c r="BC38" s="14"/>
       <c r="BD38" s="7"/>
@@ -4705,7 +4718,7 @@
       <c r="BH38" s="7"/>
       <c r="BI38" s="7"/>
     </row>
-    <row r="39" spans="1:61" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:61" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A39" s="6">
         <v>38</v>
       </c>
@@ -4735,13 +4748,13 @@
       <c r="Y39" s="14"/>
       <c r="Z39" s="14"/>
       <c r="AA39" s="14"/>
-      <c r="AB39" s="14"/>
-      <c r="AC39" s="15"/>
-      <c r="AD39" s="81"/>
-      <c r="AE39" s="80"/>
-      <c r="AF39" s="12"/>
-      <c r="AG39" s="12"/>
-      <c r="AH39" s="72"/>
+      <c r="AB39" s="66"/>
+      <c r="AC39" s="116"/>
+      <c r="AD39" s="113"/>
+      <c r="AE39" s="113"/>
+      <c r="AF39" s="113"/>
+      <c r="AG39" s="113"/>
+      <c r="AH39" s="100"/>
       <c r="AI39" s="55"/>
       <c r="AJ39" s="7"/>
       <c r="AK39" s="7"/>
@@ -4752,15 +4765,15 @@
       <c r="AP39" s="7"/>
       <c r="AQ39" s="7"/>
       <c r="AR39" s="66"/>
-      <c r="AS39" s="113"/>
-      <c r="AT39" s="109"/>
-      <c r="AU39" s="109"/>
-      <c r="AV39" s="109"/>
-      <c r="AW39" s="109"/>
-      <c r="AX39" s="109"/>
-      <c r="AY39" s="109"/>
-      <c r="AZ39" s="109"/>
-      <c r="BA39" s="114"/>
+      <c r="AS39" s="108"/>
+      <c r="AT39" s="104"/>
+      <c r="AU39" s="104"/>
+      <c r="AV39" s="104"/>
+      <c r="AW39" s="104"/>
+      <c r="AX39" s="104"/>
+      <c r="AY39" s="104"/>
+      <c r="AZ39" s="104"/>
+      <c r="BA39" s="109"/>
       <c r="BB39" s="55"/>
       <c r="BC39" s="14"/>
       <c r="BD39" s="7"/>
@@ -4800,13 +4813,13 @@
       <c r="Y40" s="7"/>
       <c r="Z40" s="7"/>
       <c r="AA40" s="14"/>
-      <c r="AB40" s="14"/>
-      <c r="AC40" s="12"/>
-      <c r="AD40" s="15"/>
-      <c r="AE40" s="81"/>
-      <c r="AF40" s="80"/>
-      <c r="AG40" s="74"/>
-      <c r="AH40" s="75"/>
+      <c r="AB40" s="66"/>
+      <c r="AC40" s="117"/>
+      <c r="AD40" s="118"/>
+      <c r="AE40" s="118"/>
+      <c r="AF40" s="118"/>
+      <c r="AG40" s="118"/>
+      <c r="AH40" s="101"/>
       <c r="AI40" s="55"/>
       <c r="AJ40" s="7"/>
       <c r="AK40" s="7"/>
@@ -4817,15 +4830,15 @@
       <c r="AP40" s="7"/>
       <c r="AQ40" s="7"/>
       <c r="AR40" s="66"/>
-      <c r="AS40" s="113"/>
-      <c r="AT40" s="109"/>
-      <c r="AU40" s="109"/>
-      <c r="AV40" s="109"/>
-      <c r="AW40" s="109"/>
-      <c r="AX40" s="109"/>
-      <c r="AY40" s="109"/>
-      <c r="AZ40" s="109"/>
-      <c r="BA40" s="114"/>
+      <c r="AS40" s="108"/>
+      <c r="AT40" s="104"/>
+      <c r="AU40" s="104"/>
+      <c r="AV40" s="104"/>
+      <c r="AW40" s="104"/>
+      <c r="AX40" s="104"/>
+      <c r="AY40" s="104"/>
+      <c r="AZ40" s="104"/>
+      <c r="BA40" s="109"/>
       <c r="BB40" s="55"/>
       <c r="BC40" s="14"/>
       <c r="BD40" s="7"/>
@@ -4866,12 +4879,12 @@
       <c r="Z41" s="7"/>
       <c r="AA41" s="14"/>
       <c r="AB41" s="14"/>
-      <c r="AC41" s="12"/>
-      <c r="AD41" s="15"/>
-      <c r="AE41" s="15"/>
-      <c r="AF41" s="15"/>
-      <c r="AG41" s="82"/>
-      <c r="AH41" s="82"/>
+      <c r="AC41" s="77"/>
+      <c r="AD41" s="77"/>
+      <c r="AE41" s="77"/>
+      <c r="AF41" s="77"/>
+      <c r="AG41" s="77"/>
+      <c r="AH41" s="77"/>
       <c r="AI41" s="14"/>
       <c r="AJ41" s="14"/>
       <c r="AK41" s="14"/>
@@ -4882,15 +4895,15 @@
       <c r="AP41" s="7"/>
       <c r="AQ41" s="7"/>
       <c r="AR41" s="66"/>
-      <c r="AS41" s="113"/>
-      <c r="AT41" s="109"/>
-      <c r="AU41" s="109"/>
-      <c r="AV41" s="109"/>
-      <c r="AW41" s="109"/>
-      <c r="AX41" s="109"/>
-      <c r="AY41" s="109"/>
-      <c r="AZ41" s="109"/>
-      <c r="BA41" s="114"/>
+      <c r="AS41" s="108"/>
+      <c r="AT41" s="104"/>
+      <c r="AU41" s="104"/>
+      <c r="AV41" s="104"/>
+      <c r="AW41" s="104"/>
+      <c r="AX41" s="104"/>
+      <c r="AY41" s="104"/>
+      <c r="AZ41" s="104"/>
+      <c r="BA41" s="109"/>
       <c r="BB41" s="55"/>
       <c r="BC41" s="14"/>
       <c r="BD41" s="7"/>
@@ -4947,15 +4960,15 @@
       <c r="AP42" s="7"/>
       <c r="AQ42" s="7"/>
       <c r="AR42" s="66"/>
-      <c r="AS42" s="115"/>
-      <c r="AT42" s="116"/>
-      <c r="AU42" s="116"/>
-      <c r="AV42" s="116"/>
-      <c r="AW42" s="116"/>
-      <c r="AX42" s="116"/>
-      <c r="AY42" s="116"/>
-      <c r="AZ42" s="116"/>
-      <c r="BA42" s="117"/>
+      <c r="AS42" s="110"/>
+      <c r="AT42" s="111"/>
+      <c r="AU42" s="111"/>
+      <c r="AV42" s="111"/>
+      <c r="AW42" s="111"/>
+      <c r="AX42" s="111"/>
+      <c r="AY42" s="111"/>
+      <c r="AZ42" s="111"/>
+      <c r="BA42" s="112"/>
       <c r="BB42" s="55"/>
       <c r="BC42" s="14"/>
       <c r="BD42" s="7"/>
@@ -5063,10 +5076,10 @@
       <c r="AB44" s="14"/>
       <c r="AC44" s="12"/>
       <c r="AD44" s="12"/>
-      <c r="AE44" s="12"/>
+      <c r="AE44" s="15"/>
       <c r="AF44" s="15"/>
       <c r="AG44" s="15"/>
-      <c r="AH44" s="12"/>
+      <c r="AH44" s="15"/>
       <c r="AI44" s="15"/>
       <c r="AJ44" s="15"/>
       <c r="AK44" s="15"/>
@@ -5192,9 +5205,9 @@
       <c r="AA46" s="14"/>
       <c r="AB46" s="14"/>
       <c r="AC46" s="14"/>
-      <c r="AD46" s="15"/>
+      <c r="AD46" s="14"/>
       <c r="AE46" s="14"/>
-      <c r="AF46" s="14"/>
+      <c r="AF46" s="15"/>
       <c r="AG46" s="14"/>
       <c r="AH46" s="14"/>
       <c r="AI46" s="14"/>
@@ -5257,9 +5270,9 @@
       <c r="AA47" s="14"/>
       <c r="AB47" s="14"/>
       <c r="AC47" s="14"/>
-      <c r="AD47" s="15"/>
+      <c r="AD47" s="14"/>
       <c r="AE47" s="14"/>
-      <c r="AF47" s="14"/>
+      <c r="AF47" s="15"/>
       <c r="AG47" s="14"/>
       <c r="AH47" s="14"/>
       <c r="AI47" s="14"/>
@@ -5322,9 +5335,9 @@
       <c r="AA48" s="7"/>
       <c r="AB48" s="7"/>
       <c r="AC48" s="7"/>
-      <c r="AD48" s="15"/>
+      <c r="AD48" s="7"/>
       <c r="AE48" s="7"/>
-      <c r="AF48" s="7"/>
+      <c r="AF48" s="15"/>
       <c r="AG48" s="7"/>
       <c r="AH48" s="7"/>
       <c r="AI48" s="7"/>
@@ -5387,8 +5400,8 @@
       <c r="AA49" s="7"/>
       <c r="AB49" s="7"/>
       <c r="AC49" s="7"/>
-      <c r="AD49" s="15"/>
-      <c r="AE49" s="15"/>
+      <c r="AD49" s="7"/>
+      <c r="AE49" s="7"/>
       <c r="AF49" s="15"/>
       <c r="AG49" s="15"/>
       <c r="AH49" s="15"/>
@@ -9160,8 +9173,8 @@
       <c r="X44" s="8"/>
       <c r="Y44" s="8"/>
       <c r="Z44" s="8"/>
-      <c r="AA44" s="8"/>
-      <c r="AB44" s="8"/>
+      <c r="AA44" s="11"/>
+      <c r="AB44" s="11"/>
       <c r="AC44" s="8"/>
       <c r="AD44" s="8"/>
       <c r="AE44" s="8"/>
@@ -9225,8 +9238,10 @@
       <c r="X45" s="8"/>
       <c r="Y45" s="8"/>
       <c r="Z45" s="8"/>
-      <c r="AA45" s="8"/>
-      <c r="AB45" s="8"/>
+      <c r="AA45" s="11"/>
+      <c r="AB45" s="11">
+        <v>1</v>
+      </c>
       <c r="AC45" s="8"/>
       <c r="AD45" s="8"/>
       <c r="AE45" s="8"/>
@@ -9290,15 +9305,15 @@
       <c r="X46" s="8"/>
       <c r="Y46" s="8"/>
       <c r="Z46" s="8"/>
-      <c r="AA46" s="8"/>
-      <c r="AB46" s="8"/>
-      <c r="AC46" s="11"/>
-      <c r="AD46" s="11">
+      <c r="AA46" s="11"/>
+      <c r="AB46" s="11"/>
+      <c r="AC46" s="8"/>
+      <c r="AD46" s="8"/>
+      <c r="AE46" s="11"/>
+      <c r="AF46" s="11">
         <v>1</v>
       </c>
-      <c r="AE46" s="11"/>
-      <c r="AF46" s="8"/>
-      <c r="AG46" s="8"/>
+      <c r="AG46" s="11"/>
       <c r="AH46" s="8"/>
       <c r="AI46" s="8"/>
       <c r="AJ46" s="8"/>
@@ -9361,9 +9376,9 @@
       <c r="AB47" s="8"/>
       <c r="AC47" s="8"/>
       <c r="AD47" s="8"/>
-      <c r="AE47" s="8"/>
-      <c r="AF47" s="8"/>
-      <c r="AG47" s="8"/>
+      <c r="AE47" s="11"/>
+      <c r="AF47" s="11"/>
+      <c r="AG47" s="11"/>
       <c r="AH47" s="8"/>
       <c r="AI47" s="8"/>
       <c r="AJ47" s="8"/>
@@ -10304,50 +10319,50 @@
       <c r="BI61" s="8"/>
     </row>
     <row r="63" spans="1:61" x14ac:dyDescent="0.25">
-      <c r="A63" s="83" t="s">
+      <c r="A63" s="78" t="s">
         <v>15</v>
       </c>
-      <c r="B63" s="84"/>
-      <c r="C63" s="84"/>
-      <c r="D63" s="84"/>
-      <c r="E63" s="84"/>
-      <c r="F63" s="84"/>
-      <c r="G63" s="84"/>
-      <c r="H63" s="84"/>
-      <c r="I63" s="84"/>
-      <c r="J63" s="84"/>
-      <c r="K63" s="84"/>
-      <c r="L63" s="84"/>
-      <c r="M63" s="84"/>
-      <c r="N63" s="84"/>
-      <c r="O63" s="84"/>
-      <c r="P63" s="84"/>
-      <c r="Q63" s="84"/>
-      <c r="R63" s="84"/>
-      <c r="S63" s="84"/>
-      <c r="T63" s="84"/>
+      <c r="B63" s="79"/>
+      <c r="C63" s="79"/>
+      <c r="D63" s="79"/>
+      <c r="E63" s="79"/>
+      <c r="F63" s="79"/>
+      <c r="G63" s="79"/>
+      <c r="H63" s="79"/>
+      <c r="I63" s="79"/>
+      <c r="J63" s="79"/>
+      <c r="K63" s="79"/>
+      <c r="L63" s="79"/>
+      <c r="M63" s="79"/>
+      <c r="N63" s="79"/>
+      <c r="O63" s="79"/>
+      <c r="P63" s="79"/>
+      <c r="Q63" s="79"/>
+      <c r="R63" s="79"/>
+      <c r="S63" s="79"/>
+      <c r="T63" s="79"/>
     </row>
     <row r="64" spans="1:61" ht="81.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A64" s="84"/>
-      <c r="B64" s="84"/>
-      <c r="C64" s="84"/>
-      <c r="D64" s="84"/>
-      <c r="E64" s="84"/>
-      <c r="F64" s="84"/>
-      <c r="G64" s="84"/>
-      <c r="H64" s="84"/>
-      <c r="I64" s="84"/>
-      <c r="J64" s="84"/>
-      <c r="K64" s="84"/>
-      <c r="L64" s="84"/>
-      <c r="M64" s="84"/>
-      <c r="N64" s="84"/>
-      <c r="O64" s="84"/>
-      <c r="P64" s="84"/>
-      <c r="Q64" s="84"/>
-      <c r="R64" s="84"/>
-      <c r="S64" s="84"/>
-      <c r="T64" s="84"/>
+      <c r="A64" s="79"/>
+      <c r="B64" s="79"/>
+      <c r="C64" s="79"/>
+      <c r="D64" s="79"/>
+      <c r="E64" s="79"/>
+      <c r="F64" s="79"/>
+      <c r="G64" s="79"/>
+      <c r="H64" s="79"/>
+      <c r="I64" s="79"/>
+      <c r="J64" s="79"/>
+      <c r="K64" s="79"/>
+      <c r="L64" s="79"/>
+      <c r="M64" s="79"/>
+      <c r="N64" s="79"/>
+      <c r="O64" s="79"/>
+      <c r="P64" s="79"/>
+      <c r="Q64" s="79"/>
+      <c r="R64" s="79"/>
+      <c r="S64" s="79"/>
+      <c r="T64" s="79"/>
     </row>
     <row r="66" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B66" s="9"/>
@@ -10382,26 +10397,26 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:4" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="A1" s="85" t="s">
+      <c r="A1" s="80" t="s">
         <v>16</v>
       </c>
-      <c r="B1" s="84"/>
-      <c r="C1" s="84"/>
-      <c r="D1" s="84"/>
+      <c r="B1" s="79"/>
+      <c r="C1" s="79"/>
+      <c r="D1" s="79"/>
     </row>
     <row r="3" spans="1:4" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="91" t="s">
+      <c r="A3" s="86" t="s">
         <v>17</v>
       </c>
-      <c r="B3" s="84"/>
-      <c r="C3" s="84"/>
-      <c r="D3" s="84"/>
+      <c r="B3" s="79"/>
+      <c r="C3" s="79"/>
+      <c r="D3" s="79"/>
     </row>
     <row r="4" spans="1:4" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="84"/>
-      <c r="B4" s="84"/>
-      <c r="C4" s="84"/>
-      <c r="D4" s="84"/>
+      <c r="A4" s="79"/>
+      <c r="B4" s="79"/>
+      <c r="C4" s="79"/>
+      <c r="D4" s="79"/>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A6" s="1" t="s">
@@ -10418,12 +10433,12 @@
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A7" s="90" t="s">
+      <c r="A7" s="85" t="s">
         <v>22</v>
       </c>
-      <c r="B7" s="84"/>
-      <c r="C7" s="84"/>
-      <c r="D7" s="84"/>
+      <c r="B7" s="79"/>
+      <c r="C7" s="79"/>
+      <c r="D7" s="79"/>
     </row>
     <row r="8" spans="1:4" ht="24" x14ac:dyDescent="0.25">
       <c r="A8" s="12"/>
@@ -10486,20 +10501,20 @@
       </c>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A13" s="88" t="s">
+      <c r="A13" s="83" t="s">
         <v>34</v>
       </c>
-      <c r="B13" s="84"/>
-      <c r="C13" s="84"/>
-      <c r="D13" s="84"/>
+      <c r="B13" s="79"/>
+      <c r="C13" s="79"/>
+      <c r="D13" s="79"/>
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A15" s="90" t="s">
+      <c r="A15" s="85" t="s">
         <v>35</v>
       </c>
-      <c r="B15" s="84"/>
-      <c r="C15" s="84"/>
-      <c r="D15" s="84"/>
+      <c r="B15" s="79"/>
+      <c r="C15" s="79"/>
+      <c r="D15" s="79"/>
     </row>
     <row r="16" spans="1:4" ht="24" x14ac:dyDescent="0.25">
       <c r="A16" s="17"/>
@@ -10574,332 +10589,332 @@
       </c>
     </row>
     <row r="22" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A22" s="88" t="s">
+      <c r="A22" s="83" t="s">
         <v>49</v>
       </c>
-      <c r="B22" s="84"/>
-      <c r="C22" s="84"/>
-      <c r="D22" s="84"/>
+      <c r="B22" s="79"/>
+      <c r="C22" s="79"/>
+      <c r="D22" s="79"/>
     </row>
     <row r="26" spans="1:4" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A26" s="89" t="s">
+      <c r="A26" s="84" t="s">
         <v>50</v>
       </c>
-      <c r="B26" s="84"/>
-      <c r="C26" s="84"/>
-      <c r="D26" s="84"/>
+      <c r="B26" s="79"/>
+      <c r="C26" s="79"/>
+      <c r="D26" s="79"/>
     </row>
     <row r="27" spans="1:4" ht="31.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A27" s="87" t="s">
+      <c r="A27" s="82" t="s">
         <v>51</v>
       </c>
-      <c r="B27" s="84"/>
-      <c r="C27" s="84"/>
-      <c r="D27" s="84"/>
+      <c r="B27" s="79"/>
+      <c r="C27" s="79"/>
+      <c r="D27" s="79"/>
     </row>
     <row r="28" spans="1:4" ht="30.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A28" s="87" t="s">
+      <c r="A28" s="82" t="s">
         <v>52</v>
       </c>
-      <c r="B28" s="84"/>
-      <c r="C28" s="84"/>
-      <c r="D28" s="84"/>
+      <c r="B28" s="79"/>
+      <c r="C28" s="79"/>
+      <c r="D28" s="79"/>
     </row>
     <row r="29" spans="1:4" ht="32.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A29" s="87" t="s">
+      <c r="A29" s="82" t="s">
         <v>53</v>
       </c>
-      <c r="B29" s="84"/>
-      <c r="C29" s="84"/>
-      <c r="D29" s="84"/>
+      <c r="B29" s="79"/>
+      <c r="C29" s="79"/>
+      <c r="D29" s="79"/>
     </row>
     <row r="30" spans="1:4" ht="34.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A30" s="87" t="s">
+      <c r="A30" s="82" t="s">
         <v>54</v>
       </c>
-      <c r="B30" s="84"/>
-      <c r="C30" s="84"/>
-      <c r="D30" s="84"/>
+      <c r="B30" s="79"/>
+      <c r="C30" s="79"/>
+      <c r="D30" s="79"/>
     </row>
     <row r="31" spans="1:4" ht="29.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A31" s="87" t="s">
+      <c r="A31" s="82" t="s">
         <v>55</v>
       </c>
-      <c r="B31" s="84"/>
-      <c r="C31" s="84"/>
-      <c r="D31" s="84"/>
+      <c r="B31" s="79"/>
+      <c r="C31" s="79"/>
+      <c r="D31" s="79"/>
     </row>
     <row r="32" spans="1:4" ht="35.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A32" s="87" t="s">
+      <c r="A32" s="82" t="s">
         <v>56</v>
       </c>
-      <c r="B32" s="84"/>
-      <c r="C32" s="84"/>
-      <c r="D32" s="84"/>
+      <c r="B32" s="79"/>
+      <c r="C32" s="79"/>
+      <c r="D32" s="79"/>
     </row>
     <row r="33" spans="1:4" ht="30.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A33" s="87" t="s">
+      <c r="A33" s="82" t="s">
         <v>57</v>
       </c>
-      <c r="B33" s="84"/>
-      <c r="C33" s="84"/>
-      <c r="D33" s="84"/>
+      <c r="B33" s="79"/>
+      <c r="C33" s="79"/>
+      <c r="D33" s="79"/>
     </row>
     <row r="34" spans="1:4" ht="30.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A34" s="87" t="s">
+      <c r="A34" s="82" t="s">
         <v>58</v>
       </c>
-      <c r="B34" s="84"/>
-      <c r="C34" s="84"/>
-      <c r="D34" s="84"/>
+      <c r="B34" s="79"/>
+      <c r="C34" s="79"/>
+      <c r="D34" s="79"/>
     </row>
     <row r="35" spans="1:4" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A35" s="87" t="s">
+      <c r="A35" s="82" t="s">
         <v>59</v>
       </c>
-      <c r="B35" s="84"/>
-      <c r="C35" s="84"/>
-      <c r="D35" s="84"/>
+      <c r="B35" s="79"/>
+      <c r="C35" s="79"/>
+      <c r="D35" s="79"/>
     </row>
     <row r="36" spans="1:4" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A36" s="87"/>
-      <c r="B36" s="84"/>
-      <c r="C36" s="84"/>
-      <c r="D36" s="84"/>
+      <c r="A36" s="82"/>
+      <c r="B36" s="79"/>
+      <c r="C36" s="79"/>
+      <c r="D36" s="79"/>
     </row>
     <row r="37" spans="1:4" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A37" s="89" t="s">
+      <c r="A37" s="84" t="s">
         <v>60</v>
       </c>
-      <c r="B37" s="84"/>
-      <c r="C37" s="84"/>
-      <c r="D37" s="84"/>
+      <c r="B37" s="79"/>
+      <c r="C37" s="79"/>
+      <c r="D37" s="79"/>
     </row>
     <row r="38" spans="1:4" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A38" s="87" t="s">
+      <c r="A38" s="82" t="s">
         <v>61</v>
       </c>
-      <c r="B38" s="84"/>
-      <c r="C38" s="84"/>
-      <c r="D38" s="84"/>
+      <c r="B38" s="79"/>
+      <c r="C38" s="79"/>
+      <c r="D38" s="79"/>
     </row>
     <row r="39" spans="1:4" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A39" s="87" t="s">
+      <c r="A39" s="82" t="s">
         <v>62</v>
       </c>
-      <c r="B39" s="84"/>
-      <c r="C39" s="84"/>
-      <c r="D39" s="84"/>
+      <c r="B39" s="79"/>
+      <c r="C39" s="79"/>
+      <c r="D39" s="79"/>
     </row>
     <row r="40" spans="1:4" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A40" s="87" t="s">
+      <c r="A40" s="82" t="s">
         <v>63</v>
       </c>
-      <c r="B40" s="84"/>
-      <c r="C40" s="84"/>
-      <c r="D40" s="84"/>
+      <c r="B40" s="79"/>
+      <c r="C40" s="79"/>
+      <c r="D40" s="79"/>
     </row>
     <row r="41" spans="1:4" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A41" s="87" t="s">
+      <c r="A41" s="82" t="s">
         <v>64</v>
       </c>
-      <c r="B41" s="84"/>
-      <c r="C41" s="84"/>
-      <c r="D41" s="84"/>
+      <c r="B41" s="79"/>
+      <c r="C41" s="79"/>
+      <c r="D41" s="79"/>
     </row>
     <row r="42" spans="1:4" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A42" s="87" t="s">
+      <c r="A42" s="82" t="s">
         <v>65</v>
       </c>
-      <c r="B42" s="84"/>
-      <c r="C42" s="84"/>
-      <c r="D42" s="84"/>
+      <c r="B42" s="79"/>
+      <c r="C42" s="79"/>
+      <c r="D42" s="79"/>
     </row>
     <row r="43" spans="1:4" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A43" s="87" t="s">
+      <c r="A43" s="82" t="s">
         <v>66</v>
       </c>
-      <c r="B43" s="84"/>
-      <c r="C43" s="84"/>
-      <c r="D43" s="84"/>
+      <c r="B43" s="79"/>
+      <c r="C43" s="79"/>
+      <c r="D43" s="79"/>
     </row>
     <row r="44" spans="1:4" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A44" s="87"/>
-      <c r="B44" s="84"/>
-      <c r="C44" s="84"/>
-      <c r="D44" s="84"/>
+      <c r="A44" s="82"/>
+      <c r="B44" s="79"/>
+      <c r="C44" s="79"/>
+      <c r="D44" s="79"/>
     </row>
     <row r="45" spans="1:4" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A45" s="89" t="s">
+      <c r="A45" s="84" t="s">
         <v>67</v>
       </c>
-      <c r="B45" s="84"/>
-      <c r="C45" s="84"/>
-      <c r="D45" s="84"/>
+      <c r="B45" s="79"/>
+      <c r="C45" s="79"/>
+      <c r="D45" s="79"/>
     </row>
     <row r="46" spans="1:4" ht="37.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A46" s="87" t="s">
+      <c r="A46" s="82" t="s">
         <v>68</v>
       </c>
-      <c r="B46" s="84"/>
-      <c r="C46" s="84"/>
-      <c r="D46" s="84"/>
+      <c r="B46" s="79"/>
+      <c r="C46" s="79"/>
+      <c r="D46" s="79"/>
     </row>
     <row r="47" spans="1:4" ht="30.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A47" s="87" t="s">
+      <c r="A47" s="82" t="s">
         <v>69</v>
       </c>
-      <c r="B47" s="84"/>
-      <c r="C47" s="84"/>
-      <c r="D47" s="84"/>
+      <c r="B47" s="79"/>
+      <c r="C47" s="79"/>
+      <c r="D47" s="79"/>
     </row>
     <row r="48" spans="1:4" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A48" s="87" t="s">
+      <c r="A48" s="82" t="s">
         <v>70</v>
       </c>
-      <c r="B48" s="84"/>
-      <c r="C48" s="84"/>
-      <c r="D48" s="84"/>
+      <c r="B48" s="79"/>
+      <c r="C48" s="79"/>
+      <c r="D48" s="79"/>
     </row>
     <row r="49" spans="1:4" ht="48" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A49" s="87" t="s">
+      <c r="A49" s="82" t="s">
         <v>71</v>
       </c>
-      <c r="B49" s="84"/>
-      <c r="C49" s="84"/>
-      <c r="D49" s="84"/>
+      <c r="B49" s="79"/>
+      <c r="C49" s="79"/>
+      <c r="D49" s="79"/>
     </row>
     <row r="50" spans="1:4" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A50" s="87"/>
-      <c r="B50" s="84"/>
-      <c r="C50" s="84"/>
-      <c r="D50" s="84"/>
+      <c r="A50" s="82"/>
+      <c r="B50" s="79"/>
+      <c r="C50" s="79"/>
+      <c r="D50" s="79"/>
     </row>
     <row r="51" spans="1:4" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A51" s="89" t="s">
+      <c r="A51" s="84" t="s">
         <v>72</v>
       </c>
-      <c r="B51" s="84"/>
-      <c r="C51" s="84"/>
-      <c r="D51" s="84"/>
+      <c r="B51" s="79"/>
+      <c r="C51" s="79"/>
+      <c r="D51" s="79"/>
     </row>
     <row r="52" spans="1:4" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A52" s="87" t="s">
+      <c r="A52" s="82" t="s">
         <v>73</v>
       </c>
-      <c r="B52" s="84"/>
-      <c r="C52" s="84"/>
-      <c r="D52" s="84"/>
+      <c r="B52" s="79"/>
+      <c r="C52" s="79"/>
+      <c r="D52" s="79"/>
     </row>
     <row r="53" spans="1:4" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A53" s="87" t="s">
+      <c r="A53" s="82" t="s">
         <v>74</v>
       </c>
-      <c r="B53" s="84"/>
-      <c r="C53" s="84"/>
-      <c r="D53" s="84"/>
+      <c r="B53" s="79"/>
+      <c r="C53" s="79"/>
+      <c r="D53" s="79"/>
     </row>
     <row r="54" spans="1:4" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A54" s="87" t="s">
+      <c r="A54" s="82" t="s">
         <v>75</v>
       </c>
-      <c r="B54" s="84"/>
-      <c r="C54" s="84"/>
-      <c r="D54" s="84"/>
+      <c r="B54" s="79"/>
+      <c r="C54" s="79"/>
+      <c r="D54" s="79"/>
     </row>
     <row r="55" spans="1:4" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A55" s="87" t="s">
+      <c r="A55" s="82" t="s">
         <v>76</v>
       </c>
-      <c r="B55" s="84"/>
-      <c r="C55" s="84"/>
-      <c r="D55" s="84"/>
+      <c r="B55" s="79"/>
+      <c r="C55" s="79"/>
+      <c r="D55" s="79"/>
     </row>
     <row r="56" spans="1:4" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A56" s="87" t="s">
+      <c r="A56" s="82" t="s">
         <v>77</v>
       </c>
-      <c r="B56" s="84"/>
-      <c r="C56" s="84"/>
-      <c r="D56" s="84"/>
+      <c r="B56" s="79"/>
+      <c r="C56" s="79"/>
+      <c r="D56" s="79"/>
     </row>
     <row r="57" spans="1:4" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A57" s="87" t="s">
+      <c r="A57" s="82" t="s">
         <v>78</v>
       </c>
-      <c r="B57" s="84"/>
-      <c r="C57" s="84"/>
-      <c r="D57" s="84"/>
+      <c r="B57" s="79"/>
+      <c r="C57" s="79"/>
+      <c r="D57" s="79"/>
     </row>
     <row r="58" spans="1:4" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A58" s="87" t="s">
+      <c r="A58" s="82" t="s">
         <v>79</v>
       </c>
-      <c r="B58" s="84"/>
-      <c r="C58" s="84"/>
-      <c r="D58" s="84"/>
+      <c r="B58" s="79"/>
+      <c r="C58" s="79"/>
+      <c r="D58" s="79"/>
     </row>
     <row r="59" spans="1:4" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A59" s="87"/>
-      <c r="B59" s="84"/>
-      <c r="C59" s="84"/>
-      <c r="D59" s="84"/>
+      <c r="A59" s="82"/>
+      <c r="B59" s="79"/>
+      <c r="C59" s="79"/>
+      <c r="D59" s="79"/>
     </row>
     <row r="60" spans="1:4" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A60" s="89" t="s">
+      <c r="A60" s="84" t="s">
         <v>80</v>
       </c>
-      <c r="B60" s="84"/>
-      <c r="C60" s="84"/>
-      <c r="D60" s="84"/>
+      <c r="B60" s="79"/>
+      <c r="C60" s="79"/>
+      <c r="D60" s="79"/>
     </row>
     <row r="61" spans="1:4" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A61" s="87" t="s">
+      <c r="A61" s="82" t="s">
         <v>81</v>
       </c>
-      <c r="B61" s="84"/>
-      <c r="C61" s="84"/>
-      <c r="D61" s="84"/>
+      <c r="B61" s="79"/>
+      <c r="C61" s="79"/>
+      <c r="D61" s="79"/>
     </row>
     <row r="62" spans="1:4" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A62" s="87" t="s">
+      <c r="A62" s="82" t="s">
         <v>82</v>
       </c>
-      <c r="B62" s="84"/>
-      <c r="C62" s="84"/>
-      <c r="D62" s="84"/>
+      <c r="B62" s="79"/>
+      <c r="C62" s="79"/>
+      <c r="D62" s="79"/>
     </row>
     <row r="63" spans="1:4" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A63" s="87" t="s">
+      <c r="A63" s="82" t="s">
         <v>83</v>
       </c>
-      <c r="B63" s="84"/>
-      <c r="C63" s="84"/>
-      <c r="D63" s="84"/>
+      <c r="B63" s="79"/>
+      <c r="C63" s="79"/>
+      <c r="D63" s="79"/>
     </row>
     <row r="64" spans="1:4" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A64" s="87" t="s">
+      <c r="A64" s="82" t="s">
         <v>84</v>
       </c>
-      <c r="B64" s="84"/>
-      <c r="C64" s="84"/>
-      <c r="D64" s="84"/>
+      <c r="B64" s="79"/>
+      <c r="C64" s="79"/>
+      <c r="D64" s="79"/>
     </row>
     <row r="65" spans="1:4" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A65" s="87" t="s">
+      <c r="A65" s="82" t="s">
         <v>85</v>
       </c>
-      <c r="B65" s="84"/>
-      <c r="C65" s="84"/>
-      <c r="D65" s="84"/>
+      <c r="B65" s="79"/>
+      <c r="C65" s="79"/>
+      <c r="D65" s="79"/>
     </row>
     <row r="66" spans="1:4" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A66" s="87" t="s">
+      <c r="A66" s="82" t="s">
         <v>86</v>
       </c>
-      <c r="B66" s="84"/>
-      <c r="C66" s="84"/>
-      <c r="D66" s="84"/>
+      <c r="B66" s="79"/>
+      <c r="C66" s="79"/>
+      <c r="D66" s="79"/>
     </row>
   </sheetData>
   <mergeCells count="47">
@@ -11515,42 +11530,42 @@
       <c r="J39" s="29"/>
     </row>
     <row r="41" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A41" s="83" t="s">
+      <c r="A41" s="78" t="s">
         <v>117</v>
       </c>
-      <c r="B41" s="84"/>
-      <c r="C41" s="84"/>
-      <c r="D41" s="84"/>
-      <c r="E41" s="84"/>
-      <c r="F41" s="84"/>
-      <c r="G41" s="84"/>
-      <c r="H41" s="84"/>
-      <c r="I41" s="84"/>
-      <c r="J41" s="84"/>
+      <c r="B41" s="79"/>
+      <c r="C41" s="79"/>
+      <c r="D41" s="79"/>
+      <c r="E41" s="79"/>
+      <c r="F41" s="79"/>
+      <c r="G41" s="79"/>
+      <c r="H41" s="79"/>
+      <c r="I41" s="79"/>
+      <c r="J41" s="79"/>
     </row>
     <row r="42" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A42" s="84"/>
-      <c r="B42" s="84"/>
-      <c r="C42" s="84"/>
-      <c r="D42" s="84"/>
-      <c r="E42" s="84"/>
-      <c r="F42" s="84"/>
-      <c r="G42" s="84"/>
-      <c r="H42" s="84"/>
-      <c r="I42" s="84"/>
-      <c r="J42" s="84"/>
+      <c r="A42" s="79"/>
+      <c r="B42" s="79"/>
+      <c r="C42" s="79"/>
+      <c r="D42" s="79"/>
+      <c r="E42" s="79"/>
+      <c r="F42" s="79"/>
+      <c r="G42" s="79"/>
+      <c r="H42" s="79"/>
+      <c r="I42" s="79"/>
+      <c r="J42" s="79"/>
     </row>
     <row r="43" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A43" s="84"/>
-      <c r="B43" s="84"/>
-      <c r="C43" s="84"/>
-      <c r="D43" s="84"/>
-      <c r="E43" s="84"/>
-      <c r="F43" s="84"/>
-      <c r="G43" s="84"/>
-      <c r="H43" s="84"/>
-      <c r="I43" s="84"/>
-      <c r="J43" s="84"/>
+      <c r="A43" s="79"/>
+      <c r="B43" s="79"/>
+      <c r="C43" s="79"/>
+      <c r="D43" s="79"/>
+      <c r="E43" s="79"/>
+      <c r="F43" s="79"/>
+      <c r="G43" s="79"/>
+      <c r="H43" s="79"/>
+      <c r="I43" s="79"/>
+      <c r="J43" s="79"/>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -11846,24 +11861,24 @@
       <c r="G24" s="29"/>
     </row>
     <row r="26" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A26" s="83" t="s">
+      <c r="A26" s="78" t="s">
         <v>134</v>
       </c>
-      <c r="B26" s="84"/>
-      <c r="C26" s="84"/>
-      <c r="D26" s="84"/>
-      <c r="E26" s="84"/>
-      <c r="F26" s="84"/>
-      <c r="G26" s="84"/>
+      <c r="B26" s="79"/>
+      <c r="C26" s="79"/>
+      <c r="D26" s="79"/>
+      <c r="E26" s="79"/>
+      <c r="F26" s="79"/>
+      <c r="G26" s="79"/>
     </row>
     <row r="27" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A27" s="84"/>
-      <c r="B27" s="84"/>
-      <c r="C27" s="84"/>
-      <c r="D27" s="84"/>
-      <c r="E27" s="84"/>
-      <c r="F27" s="84"/>
-      <c r="G27" s="84"/>
+      <c r="A27" s="79"/>
+      <c r="B27" s="79"/>
+      <c r="C27" s="79"/>
+      <c r="D27" s="79"/>
+      <c r="E27" s="79"/>
+      <c r="F27" s="79"/>
+      <c r="G27" s="79"/>
     </row>
   </sheetData>
   <mergeCells count="1">

</xml_diff>

<commit_message>
chore(holomap): met a jour le gabarit carte_holomap.xlsx
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Carte Holo/carte_holomap.xlsx
+++ b/Carte Holo/carte_holomap.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Projets\IdleEvolution\Carte Holo\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{20049AA6-2974-49E6-8853-8A1AAABC2769}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7E30374E-4982-48EB-BD4A-E45FE83E6DBC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1551,7 +1551,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="119">
+  <cellXfs count="117">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -1631,7 +1631,6 @@
     <xf numFmtId="0" fontId="0" fillId="10" borderId="28" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="10" borderId="29" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="10" borderId="30" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="30" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="8" borderId="31" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="8" borderId="32" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="10" borderId="20" xfId="0" applyFill="1" applyBorder="1"/>
@@ -1650,23 +1649,6 @@
     <xf numFmtId="0" fontId="0" fillId="8" borderId="43" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="8" borderId="20" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="9" borderId="20" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="6" borderId="45" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="8" borderId="46" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="8" borderId="47" xfId="0" applyFill="1" applyBorder="1"/>
@@ -1683,7 +1665,6 @@
     <xf numFmtId="0" fontId="0" fillId="8" borderId="59" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="8" borderId="60" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="8" borderId="44" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="14" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="14" borderId="2" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="14" borderId="46" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="14" borderId="47" xfId="0" applyFill="1" applyBorder="1"/>
@@ -1693,12 +1674,29 @@
     <xf numFmtId="0" fontId="0" fillId="14" borderId="49" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="14" borderId="50" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="14" borderId="51" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="8" borderId="0" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="8" borderId="63" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="8" borderId="64" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="8" borderId="65" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="8" borderId="66" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="8" borderId="67" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -2015,11 +2013,11 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="A1" s="80" t="s">
+      <c r="A1" s="108" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="79"/>
-      <c r="C1" s="79"/>
+      <c r="B1" s="109"/>
+      <c r="C1" s="109"/>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
@@ -2077,11 +2075,11 @@
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A9" s="81" t="s">
+      <c r="A9" s="110" t="s">
         <v>13</v>
       </c>
-      <c r="B9" s="79"/>
-      <c r="C9" s="79"/>
+      <c r="B9" s="109"/>
+      <c r="C9" s="109"/>
     </row>
   </sheetData>
   <mergeCells count="2">
@@ -3352,16 +3350,16 @@
       <c r="T18" s="7"/>
       <c r="U18" s="7"/>
       <c r="V18" s="7"/>
-      <c r="W18" s="15"/>
-      <c r="X18" s="7"/>
-      <c r="Y18" s="7"/>
-      <c r="Z18" s="7"/>
-      <c r="AA18" s="7"/>
-      <c r="AB18" s="7"/>
-      <c r="AC18" s="7"/>
-      <c r="AD18" s="7"/>
-      <c r="AE18" s="7"/>
-      <c r="AF18" s="7"/>
+      <c r="W18" s="14"/>
+      <c r="X18" s="14"/>
+      <c r="Y18" s="14"/>
+      <c r="Z18" s="14"/>
+      <c r="AA18" s="14"/>
+      <c r="AB18" s="14"/>
+      <c r="AC18" s="14"/>
+      <c r="AD18" s="14"/>
+      <c r="AE18" s="14"/>
+      <c r="AF18" s="14"/>
       <c r="AG18" s="7"/>
       <c r="AH18" s="7"/>
       <c r="AI18" s="7"/>
@@ -3417,7 +3415,7 @@
       <c r="T19" s="7"/>
       <c r="U19" s="7"/>
       <c r="V19" s="7"/>
-      <c r="W19" s="15"/>
+      <c r="W19" s="14"/>
       <c r="X19" s="14"/>
       <c r="Y19" s="43"/>
       <c r="Z19" s="43"/>
@@ -3426,7 +3424,7 @@
       <c r="AC19" s="43"/>
       <c r="AD19" s="43"/>
       <c r="AE19" s="14"/>
-      <c r="AF19" s="7"/>
+      <c r="AF19" s="14"/>
       <c r="AG19" s="7"/>
       <c r="AH19" s="7"/>
       <c r="AI19" s="7"/>
@@ -3482,16 +3480,16 @@
       <c r="T20" s="7"/>
       <c r="U20" s="7"/>
       <c r="V20" s="7"/>
-      <c r="W20" s="15"/>
-      <c r="X20" s="66"/>
-      <c r="Y20" s="88"/>
-      <c r="Z20" s="89"/>
-      <c r="AA20" s="89"/>
-      <c r="AB20" s="89"/>
-      <c r="AC20" s="94"/>
-      <c r="AD20" s="99"/>
+      <c r="W20" s="14"/>
+      <c r="X20" s="65"/>
+      <c r="Y20" s="78"/>
+      <c r="Z20" s="79"/>
+      <c r="AA20" s="79"/>
+      <c r="AB20" s="79"/>
+      <c r="AC20" s="84"/>
+      <c r="AD20" s="89"/>
       <c r="AE20" s="55"/>
-      <c r="AF20" s="7"/>
+      <c r="AF20" s="14"/>
       <c r="AG20" s="7"/>
       <c r="AH20" s="7"/>
       <c r="AI20" s="7"/>
@@ -3540,7 +3538,7 @@
       <c r="M21" s="7"/>
       <c r="N21" s="7"/>
       <c r="O21" s="7"/>
-      <c r="P21" s="14"/>
+      <c r="P21" s="7"/>
       <c r="Q21" s="14"/>
       <c r="R21" s="43"/>
       <c r="S21" s="43"/>
@@ -3548,17 +3546,17 @@
       <c r="U21" s="43"/>
       <c r="V21" s="43"/>
       <c r="W21" s="14"/>
-      <c r="X21" s="66"/>
-      <c r="Y21" s="96"/>
-      <c r="Z21" s="97"/>
-      <c r="AA21" s="97" t="s">
+      <c r="X21" s="65"/>
+      <c r="Y21" s="86"/>
+      <c r="Z21" s="87"/>
+      <c r="AA21" s="87" t="s">
         <v>139</v>
       </c>
-      <c r="AB21" s="97"/>
-      <c r="AC21" s="98"/>
-      <c r="AD21" s="100"/>
+      <c r="AB21" s="87"/>
+      <c r="AC21" s="88"/>
+      <c r="AD21" s="90"/>
       <c r="AE21" s="55"/>
-      <c r="AF21" s="7"/>
+      <c r="AF21" s="14"/>
       <c r="AG21" s="7"/>
       <c r="AH21" s="7"/>
       <c r="AI21" s="7"/>
@@ -3607,33 +3605,33 @@
       <c r="M22" s="7"/>
       <c r="N22" s="7"/>
       <c r="O22" s="7"/>
-      <c r="P22" s="14"/>
-      <c r="Q22" s="66"/>
-      <c r="R22" s="102">
+      <c r="P22" s="7"/>
+      <c r="Q22" s="65"/>
+      <c r="R22" s="92">
         <v>6</v>
       </c>
-      <c r="S22" s="102">
+      <c r="S22" s="92">
         <v>4</v>
       </c>
-      <c r="T22" s="102">
+      <c r="T22" s="92">
         <v>8</v>
       </c>
-      <c r="U22" s="102">
+      <c r="U22" s="92">
         <v>9</v>
       </c>
-      <c r="V22" s="102">
+      <c r="V22" s="92">
         <v>4</v>
       </c>
-      <c r="W22" s="103"/>
-      <c r="X22" s="66"/>
-      <c r="Y22" s="95"/>
-      <c r="Z22" s="76"/>
-      <c r="AA22" s="76"/>
-      <c r="AB22" s="76"/>
-      <c r="AC22" s="92"/>
-      <c r="AD22" s="100"/>
+      <c r="W22" s="14"/>
+      <c r="X22" s="65"/>
+      <c r="Y22" s="85"/>
+      <c r="Z22" s="75"/>
+      <c r="AA22" s="75"/>
+      <c r="AB22" s="75"/>
+      <c r="AC22" s="82"/>
+      <c r="AD22" s="90"/>
       <c r="AE22" s="55"/>
-      <c r="AF22" s="7"/>
+      <c r="AF22" s="14"/>
       <c r="AG22" s="7"/>
       <c r="AH22" s="7"/>
       <c r="AI22" s="7"/>
@@ -3683,32 +3681,32 @@
       <c r="N23" s="14"/>
       <c r="O23" s="14"/>
       <c r="P23" s="14"/>
-      <c r="Q23" s="66"/>
-      <c r="R23" s="102">
+      <c r="Q23" s="65"/>
+      <c r="R23" s="92">
         <v>6</v>
       </c>
-      <c r="S23" s="102">
+      <c r="S23" s="92">
         <v>7</v>
       </c>
-      <c r="T23" s="102">
+      <c r="T23" s="92">
         <v>8</v>
       </c>
-      <c r="U23" s="102">
+      <c r="U23" s="92">
         <v>9</v>
       </c>
-      <c r="V23" s="102">
+      <c r="V23" s="92">
         <v>5</v>
       </c>
-      <c r="W23" s="103"/>
-      <c r="X23" s="66"/>
-      <c r="Y23" s="90"/>
-      <c r="Z23" s="91"/>
-      <c r="AA23" s="91"/>
-      <c r="AB23" s="91"/>
-      <c r="AC23" s="93"/>
-      <c r="AD23" s="101"/>
+      <c r="W23" s="14"/>
+      <c r="X23" s="65"/>
+      <c r="Y23" s="80"/>
+      <c r="Z23" s="81"/>
+      <c r="AA23" s="81"/>
+      <c r="AB23" s="81"/>
+      <c r="AC23" s="83"/>
+      <c r="AD23" s="91"/>
       <c r="AE23" s="55"/>
-      <c r="AF23" s="7"/>
+      <c r="AF23" s="14"/>
       <c r="AG23" s="7"/>
       <c r="AH23" s="7"/>
       <c r="AI23" s="7"/>
@@ -3757,23 +3755,23 @@
       <c r="M24" s="12"/>
       <c r="N24" s="12"/>
       <c r="O24" s="12"/>
-      <c r="P24" s="14"/>
+      <c r="P24" s="54"/>
       <c r="Q24" s="14"/>
-      <c r="R24" s="70"/>
-      <c r="S24" s="70"/>
-      <c r="T24" s="70"/>
-      <c r="U24" s="70"/>
-      <c r="V24" s="70"/>
+      <c r="R24" s="69"/>
+      <c r="S24" s="69"/>
+      <c r="T24" s="69"/>
+      <c r="U24" s="69"/>
+      <c r="V24" s="69"/>
       <c r="W24" s="43"/>
       <c r="X24" s="43"/>
-      <c r="Y24" s="87"/>
-      <c r="Z24" s="87"/>
-      <c r="AA24" s="70"/>
-      <c r="AB24" s="70"/>
-      <c r="AC24" s="70"/>
+      <c r="Y24" s="77"/>
+      <c r="Z24" s="77"/>
+      <c r="AA24" s="69"/>
+      <c r="AB24" s="69"/>
+      <c r="AC24" s="69"/>
       <c r="AD24" s="14"/>
       <c r="AE24" s="14"/>
-      <c r="AF24" s="7"/>
+      <c r="AF24" s="14"/>
       <c r="AG24" s="7"/>
       <c r="AH24" s="7"/>
       <c r="AI24" s="7"/>
@@ -3819,10 +3817,10 @@
       <c r="J25" s="14"/>
       <c r="K25" s="14"/>
       <c r="L25" s="14"/>
-      <c r="M25" s="14"/>
+      <c r="M25" s="62"/>
       <c r="N25" s="12"/>
       <c r="O25" s="12"/>
-      <c r="P25" s="14"/>
+      <c r="P25" s="54"/>
       <c r="Q25" s="14"/>
       <c r="R25" s="12"/>
       <c r="S25" s="12"/>
@@ -3835,9 +3833,9 @@
       <c r="Z25" s="48"/>
       <c r="AA25" s="48"/>
       <c r="AB25" s="16"/>
-      <c r="AC25" s="16"/>
+      <c r="AC25" s="14"/>
       <c r="AD25" s="14"/>
-      <c r="AE25" s="14"/>
+      <c r="AE25" s="7"/>
       <c r="AF25" s="7"/>
       <c r="AG25" s="7"/>
       <c r="AH25" s="7"/>
@@ -3883,7 +3881,7 @@
       <c r="I26" s="7"/>
       <c r="J26" s="7"/>
       <c r="K26" s="7"/>
-      <c r="L26" s="7"/>
+      <c r="L26" s="14"/>
       <c r="M26" s="14"/>
       <c r="N26" s="43"/>
       <c r="O26" s="43"/>
@@ -3900,9 +3898,9 @@
       <c r="Z26" s="48"/>
       <c r="AA26" s="48"/>
       <c r="AB26" s="16"/>
-      <c r="AC26" s="16"/>
+      <c r="AC26" s="14"/>
       <c r="AD26" s="14"/>
-      <c r="AE26" s="14"/>
+      <c r="AE26" s="7"/>
       <c r="AF26" s="7"/>
       <c r="AG26" s="7"/>
       <c r="AH26" s="7"/>
@@ -3948,11 +3946,11 @@
       <c r="I27" s="7"/>
       <c r="J27" s="7"/>
       <c r="K27" s="7"/>
-      <c r="L27" s="7"/>
-      <c r="M27" s="52"/>
+      <c r="L27" s="14"/>
+      <c r="M27" s="62"/>
       <c r="N27" s="53"/>
       <c r="O27" s="54"/>
-      <c r="P27" s="55"/>
+      <c r="P27" s="54"/>
       <c r="Q27" s="14"/>
       <c r="R27" s="16"/>
       <c r="S27" s="16"/>
@@ -4014,20 +4012,20 @@
       <c r="J28" s="7"/>
       <c r="K28" s="7"/>
       <c r="L28" s="14"/>
-      <c r="M28" s="59"/>
-      <c r="N28" s="60"/>
-      <c r="O28" s="61"/>
-      <c r="P28" s="55"/>
+      <c r="M28" s="62"/>
+      <c r="N28" s="59"/>
+      <c r="O28" s="60"/>
+      <c r="P28" s="54"/>
       <c r="Q28" s="14"/>
       <c r="R28" s="12"/>
       <c r="S28" s="12"/>
       <c r="T28" s="16"/>
       <c r="U28" s="12"/>
       <c r="V28" s="12"/>
-      <c r="W28" s="62"/>
-      <c r="X28" s="62"/>
-      <c r="Y28" s="62"/>
-      <c r="Z28" s="62"/>
+      <c r="W28" s="61"/>
+      <c r="X28" s="61"/>
+      <c r="Y28" s="61"/>
+      <c r="Z28" s="61"/>
       <c r="AA28" s="14"/>
       <c r="AB28" s="14"/>
       <c r="AC28" s="43"/>
@@ -4079,10 +4077,10 @@
       <c r="J29" s="7"/>
       <c r="K29" s="7"/>
       <c r="L29" s="52"/>
-      <c r="M29" s="63"/>
-      <c r="N29" s="64"/>
-      <c r="O29" s="65"/>
-      <c r="P29" s="55"/>
+      <c r="M29" s="62"/>
+      <c r="N29" s="63"/>
+      <c r="O29" s="64"/>
+      <c r="P29" s="54"/>
       <c r="Q29" s="14"/>
       <c r="R29" s="12"/>
       <c r="S29" s="12"/>
@@ -4094,12 +4092,12 @@
       <c r="Y29" s="16"/>
       <c r="Z29" s="16"/>
       <c r="AA29" s="14"/>
-      <c r="AB29" s="66"/>
-      <c r="AC29" s="67"/>
-      <c r="AD29" s="68"/>
-      <c r="AE29" s="68"/>
-      <c r="AF29" s="68"/>
-      <c r="AG29" s="69"/>
+      <c r="AB29" s="65"/>
+      <c r="AC29" s="66"/>
+      <c r="AD29" s="67"/>
+      <c r="AE29" s="67"/>
+      <c r="AF29" s="67"/>
+      <c r="AG29" s="68"/>
       <c r="AH29" s="55"/>
       <c r="AI29" s="14"/>
       <c r="AJ29" s="7"/>
@@ -4144,9 +4142,9 @@
       <c r="J30" s="7"/>
       <c r="K30" s="7"/>
       <c r="L30" s="14"/>
-      <c r="M30" s="70"/>
-      <c r="N30" s="70"/>
-      <c r="O30" s="70"/>
+      <c r="M30" s="69"/>
+      <c r="N30" s="69"/>
+      <c r="O30" s="69"/>
       <c r="P30" s="14"/>
       <c r="Q30" s="14"/>
       <c r="R30" s="12"/>
@@ -4159,12 +4157,12 @@
       <c r="Y30" s="16"/>
       <c r="Z30" s="16"/>
       <c r="AA30" s="14"/>
-      <c r="AB30" s="66"/>
-      <c r="AC30" s="71"/>
+      <c r="AB30" s="65"/>
+      <c r="AC30" s="70"/>
       <c r="AD30" s="12"/>
       <c r="AE30" s="12"/>
       <c r="AF30" s="12"/>
-      <c r="AG30" s="72"/>
+      <c r="AG30" s="71"/>
       <c r="AH30" s="55"/>
       <c r="AI30" s="14"/>
       <c r="AJ30" s="7"/>
@@ -4212,7 +4210,7 @@
       <c r="M31" s="7"/>
       <c r="N31" s="7"/>
       <c r="O31" s="7"/>
-      <c r="P31" s="14"/>
+      <c r="P31" s="7"/>
       <c r="Q31" s="14"/>
       <c r="R31" s="12"/>
       <c r="S31" s="12"/>
@@ -4224,14 +4222,14 @@
       <c r="Y31" s="16"/>
       <c r="Z31" s="16"/>
       <c r="AA31" s="14"/>
-      <c r="AB31" s="66"/>
-      <c r="AC31" s="71"/>
+      <c r="AB31" s="65"/>
+      <c r="AC31" s="70"/>
       <c r="AD31" s="12"/>
       <c r="AE31" s="12" t="s">
         <v>136</v>
       </c>
       <c r="AF31" s="12"/>
-      <c r="AG31" s="72"/>
+      <c r="AG31" s="71"/>
       <c r="AH31" s="55"/>
       <c r="AI31" s="14"/>
       <c r="AJ31" s="16"/>
@@ -4279,7 +4277,7 @@
       <c r="M32" s="7"/>
       <c r="N32" s="7"/>
       <c r="O32" s="7"/>
-      <c r="P32" s="14"/>
+      <c r="P32" s="7"/>
       <c r="Q32" s="14"/>
       <c r="R32" s="12"/>
       <c r="S32" s="16"/>
@@ -4291,12 +4289,12 @@
       <c r="Y32" s="16"/>
       <c r="Z32" s="16"/>
       <c r="AA32" s="14"/>
-      <c r="AB32" s="66"/>
-      <c r="AC32" s="71"/>
+      <c r="AB32" s="65"/>
+      <c r="AC32" s="70"/>
       <c r="AD32" s="12"/>
       <c r="AE32" s="12"/>
       <c r="AF32" s="12"/>
-      <c r="AG32" s="72"/>
+      <c r="AG32" s="71"/>
       <c r="AH32" s="55"/>
       <c r="AI32" s="14"/>
       <c r="AJ32" s="16"/>
@@ -4344,7 +4342,7 @@
       <c r="M33" s="7"/>
       <c r="N33" s="7"/>
       <c r="O33" s="7"/>
-      <c r="P33" s="14"/>
+      <c r="P33" s="7"/>
       <c r="Q33" s="14"/>
       <c r="R33" s="16"/>
       <c r="S33" s="12"/>
@@ -4356,12 +4354,12 @@
       <c r="Y33" s="16"/>
       <c r="Z33" s="16"/>
       <c r="AA33" s="14"/>
-      <c r="AB33" s="66"/>
-      <c r="AC33" s="73"/>
-      <c r="AD33" s="74"/>
-      <c r="AE33" s="74"/>
-      <c r="AF33" s="74"/>
-      <c r="AG33" s="75"/>
+      <c r="AB33" s="65"/>
+      <c r="AC33" s="72"/>
+      <c r="AD33" s="73"/>
+      <c r="AE33" s="73"/>
+      <c r="AF33" s="73"/>
+      <c r="AG33" s="74"/>
       <c r="AH33" s="55"/>
       <c r="AI33" s="14"/>
       <c r="AJ33" s="16"/>
@@ -4422,11 +4420,11 @@
       <c r="Z34" s="14"/>
       <c r="AA34" s="14"/>
       <c r="AB34" s="14"/>
-      <c r="AC34" s="70"/>
-      <c r="AD34" s="70"/>
-      <c r="AE34" s="70"/>
-      <c r="AF34" s="70"/>
-      <c r="AG34" s="70"/>
+      <c r="AC34" s="69"/>
+      <c r="AD34" s="69"/>
+      <c r="AE34" s="69"/>
+      <c r="AF34" s="69"/>
+      <c r="AG34" s="69"/>
       <c r="AH34" s="14"/>
       <c r="AI34" s="14"/>
       <c r="AJ34" s="14"/>
@@ -4539,7 +4537,7 @@
       <c r="M36" s="7"/>
       <c r="N36" s="7"/>
       <c r="O36" s="7"/>
-      <c r="P36" s="14"/>
+      <c r="P36" s="7"/>
       <c r="Q36" s="14"/>
       <c r="R36" s="7"/>
       <c r="S36" s="7"/>
@@ -4551,13 +4549,13 @@
       <c r="Y36" s="16"/>
       <c r="Z36" s="16"/>
       <c r="AA36" s="14"/>
-      <c r="AB36" s="66"/>
-      <c r="AC36" s="114"/>
-      <c r="AD36" s="115"/>
-      <c r="AE36" s="115"/>
-      <c r="AF36" s="115"/>
-      <c r="AG36" s="115"/>
-      <c r="AH36" s="99"/>
+      <c r="AB36" s="65"/>
+      <c r="AC36" s="103"/>
+      <c r="AD36" s="104"/>
+      <c r="AE36" s="104"/>
+      <c r="AF36" s="104"/>
+      <c r="AG36" s="104"/>
+      <c r="AH36" s="89"/>
       <c r="AI36" s="55"/>
       <c r="AJ36" s="16"/>
       <c r="AK36" s="16"/>
@@ -4566,17 +4564,17 @@
       <c r="AN36" s="7"/>
       <c r="AO36" s="7"/>
       <c r="AP36" s="7"/>
-      <c r="AQ36" s="7"/>
-      <c r="AR36" s="66"/>
-      <c r="AS36" s="105"/>
-      <c r="AT36" s="106"/>
-      <c r="AU36" s="106"/>
-      <c r="AV36" s="106"/>
-      <c r="AW36" s="106"/>
-      <c r="AX36" s="106"/>
-      <c r="AY36" s="106"/>
-      <c r="AZ36" s="106"/>
-      <c r="BA36" s="107"/>
+      <c r="AQ36" s="14"/>
+      <c r="AR36" s="65"/>
+      <c r="AS36" s="94"/>
+      <c r="AT36" s="95"/>
+      <c r="AU36" s="95"/>
+      <c r="AV36" s="95"/>
+      <c r="AW36" s="95"/>
+      <c r="AX36" s="95"/>
+      <c r="AY36" s="95"/>
+      <c r="AZ36" s="95"/>
+      <c r="BA36" s="96"/>
       <c r="BB36" s="55"/>
       <c r="BC36" s="14"/>
       <c r="BD36" s="7"/>
@@ -4604,11 +4602,11 @@
       <c r="M37" s="7"/>
       <c r="N37" s="7"/>
       <c r="O37" s="7"/>
-      <c r="P37" s="14"/>
+      <c r="P37" s="7"/>
       <c r="Q37" s="14"/>
       <c r="R37" s="14"/>
       <c r="S37" s="14"/>
-      <c r="T37" s="7"/>
+      <c r="T37" s="14"/>
       <c r="U37" s="7"/>
       <c r="V37" s="7"/>
       <c r="W37" s="15"/>
@@ -4616,15 +4614,15 @@
       <c r="Y37" s="16"/>
       <c r="Z37" s="16"/>
       <c r="AA37" s="14"/>
-      <c r="AB37" s="66"/>
-      <c r="AC37" s="116"/>
-      <c r="AD37" s="113"/>
-      <c r="AE37" s="113"/>
-      <c r="AF37" s="113" t="s">
+      <c r="AB37" s="65"/>
+      <c r="AC37" s="105"/>
+      <c r="AD37" s="102"/>
+      <c r="AE37" s="102"/>
+      <c r="AF37" s="102" t="s">
         <v>137</v>
       </c>
-      <c r="AG37" s="113"/>
-      <c r="AH37" s="100"/>
+      <c r="AG37" s="102"/>
+      <c r="AH37" s="90"/>
       <c r="AI37" s="55"/>
       <c r="AJ37" s="16"/>
       <c r="AK37" s="16"/>
@@ -4633,17 +4631,17 @@
       <c r="AN37" s="7"/>
       <c r="AO37" s="7"/>
       <c r="AP37" s="7"/>
-      <c r="AQ37" s="7"/>
-      <c r="AR37" s="66"/>
-      <c r="AS37" s="108"/>
-      <c r="AT37" s="104"/>
-      <c r="AU37" s="104"/>
-      <c r="AV37" s="104"/>
-      <c r="AW37" s="104"/>
-      <c r="AX37" s="104"/>
-      <c r="AY37" s="104"/>
-      <c r="AZ37" s="104"/>
-      <c r="BA37" s="109"/>
+      <c r="AQ37" s="14"/>
+      <c r="AR37" s="65"/>
+      <c r="AS37" s="97"/>
+      <c r="AT37" s="93"/>
+      <c r="AU37" s="93"/>
+      <c r="AV37" s="93"/>
+      <c r="AW37" s="93"/>
+      <c r="AX37" s="93"/>
+      <c r="AY37" s="93"/>
+      <c r="AZ37" s="93"/>
+      <c r="BA37" s="98"/>
       <c r="BB37" s="55"/>
       <c r="BC37" s="14"/>
       <c r="BD37" s="7"/>
@@ -4674,7 +4672,7 @@
       <c r="P38" s="7"/>
       <c r="Q38" s="7"/>
       <c r="R38" s="7"/>
-      <c r="S38" s="14"/>
+      <c r="S38" s="7"/>
       <c r="T38" s="14"/>
       <c r="U38" s="7"/>
       <c r="V38" s="7"/>
@@ -4683,13 +4681,13 @@
       <c r="Y38" s="16"/>
       <c r="Z38" s="16"/>
       <c r="AA38" s="14"/>
-      <c r="AB38" s="66"/>
-      <c r="AC38" s="116"/>
-      <c r="AD38" s="113"/>
-      <c r="AE38" s="113"/>
-      <c r="AF38" s="113"/>
-      <c r="AG38" s="113"/>
-      <c r="AH38" s="100"/>
+      <c r="AB38" s="65"/>
+      <c r="AC38" s="105"/>
+      <c r="AD38" s="102"/>
+      <c r="AE38" s="102"/>
+      <c r="AF38" s="102"/>
+      <c r="AG38" s="102"/>
+      <c r="AH38" s="90"/>
       <c r="AI38" s="55"/>
       <c r="AJ38" s="16"/>
       <c r="AK38" s="16"/>
@@ -4698,17 +4696,17 @@
       <c r="AN38" s="7"/>
       <c r="AO38" s="7"/>
       <c r="AP38" s="7"/>
-      <c r="AQ38" s="7"/>
-      <c r="AR38" s="66"/>
-      <c r="AS38" s="108"/>
-      <c r="AT38" s="104"/>
-      <c r="AU38" s="104"/>
-      <c r="AV38" s="104"/>
-      <c r="AW38" s="104"/>
-      <c r="AX38" s="104"/>
-      <c r="AY38" s="104"/>
-      <c r="AZ38" s="104"/>
-      <c r="BA38" s="109"/>
+      <c r="AQ38" s="14"/>
+      <c r="AR38" s="65"/>
+      <c r="AS38" s="97"/>
+      <c r="AT38" s="93"/>
+      <c r="AU38" s="93"/>
+      <c r="AV38" s="93"/>
+      <c r="AW38" s="93"/>
+      <c r="AX38" s="93"/>
+      <c r="AY38" s="93"/>
+      <c r="AZ38" s="93"/>
+      <c r="BA38" s="98"/>
       <c r="BB38" s="55"/>
       <c r="BC38" s="14"/>
       <c r="BD38" s="7"/>
@@ -4748,13 +4746,13 @@
       <c r="Y39" s="14"/>
       <c r="Z39" s="14"/>
       <c r="AA39" s="14"/>
-      <c r="AB39" s="66"/>
-      <c r="AC39" s="116"/>
-      <c r="AD39" s="113"/>
-      <c r="AE39" s="113"/>
-      <c r="AF39" s="113"/>
-      <c r="AG39" s="113"/>
-      <c r="AH39" s="100"/>
+      <c r="AB39" s="65"/>
+      <c r="AC39" s="105"/>
+      <c r="AD39" s="102"/>
+      <c r="AE39" s="102"/>
+      <c r="AF39" s="102"/>
+      <c r="AG39" s="102"/>
+      <c r="AH39" s="90"/>
       <c r="AI39" s="55"/>
       <c r="AJ39" s="7"/>
       <c r="AK39" s="7"/>
@@ -4763,17 +4761,17 @@
       <c r="AN39" s="7"/>
       <c r="AO39" s="7"/>
       <c r="AP39" s="7"/>
-      <c r="AQ39" s="7"/>
-      <c r="AR39" s="66"/>
-      <c r="AS39" s="108"/>
-      <c r="AT39" s="104"/>
-      <c r="AU39" s="104"/>
-      <c r="AV39" s="104"/>
-      <c r="AW39" s="104"/>
-      <c r="AX39" s="104"/>
-      <c r="AY39" s="104"/>
-      <c r="AZ39" s="104"/>
-      <c r="BA39" s="109"/>
+      <c r="AQ39" s="14"/>
+      <c r="AR39" s="65"/>
+      <c r="AS39" s="97"/>
+      <c r="AT39" s="93"/>
+      <c r="AU39" s="93"/>
+      <c r="AV39" s="93"/>
+      <c r="AW39" s="93"/>
+      <c r="AX39" s="93"/>
+      <c r="AY39" s="93"/>
+      <c r="AZ39" s="93"/>
+      <c r="BA39" s="98"/>
       <c r="BB39" s="55"/>
       <c r="BC39" s="14"/>
       <c r="BD39" s="7"/>
@@ -4813,13 +4811,13 @@
       <c r="Y40" s="7"/>
       <c r="Z40" s="7"/>
       <c r="AA40" s="14"/>
-      <c r="AB40" s="66"/>
-      <c r="AC40" s="117"/>
-      <c r="AD40" s="118"/>
-      <c r="AE40" s="118"/>
-      <c r="AF40" s="118"/>
-      <c r="AG40" s="118"/>
-      <c r="AH40" s="101"/>
+      <c r="AB40" s="65"/>
+      <c r="AC40" s="106"/>
+      <c r="AD40" s="107"/>
+      <c r="AE40" s="107"/>
+      <c r="AF40" s="107"/>
+      <c r="AG40" s="107"/>
+      <c r="AH40" s="91"/>
       <c r="AI40" s="55"/>
       <c r="AJ40" s="7"/>
       <c r="AK40" s="7"/>
@@ -4828,17 +4826,17 @@
       <c r="AN40" s="7"/>
       <c r="AO40" s="7"/>
       <c r="AP40" s="7"/>
-      <c r="AQ40" s="7"/>
-      <c r="AR40" s="66"/>
-      <c r="AS40" s="108"/>
-      <c r="AT40" s="104"/>
-      <c r="AU40" s="104"/>
-      <c r="AV40" s="104"/>
-      <c r="AW40" s="104"/>
-      <c r="AX40" s="104"/>
-      <c r="AY40" s="104"/>
-      <c r="AZ40" s="104"/>
-      <c r="BA40" s="109"/>
+      <c r="AQ40" s="14"/>
+      <c r="AR40" s="65"/>
+      <c r="AS40" s="97"/>
+      <c r="AT40" s="93"/>
+      <c r="AU40" s="93"/>
+      <c r="AV40" s="93"/>
+      <c r="AW40" s="93"/>
+      <c r="AX40" s="93"/>
+      <c r="AY40" s="93"/>
+      <c r="AZ40" s="93"/>
+      <c r="BA40" s="98"/>
       <c r="BB40" s="55"/>
       <c r="BC40" s="14"/>
       <c r="BD40" s="7"/>
@@ -4879,31 +4877,31 @@
       <c r="Z41" s="7"/>
       <c r="AA41" s="14"/>
       <c r="AB41" s="14"/>
-      <c r="AC41" s="77"/>
-      <c r="AD41" s="77"/>
-      <c r="AE41" s="77"/>
-      <c r="AF41" s="77"/>
-      <c r="AG41" s="77"/>
-      <c r="AH41" s="77"/>
+      <c r="AC41" s="76"/>
+      <c r="AD41" s="76"/>
+      <c r="AE41" s="76"/>
+      <c r="AF41" s="76"/>
+      <c r="AG41" s="76"/>
+      <c r="AH41" s="76"/>
       <c r="AI41" s="14"/>
       <c r="AJ41" s="14"/>
       <c r="AK41" s="14"/>
       <c r="AL41" s="14"/>
-      <c r="AM41" s="7"/>
-      <c r="AN41" s="7"/>
+      <c r="AM41" s="14"/>
+      <c r="AN41" s="14"/>
       <c r="AO41" s="7"/>
       <c r="AP41" s="7"/>
-      <c r="AQ41" s="7"/>
-      <c r="AR41" s="66"/>
-      <c r="AS41" s="108"/>
-      <c r="AT41" s="104"/>
-      <c r="AU41" s="104"/>
-      <c r="AV41" s="104"/>
-      <c r="AW41" s="104"/>
-      <c r="AX41" s="104"/>
-      <c r="AY41" s="104"/>
-      <c r="AZ41" s="104"/>
-      <c r="BA41" s="109"/>
+      <c r="AQ41" s="14"/>
+      <c r="AR41" s="65"/>
+      <c r="AS41" s="97"/>
+      <c r="AT41" s="93"/>
+      <c r="AU41" s="93"/>
+      <c r="AV41" s="93"/>
+      <c r="AW41" s="93"/>
+      <c r="AX41" s="93"/>
+      <c r="AY41" s="93"/>
+      <c r="AZ41" s="93"/>
+      <c r="BA41" s="98"/>
       <c r="BB41" s="55"/>
       <c r="BC41" s="14"/>
       <c r="BD41" s="7"/>
@@ -4953,22 +4951,22 @@
       <c r="AI42" s="14"/>
       <c r="AJ42" s="15"/>
       <c r="AK42" s="15"/>
-      <c r="AL42" s="14"/>
-      <c r="AM42" s="14"/>
+      <c r="AL42" s="15"/>
+      <c r="AM42" s="15"/>
       <c r="AN42" s="14"/>
       <c r="AO42" s="7"/>
       <c r="AP42" s="7"/>
-      <c r="AQ42" s="7"/>
-      <c r="AR42" s="66"/>
-      <c r="AS42" s="110"/>
-      <c r="AT42" s="111"/>
-      <c r="AU42" s="111"/>
-      <c r="AV42" s="111"/>
-      <c r="AW42" s="111"/>
-      <c r="AX42" s="111"/>
-      <c r="AY42" s="111"/>
-      <c r="AZ42" s="111"/>
-      <c r="BA42" s="112"/>
+      <c r="AQ42" s="14"/>
+      <c r="AR42" s="65"/>
+      <c r="AS42" s="99"/>
+      <c r="AT42" s="100"/>
+      <c r="AU42" s="100"/>
+      <c r="AV42" s="100"/>
+      <c r="AW42" s="100"/>
+      <c r="AX42" s="100"/>
+      <c r="AY42" s="100"/>
+      <c r="AZ42" s="100"/>
+      <c r="BA42" s="101"/>
       <c r="BB42" s="55"/>
       <c r="BC42" s="14"/>
       <c r="BD42" s="7"/>
@@ -5023,17 +5021,17 @@
       <c r="AN43" s="14"/>
       <c r="AO43" s="15"/>
       <c r="AP43" s="15"/>
-      <c r="AQ43" s="15"/>
+      <c r="AQ43" s="14"/>
       <c r="AR43" s="14"/>
-      <c r="AS43" s="70"/>
-      <c r="AT43" s="70"/>
-      <c r="AU43" s="70"/>
-      <c r="AV43" s="70"/>
-      <c r="AW43" s="70"/>
-      <c r="AX43" s="70"/>
-      <c r="AY43" s="70"/>
-      <c r="AZ43" s="70"/>
-      <c r="BA43" s="70"/>
+      <c r="AS43" s="69"/>
+      <c r="AT43" s="69"/>
+      <c r="AU43" s="69"/>
+      <c r="AV43" s="69"/>
+      <c r="AW43" s="69"/>
+      <c r="AX43" s="69"/>
+      <c r="AY43" s="69"/>
+      <c r="AZ43" s="69"/>
+      <c r="BA43" s="69"/>
       <c r="BB43" s="14"/>
       <c r="BC43" s="14"/>
       <c r="BD43" s="7"/>
@@ -5089,9 +5087,9 @@
       <c r="AO44" s="15"/>
       <c r="AP44" s="15"/>
       <c r="AQ44" s="15"/>
-      <c r="AR44" s="14"/>
+      <c r="AR44" s="15"/>
       <c r="AS44" s="14"/>
-      <c r="AT44" s="7"/>
+      <c r="AT44" s="14"/>
       <c r="AU44" s="7"/>
       <c r="AV44" s="7"/>
       <c r="AW44" s="7"/>
@@ -5154,9 +5152,9 @@
       <c r="AO45" s="15"/>
       <c r="AP45" s="15"/>
       <c r="AQ45" s="15"/>
-      <c r="AR45" s="14"/>
+      <c r="AR45" s="15"/>
       <c r="AS45" s="14"/>
-      <c r="AT45" s="7"/>
+      <c r="AT45" s="14"/>
       <c r="AU45" s="7"/>
       <c r="AV45" s="7"/>
       <c r="AW45" s="7"/>
@@ -5221,7 +5219,7 @@
       <c r="AQ46" s="14"/>
       <c r="AR46" s="14"/>
       <c r="AS46" s="14"/>
-      <c r="AT46" s="15"/>
+      <c r="AT46" s="14"/>
       <c r="AU46" s="15"/>
       <c r="AV46" s="15"/>
       <c r="AW46" s="15"/>
@@ -5286,7 +5284,7 @@
       <c r="AQ47" s="14"/>
       <c r="AR47" s="14"/>
       <c r="AS47" s="14"/>
-      <c r="AT47" s="7"/>
+      <c r="AT47" s="14"/>
       <c r="AU47" s="7"/>
       <c r="AV47" s="7"/>
       <c r="AW47" s="7"/>
@@ -10319,50 +10317,50 @@
       <c r="BI61" s="8"/>
     </row>
     <row r="63" spans="1:61" x14ac:dyDescent="0.25">
-      <c r="A63" s="78" t="s">
+      <c r="A63" s="111" t="s">
         <v>15</v>
       </c>
-      <c r="B63" s="79"/>
-      <c r="C63" s="79"/>
-      <c r="D63" s="79"/>
-      <c r="E63" s="79"/>
-      <c r="F63" s="79"/>
-      <c r="G63" s="79"/>
-      <c r="H63" s="79"/>
-      <c r="I63" s="79"/>
-      <c r="J63" s="79"/>
-      <c r="K63" s="79"/>
-      <c r="L63" s="79"/>
-      <c r="M63" s="79"/>
-      <c r="N63" s="79"/>
-      <c r="O63" s="79"/>
-      <c r="P63" s="79"/>
-      <c r="Q63" s="79"/>
-      <c r="R63" s="79"/>
-      <c r="S63" s="79"/>
-      <c r="T63" s="79"/>
+      <c r="B63" s="109"/>
+      <c r="C63" s="109"/>
+      <c r="D63" s="109"/>
+      <c r="E63" s="109"/>
+      <c r="F63" s="109"/>
+      <c r="G63" s="109"/>
+      <c r="H63" s="109"/>
+      <c r="I63" s="109"/>
+      <c r="J63" s="109"/>
+      <c r="K63" s="109"/>
+      <c r="L63" s="109"/>
+      <c r="M63" s="109"/>
+      <c r="N63" s="109"/>
+      <c r="O63" s="109"/>
+      <c r="P63" s="109"/>
+      <c r="Q63" s="109"/>
+      <c r="R63" s="109"/>
+      <c r="S63" s="109"/>
+      <c r="T63" s="109"/>
     </row>
     <row r="64" spans="1:61" ht="81.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A64" s="79"/>
-      <c r="B64" s="79"/>
-      <c r="C64" s="79"/>
-      <c r="D64" s="79"/>
-      <c r="E64" s="79"/>
-      <c r="F64" s="79"/>
-      <c r="G64" s="79"/>
-      <c r="H64" s="79"/>
-      <c r="I64" s="79"/>
-      <c r="J64" s="79"/>
-      <c r="K64" s="79"/>
-      <c r="L64" s="79"/>
-      <c r="M64" s="79"/>
-      <c r="N64" s="79"/>
-      <c r="O64" s="79"/>
-      <c r="P64" s="79"/>
-      <c r="Q64" s="79"/>
-      <c r="R64" s="79"/>
-      <c r="S64" s="79"/>
-      <c r="T64" s="79"/>
+      <c r="A64" s="109"/>
+      <c r="B64" s="109"/>
+      <c r="C64" s="109"/>
+      <c r="D64" s="109"/>
+      <c r="E64" s="109"/>
+      <c r="F64" s="109"/>
+      <c r="G64" s="109"/>
+      <c r="H64" s="109"/>
+      <c r="I64" s="109"/>
+      <c r="J64" s="109"/>
+      <c r="K64" s="109"/>
+      <c r="L64" s="109"/>
+      <c r="M64" s="109"/>
+      <c r="N64" s="109"/>
+      <c r="O64" s="109"/>
+      <c r="P64" s="109"/>
+      <c r="Q64" s="109"/>
+      <c r="R64" s="109"/>
+      <c r="S64" s="109"/>
+      <c r="T64" s="109"/>
     </row>
     <row r="66" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B66" s="9"/>
@@ -10397,26 +10395,26 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:4" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="A1" s="80" t="s">
+      <c r="A1" s="108" t="s">
         <v>16</v>
       </c>
-      <c r="B1" s="79"/>
-      <c r="C1" s="79"/>
-      <c r="D1" s="79"/>
+      <c r="B1" s="109"/>
+      <c r="C1" s="109"/>
+      <c r="D1" s="109"/>
     </row>
     <row r="3" spans="1:4" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="86" t="s">
+      <c r="A3" s="115" t="s">
         <v>17</v>
       </c>
-      <c r="B3" s="79"/>
-      <c r="C3" s="79"/>
-      <c r="D3" s="79"/>
+      <c r="B3" s="109"/>
+      <c r="C3" s="109"/>
+      <c r="D3" s="109"/>
     </row>
     <row r="4" spans="1:4" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="79"/>
-      <c r="B4" s="79"/>
-      <c r="C4" s="79"/>
-      <c r="D4" s="79"/>
+      <c r="A4" s="109"/>
+      <c r="B4" s="109"/>
+      <c r="C4" s="109"/>
+      <c r="D4" s="109"/>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A6" s="1" t="s">
@@ -10433,12 +10431,12 @@
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A7" s="85" t="s">
+      <c r="A7" s="114" t="s">
         <v>22</v>
       </c>
-      <c r="B7" s="79"/>
-      <c r="C7" s="79"/>
-      <c r="D7" s="79"/>
+      <c r="B7" s="109"/>
+      <c r="C7" s="109"/>
+      <c r="D7" s="109"/>
     </row>
     <row r="8" spans="1:4" ht="24" x14ac:dyDescent="0.25">
       <c r="A8" s="12"/>
@@ -10501,20 +10499,20 @@
       </c>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A13" s="83" t="s">
+      <c r="A13" s="116" t="s">
         <v>34</v>
       </c>
-      <c r="B13" s="79"/>
-      <c r="C13" s="79"/>
-      <c r="D13" s="79"/>
+      <c r="B13" s="109"/>
+      <c r="C13" s="109"/>
+      <c r="D13" s="109"/>
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A15" s="85" t="s">
+      <c r="A15" s="114" t="s">
         <v>35</v>
       </c>
-      <c r="B15" s="79"/>
-      <c r="C15" s="79"/>
-      <c r="D15" s="79"/>
+      <c r="B15" s="109"/>
+      <c r="C15" s="109"/>
+      <c r="D15" s="109"/>
     </row>
     <row r="16" spans="1:4" ht="24" x14ac:dyDescent="0.25">
       <c r="A16" s="17"/>
@@ -10589,335 +10587,366 @@
       </c>
     </row>
     <row r="22" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A22" s="83" t="s">
+      <c r="A22" s="116" t="s">
         <v>49</v>
       </c>
-      <c r="B22" s="79"/>
-      <c r="C22" s="79"/>
-      <c r="D22" s="79"/>
+      <c r="B22" s="109"/>
+      <c r="C22" s="109"/>
+      <c r="D22" s="109"/>
     </row>
     <row r="26" spans="1:4" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A26" s="84" t="s">
+      <c r="A26" s="113" t="s">
         <v>50</v>
       </c>
-      <c r="B26" s="79"/>
-      <c r="C26" s="79"/>
-      <c r="D26" s="79"/>
+      <c r="B26" s="109"/>
+      <c r="C26" s="109"/>
+      <c r="D26" s="109"/>
     </row>
     <row r="27" spans="1:4" ht="31.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A27" s="82" t="s">
+      <c r="A27" s="112" t="s">
         <v>51</v>
       </c>
-      <c r="B27" s="79"/>
-      <c r="C27" s="79"/>
-      <c r="D27" s="79"/>
+      <c r="B27" s="109"/>
+      <c r="C27" s="109"/>
+      <c r="D27" s="109"/>
     </row>
     <row r="28" spans="1:4" ht="30.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A28" s="82" t="s">
+      <c r="A28" s="112" t="s">
         <v>52</v>
       </c>
-      <c r="B28" s="79"/>
-      <c r="C28" s="79"/>
-      <c r="D28" s="79"/>
+      <c r="B28" s="109"/>
+      <c r="C28" s="109"/>
+      <c r="D28" s="109"/>
     </row>
     <row r="29" spans="1:4" ht="32.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A29" s="82" t="s">
+      <c r="A29" s="112" t="s">
         <v>53</v>
       </c>
-      <c r="B29" s="79"/>
-      <c r="C29" s="79"/>
-      <c r="D29" s="79"/>
+      <c r="B29" s="109"/>
+      <c r="C29" s="109"/>
+      <c r="D29" s="109"/>
     </row>
     <row r="30" spans="1:4" ht="34.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A30" s="82" t="s">
+      <c r="A30" s="112" t="s">
         <v>54</v>
       </c>
-      <c r="B30" s="79"/>
-      <c r="C30" s="79"/>
-      <c r="D30" s="79"/>
+      <c r="B30" s="109"/>
+      <c r="C30" s="109"/>
+      <c r="D30" s="109"/>
     </row>
     <row r="31" spans="1:4" ht="29.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A31" s="82" t="s">
+      <c r="A31" s="112" t="s">
         <v>55</v>
       </c>
-      <c r="B31" s="79"/>
-      <c r="C31" s="79"/>
-      <c r="D31" s="79"/>
+      <c r="B31" s="109"/>
+      <c r="C31" s="109"/>
+      <c r="D31" s="109"/>
     </row>
     <row r="32" spans="1:4" ht="35.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A32" s="82" t="s">
+      <c r="A32" s="112" t="s">
         <v>56</v>
       </c>
-      <c r="B32" s="79"/>
-      <c r="C32" s="79"/>
-      <c r="D32" s="79"/>
+      <c r="B32" s="109"/>
+      <c r="C32" s="109"/>
+      <c r="D32" s="109"/>
     </row>
     <row r="33" spans="1:4" ht="30.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A33" s="82" t="s">
+      <c r="A33" s="112" t="s">
         <v>57</v>
       </c>
-      <c r="B33" s="79"/>
-      <c r="C33" s="79"/>
-      <c r="D33" s="79"/>
+      <c r="B33" s="109"/>
+      <c r="C33" s="109"/>
+      <c r="D33" s="109"/>
     </row>
     <row r="34" spans="1:4" ht="30.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A34" s="82" t="s">
+      <c r="A34" s="112" t="s">
         <v>58</v>
       </c>
-      <c r="B34" s="79"/>
-      <c r="C34" s="79"/>
-      <c r="D34" s="79"/>
+      <c r="B34" s="109"/>
+      <c r="C34" s="109"/>
+      <c r="D34" s="109"/>
     </row>
     <row r="35" spans="1:4" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A35" s="82" t="s">
+      <c r="A35" s="112" t="s">
         <v>59</v>
       </c>
-      <c r="B35" s="79"/>
-      <c r="C35" s="79"/>
-      <c r="D35" s="79"/>
+      <c r="B35" s="109"/>
+      <c r="C35" s="109"/>
+      <c r="D35" s="109"/>
     </row>
     <row r="36" spans="1:4" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A36" s="82"/>
-      <c r="B36" s="79"/>
-      <c r="C36" s="79"/>
-      <c r="D36" s="79"/>
+      <c r="A36" s="112"/>
+      <c r="B36" s="109"/>
+      <c r="C36" s="109"/>
+      <c r="D36" s="109"/>
     </row>
     <row r="37" spans="1:4" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A37" s="84" t="s">
+      <c r="A37" s="113" t="s">
         <v>60</v>
       </c>
-      <c r="B37" s="79"/>
-      <c r="C37" s="79"/>
-      <c r="D37" s="79"/>
+      <c r="B37" s="109"/>
+      <c r="C37" s="109"/>
+      <c r="D37" s="109"/>
     </row>
     <row r="38" spans="1:4" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A38" s="82" t="s">
+      <c r="A38" s="112" t="s">
         <v>61</v>
       </c>
-      <c r="B38" s="79"/>
-      <c r="C38" s="79"/>
-      <c r="D38" s="79"/>
+      <c r="B38" s="109"/>
+      <c r="C38" s="109"/>
+      <c r="D38" s="109"/>
     </row>
     <row r="39" spans="1:4" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A39" s="82" t="s">
+      <c r="A39" s="112" t="s">
         <v>62</v>
       </c>
-      <c r="B39" s="79"/>
-      <c r="C39" s="79"/>
-      <c r="D39" s="79"/>
+      <c r="B39" s="109"/>
+      <c r="C39" s="109"/>
+      <c r="D39" s="109"/>
     </row>
     <row r="40" spans="1:4" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A40" s="82" t="s">
+      <c r="A40" s="112" t="s">
         <v>63</v>
       </c>
-      <c r="B40" s="79"/>
-      <c r="C40" s="79"/>
-      <c r="D40" s="79"/>
+      <c r="B40" s="109"/>
+      <c r="C40" s="109"/>
+      <c r="D40" s="109"/>
     </row>
     <row r="41" spans="1:4" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A41" s="82" t="s">
+      <c r="A41" s="112" t="s">
         <v>64</v>
       </c>
-      <c r="B41" s="79"/>
-      <c r="C41" s="79"/>
-      <c r="D41" s="79"/>
+      <c r="B41" s="109"/>
+      <c r="C41" s="109"/>
+      <c r="D41" s="109"/>
     </row>
     <row r="42" spans="1:4" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A42" s="82" t="s">
+      <c r="A42" s="112" t="s">
         <v>65</v>
       </c>
-      <c r="B42" s="79"/>
-      <c r="C42" s="79"/>
-      <c r="D42" s="79"/>
+      <c r="B42" s="109"/>
+      <c r="C42" s="109"/>
+      <c r="D42" s="109"/>
     </row>
     <row r="43" spans="1:4" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A43" s="82" t="s">
+      <c r="A43" s="112" t="s">
         <v>66</v>
       </c>
-      <c r="B43" s="79"/>
-      <c r="C43" s="79"/>
-      <c r="D43" s="79"/>
+      <c r="B43" s="109"/>
+      <c r="C43" s="109"/>
+      <c r="D43" s="109"/>
     </row>
     <row r="44" spans="1:4" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A44" s="82"/>
-      <c r="B44" s="79"/>
-      <c r="C44" s="79"/>
-      <c r="D44" s="79"/>
+      <c r="A44" s="112"/>
+      <c r="B44" s="109"/>
+      <c r="C44" s="109"/>
+      <c r="D44" s="109"/>
     </row>
     <row r="45" spans="1:4" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A45" s="84" t="s">
+      <c r="A45" s="113" t="s">
         <v>67</v>
       </c>
-      <c r="B45" s="79"/>
-      <c r="C45" s="79"/>
-      <c r="D45" s="79"/>
+      <c r="B45" s="109"/>
+      <c r="C45" s="109"/>
+      <c r="D45" s="109"/>
     </row>
     <row r="46" spans="1:4" ht="37.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A46" s="82" t="s">
+      <c r="A46" s="112" t="s">
         <v>68</v>
       </c>
-      <c r="B46" s="79"/>
-      <c r="C46" s="79"/>
-      <c r="D46" s="79"/>
+      <c r="B46" s="109"/>
+      <c r="C46" s="109"/>
+      <c r="D46" s="109"/>
     </row>
     <row r="47" spans="1:4" ht="30.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A47" s="82" t="s">
+      <c r="A47" s="112" t="s">
         <v>69</v>
       </c>
-      <c r="B47" s="79"/>
-      <c r="C47" s="79"/>
-      <c r="D47" s="79"/>
+      <c r="B47" s="109"/>
+      <c r="C47" s="109"/>
+      <c r="D47" s="109"/>
     </row>
     <row r="48" spans="1:4" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A48" s="82" t="s">
+      <c r="A48" s="112" t="s">
         <v>70</v>
       </c>
-      <c r="B48" s="79"/>
-      <c r="C48" s="79"/>
-      <c r="D48" s="79"/>
+      <c r="B48" s="109"/>
+      <c r="C48" s="109"/>
+      <c r="D48" s="109"/>
     </row>
     <row r="49" spans="1:4" ht="48" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A49" s="82" t="s">
+      <c r="A49" s="112" t="s">
         <v>71</v>
       </c>
-      <c r="B49" s="79"/>
-      <c r="C49" s="79"/>
-      <c r="D49" s="79"/>
+      <c r="B49" s="109"/>
+      <c r="C49" s="109"/>
+      <c r="D49" s="109"/>
     </row>
     <row r="50" spans="1:4" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A50" s="82"/>
-      <c r="B50" s="79"/>
-      <c r="C50" s="79"/>
-      <c r="D50" s="79"/>
+      <c r="A50" s="112"/>
+      <c r="B50" s="109"/>
+      <c r="C50" s="109"/>
+      <c r="D50" s="109"/>
     </row>
     <row r="51" spans="1:4" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A51" s="84" t="s">
+      <c r="A51" s="113" t="s">
         <v>72</v>
       </c>
-      <c r="B51" s="79"/>
-      <c r="C51" s="79"/>
-      <c r="D51" s="79"/>
+      <c r="B51" s="109"/>
+      <c r="C51" s="109"/>
+      <c r="D51" s="109"/>
     </row>
     <row r="52" spans="1:4" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A52" s="82" t="s">
+      <c r="A52" s="112" t="s">
         <v>73</v>
       </c>
-      <c r="B52" s="79"/>
-      <c r="C52" s="79"/>
-      <c r="D52" s="79"/>
+      <c r="B52" s="109"/>
+      <c r="C52" s="109"/>
+      <c r="D52" s="109"/>
     </row>
     <row r="53" spans="1:4" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A53" s="82" t="s">
+      <c r="A53" s="112" t="s">
         <v>74</v>
       </c>
-      <c r="B53" s="79"/>
-      <c r="C53" s="79"/>
-      <c r="D53" s="79"/>
+      <c r="B53" s="109"/>
+      <c r="C53" s="109"/>
+      <c r="D53" s="109"/>
     </row>
     <row r="54" spans="1:4" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A54" s="82" t="s">
+      <c r="A54" s="112" t="s">
         <v>75</v>
       </c>
-      <c r="B54" s="79"/>
-      <c r="C54" s="79"/>
-      <c r="D54" s="79"/>
+      <c r="B54" s="109"/>
+      <c r="C54" s="109"/>
+      <c r="D54" s="109"/>
     </row>
     <row r="55" spans="1:4" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A55" s="82" t="s">
+      <c r="A55" s="112" t="s">
         <v>76</v>
       </c>
-      <c r="B55" s="79"/>
-      <c r="C55" s="79"/>
-      <c r="D55" s="79"/>
+      <c r="B55" s="109"/>
+      <c r="C55" s="109"/>
+      <c r="D55" s="109"/>
     </row>
     <row r="56" spans="1:4" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A56" s="82" t="s">
+      <c r="A56" s="112" t="s">
         <v>77</v>
       </c>
-      <c r="B56" s="79"/>
-      <c r="C56" s="79"/>
-      <c r="D56" s="79"/>
+      <c r="B56" s="109"/>
+      <c r="C56" s="109"/>
+      <c r="D56" s="109"/>
     </row>
     <row r="57" spans="1:4" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A57" s="82" t="s">
+      <c r="A57" s="112" t="s">
         <v>78</v>
       </c>
-      <c r="B57" s="79"/>
-      <c r="C57" s="79"/>
-      <c r="D57" s="79"/>
+      <c r="B57" s="109"/>
+      <c r="C57" s="109"/>
+      <c r="D57" s="109"/>
     </row>
     <row r="58" spans="1:4" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A58" s="82" t="s">
+      <c r="A58" s="112" t="s">
         <v>79</v>
       </c>
-      <c r="B58" s="79"/>
-      <c r="C58" s="79"/>
-      <c r="D58" s="79"/>
+      <c r="B58" s="109"/>
+      <c r="C58" s="109"/>
+      <c r="D58" s="109"/>
     </row>
     <row r="59" spans="1:4" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A59" s="82"/>
-      <c r="B59" s="79"/>
-      <c r="C59" s="79"/>
-      <c r="D59" s="79"/>
+      <c r="A59" s="112"/>
+      <c r="B59" s="109"/>
+      <c r="C59" s="109"/>
+      <c r="D59" s="109"/>
     </row>
     <row r="60" spans="1:4" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A60" s="84" t="s">
+      <c r="A60" s="113" t="s">
         <v>80</v>
       </c>
-      <c r="B60" s="79"/>
-      <c r="C60" s="79"/>
-      <c r="D60" s="79"/>
+      <c r="B60" s="109"/>
+      <c r="C60" s="109"/>
+      <c r="D60" s="109"/>
     </row>
     <row r="61" spans="1:4" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A61" s="82" t="s">
+      <c r="A61" s="112" t="s">
         <v>81</v>
       </c>
-      <c r="B61" s="79"/>
-      <c r="C61" s="79"/>
-      <c r="D61" s="79"/>
+      <c r="B61" s="109"/>
+      <c r="C61" s="109"/>
+      <c r="D61" s="109"/>
     </row>
     <row r="62" spans="1:4" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A62" s="82" t="s">
+      <c r="A62" s="112" t="s">
         <v>82</v>
       </c>
-      <c r="B62" s="79"/>
-      <c r="C62" s="79"/>
-      <c r="D62" s="79"/>
+      <c r="B62" s="109"/>
+      <c r="C62" s="109"/>
+      <c r="D62" s="109"/>
     </row>
     <row r="63" spans="1:4" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A63" s="82" t="s">
+      <c r="A63" s="112" t="s">
         <v>83</v>
       </c>
-      <c r="B63" s="79"/>
-      <c r="C63" s="79"/>
-      <c r="D63" s="79"/>
+      <c r="B63" s="109"/>
+      <c r="C63" s="109"/>
+      <c r="D63" s="109"/>
     </row>
     <row r="64" spans="1:4" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A64" s="82" t="s">
+      <c r="A64" s="112" t="s">
         <v>84</v>
       </c>
-      <c r="B64" s="79"/>
-      <c r="C64" s="79"/>
-      <c r="D64" s="79"/>
+      <c r="B64" s="109"/>
+      <c r="C64" s="109"/>
+      <c r="D64" s="109"/>
     </row>
     <row r="65" spans="1:4" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A65" s="82" t="s">
+      <c r="A65" s="112" t="s">
         <v>85</v>
       </c>
-      <c r="B65" s="79"/>
-      <c r="C65" s="79"/>
-      <c r="D65" s="79"/>
+      <c r="B65" s="109"/>
+      <c r="C65" s="109"/>
+      <c r="D65" s="109"/>
     </row>
     <row r="66" spans="1:4" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A66" s="82" t="s">
+      <c r="A66" s="112" t="s">
         <v>86</v>
       </c>
-      <c r="B66" s="79"/>
-      <c r="C66" s="79"/>
-      <c r="D66" s="79"/>
+      <c r="B66" s="109"/>
+      <c r="C66" s="109"/>
+      <c r="D66" s="109"/>
     </row>
   </sheetData>
   <mergeCells count="47">
+    <mergeCell ref="A62:D62"/>
+    <mergeCell ref="A38:D38"/>
+    <mergeCell ref="A29:D29"/>
+    <mergeCell ref="A52:D52"/>
+    <mergeCell ref="A43:D43"/>
+    <mergeCell ref="A28:D28"/>
+    <mergeCell ref="A13:D13"/>
+    <mergeCell ref="A44:D44"/>
+    <mergeCell ref="A40:D40"/>
+    <mergeCell ref="A31:D31"/>
+    <mergeCell ref="A34:D34"/>
+    <mergeCell ref="A30:D30"/>
+    <mergeCell ref="A39:D39"/>
+    <mergeCell ref="A22:D22"/>
+    <mergeCell ref="A35:D35"/>
+    <mergeCell ref="A1:D1"/>
+    <mergeCell ref="A45:D45"/>
+    <mergeCell ref="A61:D61"/>
+    <mergeCell ref="A54:D54"/>
+    <mergeCell ref="A7:D7"/>
+    <mergeCell ref="A27:D27"/>
+    <mergeCell ref="A26:D26"/>
+    <mergeCell ref="A33:D33"/>
+    <mergeCell ref="A32:D32"/>
+    <mergeCell ref="A3:D4"/>
+    <mergeCell ref="A15:D15"/>
+    <mergeCell ref="A59:D59"/>
+    <mergeCell ref="A49:D49"/>
+    <mergeCell ref="A51:D51"/>
+    <mergeCell ref="A60:D60"/>
+    <mergeCell ref="A36:D36"/>
     <mergeCell ref="A65:D65"/>
     <mergeCell ref="A41:D41"/>
     <mergeCell ref="A46:D46"/>
@@ -10934,37 +10963,6 @@
     <mergeCell ref="A58:D58"/>
     <mergeCell ref="A48:D48"/>
     <mergeCell ref="A53:D53"/>
-    <mergeCell ref="A1:D1"/>
-    <mergeCell ref="A45:D45"/>
-    <mergeCell ref="A61:D61"/>
-    <mergeCell ref="A54:D54"/>
-    <mergeCell ref="A7:D7"/>
-    <mergeCell ref="A27:D27"/>
-    <mergeCell ref="A26:D26"/>
-    <mergeCell ref="A33:D33"/>
-    <mergeCell ref="A32:D32"/>
-    <mergeCell ref="A3:D4"/>
-    <mergeCell ref="A15:D15"/>
-    <mergeCell ref="A59:D59"/>
-    <mergeCell ref="A49:D49"/>
-    <mergeCell ref="A51:D51"/>
-    <mergeCell ref="A60:D60"/>
-    <mergeCell ref="A36:D36"/>
-    <mergeCell ref="A28:D28"/>
-    <mergeCell ref="A13:D13"/>
-    <mergeCell ref="A44:D44"/>
-    <mergeCell ref="A40:D40"/>
-    <mergeCell ref="A31:D31"/>
-    <mergeCell ref="A34:D34"/>
-    <mergeCell ref="A30:D30"/>
-    <mergeCell ref="A39:D39"/>
-    <mergeCell ref="A22:D22"/>
-    <mergeCell ref="A35:D35"/>
-    <mergeCell ref="A62:D62"/>
-    <mergeCell ref="A38:D38"/>
-    <mergeCell ref="A29:D29"/>
-    <mergeCell ref="A52:D52"/>
-    <mergeCell ref="A43:D43"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -11530,42 +11528,42 @@
       <c r="J39" s="29"/>
     </row>
     <row r="41" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A41" s="78" t="s">
+      <c r="A41" s="111" t="s">
         <v>117</v>
       </c>
-      <c r="B41" s="79"/>
-      <c r="C41" s="79"/>
-      <c r="D41" s="79"/>
-      <c r="E41" s="79"/>
-      <c r="F41" s="79"/>
-      <c r="G41" s="79"/>
-      <c r="H41" s="79"/>
-      <c r="I41" s="79"/>
-      <c r="J41" s="79"/>
+      <c r="B41" s="109"/>
+      <c r="C41" s="109"/>
+      <c r="D41" s="109"/>
+      <c r="E41" s="109"/>
+      <c r="F41" s="109"/>
+      <c r="G41" s="109"/>
+      <c r="H41" s="109"/>
+      <c r="I41" s="109"/>
+      <c r="J41" s="109"/>
     </row>
     <row r="42" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A42" s="79"/>
-      <c r="B42" s="79"/>
-      <c r="C42" s="79"/>
-      <c r="D42" s="79"/>
-      <c r="E42" s="79"/>
-      <c r="F42" s="79"/>
-      <c r="G42" s="79"/>
-      <c r="H42" s="79"/>
-      <c r="I42" s="79"/>
-      <c r="J42" s="79"/>
+      <c r="A42" s="109"/>
+      <c r="B42" s="109"/>
+      <c r="C42" s="109"/>
+      <c r="D42" s="109"/>
+      <c r="E42" s="109"/>
+      <c r="F42" s="109"/>
+      <c r="G42" s="109"/>
+      <c r="H42" s="109"/>
+      <c r="I42" s="109"/>
+      <c r="J42" s="109"/>
     </row>
     <row r="43" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A43" s="79"/>
-      <c r="B43" s="79"/>
-      <c r="C43" s="79"/>
-      <c r="D43" s="79"/>
-      <c r="E43" s="79"/>
-      <c r="F43" s="79"/>
-      <c r="G43" s="79"/>
-      <c r="H43" s="79"/>
-      <c r="I43" s="79"/>
-      <c r="J43" s="79"/>
+      <c r="A43" s="109"/>
+      <c r="B43" s="109"/>
+      <c r="C43" s="109"/>
+      <c r="D43" s="109"/>
+      <c r="E43" s="109"/>
+      <c r="F43" s="109"/>
+      <c r="G43" s="109"/>
+      <c r="H43" s="109"/>
+      <c r="I43" s="109"/>
+      <c r="J43" s="109"/>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -11861,24 +11859,24 @@
       <c r="G24" s="29"/>
     </row>
     <row r="26" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A26" s="78" t="s">
+      <c r="A26" s="111" t="s">
         <v>134</v>
       </c>
-      <c r="B26" s="79"/>
-      <c r="C26" s="79"/>
-      <c r="D26" s="79"/>
-      <c r="E26" s="79"/>
-      <c r="F26" s="79"/>
-      <c r="G26" s="79"/>
+      <c r="B26" s="109"/>
+      <c r="C26" s="109"/>
+      <c r="D26" s="109"/>
+      <c r="E26" s="109"/>
+      <c r="F26" s="109"/>
+      <c r="G26" s="109"/>
     </row>
     <row r="27" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A27" s="79"/>
-      <c r="B27" s="79"/>
-      <c r="C27" s="79"/>
-      <c r="D27" s="79"/>
-      <c r="E27" s="79"/>
-      <c r="F27" s="79"/>
-      <c r="G27" s="79"/>
+      <c r="A27" s="109"/>
+      <c r="B27" s="109"/>
+      <c r="C27" s="109"/>
+      <c r="D27" s="109"/>
+      <c r="E27" s="109"/>
+      <c r="F27" s="109"/>
+      <c r="G27" s="109"/>
     </row>
   </sheetData>
   <mergeCells count="1">

</xml_diff>

<commit_message>
content(holomap): mise à jour du gabarit de carte (playtest)
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Carte Holo/carte_holomap.xlsx
+++ b/Carte Holo/carte_holomap.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\b.consol\Downloads\Divers\ecole\Dossier UE9\IdleEvolution\Carte Holo\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Projets\IdleEvolution\Carte Holo\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A490C6AE-CB9D-4551-93D1-A8FC7137F959}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{307B4E37-B03E-450A-B9B5-1E97B2D9C16B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Paramètres" sheetId="1" r:id="rId1"/>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="190" uniqueCount="162">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="191" uniqueCount="163">
   <si>
     <t>Paramètres globaux — HoloMap</t>
   </si>
@@ -493,9 +493,6 @@
     <t>10d</t>
   </si>
   <si>
-    <t>12p</t>
-  </si>
-  <si>
     <t>12g</t>
   </si>
   <si>
@@ -524,6 +521,12 @@
   </si>
   <si>
     <t>biome_montagne</t>
+  </si>
+  <si>
+    <t>2p</t>
+  </si>
+  <si>
+    <t>24g</t>
   </si>
 </sst>
 </file>
@@ -712,7 +715,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="105">
+  <borders count="109">
     <border>
       <left/>
       <right/>
@@ -1954,11 +1957,55 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="FFD0D0D0"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color rgb="FFD0D0D0"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color theme="1" tint="0.499984740745262"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom style="medium">
+        <color theme="1" tint="0.499984740745262"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="FF9AA0A6"/>
+      </right>
+      <top/>
+      <bottom style="medium">
+        <color theme="1" tint="0.499984740745262"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color theme="1" tint="0.499984740745262"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF9AA0A6"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="173">
+  <cellXfs count="174">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -2087,29 +2134,10 @@
     <xf numFmtId="0" fontId="0" fillId="13" borderId="54" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="13" borderId="55" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="13" borderId="34" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="15" borderId="0" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="20" borderId="0" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="14" borderId="0" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="12" borderId="0" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="13" borderId="0" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="8" borderId="0" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="15" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="20" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="14" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="12" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="13" borderId="57" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="13" borderId="58" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="13" borderId="59" xfId="0" applyFill="1" applyBorder="1"/>
@@ -2150,7 +2178,6 @@
     <xf numFmtId="0" fontId="0" fillId="15" borderId="94" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="15" borderId="95" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="15" borderId="96" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="14" borderId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="0" fillId="8" borderId="97" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="8" borderId="98" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="8" borderId="99" xfId="0" applyFill="1" applyBorder="1"/>
@@ -2159,7 +2186,28 @@
     <xf numFmtId="0" fontId="0" fillId="8" borderId="102" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="8" borderId="103" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="8" borderId="104" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="14" borderId="76" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="105" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="0" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="106" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="107" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="108" xfId="0" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -2482,11 +2530,11 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="A1" s="108" t="s">
+      <c r="A1" s="164" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="109"/>
-      <c r="C1" s="109"/>
+      <c r="B1" s="161"/>
+      <c r="C1" s="161"/>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
@@ -2544,11 +2592,11 @@
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A9" s="110" t="s">
+      <c r="A9" s="167" t="s">
         <v>13</v>
       </c>
-      <c r="B9" s="109"/>
-      <c r="C9" s="109"/>
+      <c r="B9" s="161"/>
+      <c r="C9" s="161"/>
     </row>
   </sheetData>
   <mergeCells count="2">
@@ -3349,12 +3397,12 @@
       <c r="E11" s="7"/>
       <c r="F11" s="7"/>
       <c r="G11" s="37"/>
-      <c r="H11" s="139"/>
-      <c r="I11" s="140"/>
-      <c r="J11" s="140"/>
-      <c r="K11" s="140"/>
-      <c r="L11" s="140"/>
-      <c r="M11" s="141"/>
+      <c r="H11" s="128"/>
+      <c r="I11" s="129"/>
+      <c r="J11" s="129"/>
+      <c r="K11" s="129"/>
+      <c r="L11" s="129"/>
+      <c r="M11" s="130"/>
       <c r="N11" s="41"/>
       <c r="O11" s="7"/>
       <c r="P11" s="7"/>
@@ -3414,12 +3462,12 @@
       <c r="E12" s="7"/>
       <c r="F12" s="7"/>
       <c r="G12" s="37"/>
-      <c r="H12" s="142"/>
-      <c r="I12" s="119"/>
-      <c r="J12" s="119"/>
-      <c r="K12" s="119"/>
-      <c r="L12" s="119"/>
-      <c r="M12" s="143"/>
+      <c r="H12" s="131"/>
+      <c r="I12" s="110"/>
+      <c r="J12" s="110"/>
+      <c r="K12" s="110"/>
+      <c r="L12" s="110"/>
+      <c r="M12" s="132"/>
       <c r="N12" s="41"/>
       <c r="O12" s="7"/>
       <c r="P12" s="7"/>
@@ -3455,13 +3503,13 @@
       <c r="AT12" s="7"/>
       <c r="AU12" s="7"/>
       <c r="AV12" s="37"/>
-      <c r="AW12" s="131"/>
-      <c r="AX12" s="132"/>
-      <c r="AY12" s="132"/>
-      <c r="AZ12" s="132"/>
-      <c r="BA12" s="132"/>
-      <c r="BB12" s="132"/>
-      <c r="BC12" s="133"/>
+      <c r="AW12" s="120"/>
+      <c r="AX12" s="121"/>
+      <c r="AY12" s="121"/>
+      <c r="AZ12" s="121"/>
+      <c r="BA12" s="121"/>
+      <c r="BB12" s="121"/>
+      <c r="BC12" s="122"/>
       <c r="BD12" s="41"/>
       <c r="BE12" s="7"/>
       <c r="BF12" s="22"/>
@@ -3479,14 +3527,14 @@
       <c r="E13" s="7"/>
       <c r="F13" s="7"/>
       <c r="G13" s="37"/>
-      <c r="H13" s="172"/>
-      <c r="I13" s="163" t="s">
-        <v>161</v>
-      </c>
-      <c r="J13" s="163"/>
-      <c r="K13" s="119"/>
-      <c r="L13" s="119"/>
-      <c r="M13" s="143"/>
+      <c r="H13" s="131"/>
+      <c r="I13" s="110" t="s">
+        <v>160</v>
+      </c>
+      <c r="J13" s="110"/>
+      <c r="K13" s="110"/>
+      <c r="L13" s="110"/>
+      <c r="M13" s="132"/>
       <c r="N13" s="41"/>
       <c r="O13" s="7"/>
       <c r="P13" s="7"/>
@@ -3522,13 +3570,13 @@
       <c r="AT13" s="7"/>
       <c r="AU13" s="7"/>
       <c r="AV13" s="37"/>
-      <c r="AW13" s="134"/>
-      <c r="AX13" s="120"/>
-      <c r="AY13" s="120"/>
-      <c r="AZ13" s="120"/>
-      <c r="BA13" s="120"/>
-      <c r="BB13" s="120"/>
-      <c r="BC13" s="135"/>
+      <c r="AW13" s="123"/>
+      <c r="AX13" s="111"/>
+      <c r="AY13" s="111"/>
+      <c r="AZ13" s="111"/>
+      <c r="BA13" s="111"/>
+      <c r="BB13" s="111"/>
+      <c r="BC13" s="124"/>
       <c r="BD13" s="41"/>
       <c r="BE13" s="7"/>
       <c r="BF13" s="22"/>
@@ -3546,12 +3594,12 @@
       <c r="E14" s="7"/>
       <c r="F14" s="7"/>
       <c r="G14" s="37"/>
-      <c r="H14" s="142"/>
-      <c r="I14" s="119"/>
-      <c r="J14" s="119"/>
-      <c r="K14" s="119"/>
-      <c r="L14" s="119"/>
-      <c r="M14" s="143"/>
+      <c r="H14" s="131"/>
+      <c r="I14" s="110"/>
+      <c r="J14" s="110"/>
+      <c r="K14" s="110"/>
+      <c r="L14" s="110"/>
+      <c r="M14" s="132"/>
       <c r="N14" s="99"/>
       <c r="O14" s="49"/>
       <c r="P14" s="49"/>
@@ -3587,13 +3635,13 @@
       <c r="AT14" s="7"/>
       <c r="AU14" s="7"/>
       <c r="AV14" s="37"/>
-      <c r="AW14" s="134"/>
-      <c r="AX14" s="120"/>
-      <c r="AY14" s="120"/>
-      <c r="AZ14" s="120"/>
-      <c r="BA14" s="120"/>
-      <c r="BB14" s="120"/>
-      <c r="BC14" s="135"/>
+      <c r="AW14" s="123"/>
+      <c r="AX14" s="111"/>
+      <c r="AY14" s="111"/>
+      <c r="AZ14" s="111"/>
+      <c r="BA14" s="111"/>
+      <c r="BB14" s="111"/>
+      <c r="BC14" s="124"/>
       <c r="BD14" s="41"/>
       <c r="BE14" s="7"/>
       <c r="BF14" s="22"/>
@@ -3601,7 +3649,7 @@
       <c r="BH14" s="22"/>
       <c r="BI14" s="22"/>
     </row>
-    <row r="15" spans="1:61" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:61" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A15" s="6">
         <v>14</v>
       </c>
@@ -3611,12 +3659,12 @@
       <c r="E15" s="7"/>
       <c r="F15" s="7"/>
       <c r="G15" s="37"/>
-      <c r="H15" s="142"/>
-      <c r="I15" s="119"/>
-      <c r="J15" s="119"/>
-      <c r="K15" s="119"/>
-      <c r="L15" s="119"/>
-      <c r="M15" s="143"/>
+      <c r="H15" s="131"/>
+      <c r="I15" s="110"/>
+      <c r="J15" s="110"/>
+      <c r="K15" s="110"/>
+      <c r="L15" s="110"/>
+      <c r="M15" s="132"/>
       <c r="N15" s="41"/>
       <c r="O15" s="7"/>
       <c r="P15" s="7"/>
@@ -3638,29 +3686,29 @@
       <c r="AF15" s="14"/>
       <c r="AG15" s="14"/>
       <c r="AH15" s="14"/>
-      <c r="AI15" s="14"/>
-      <c r="AJ15" s="14"/>
-      <c r="AK15" s="14"/>
-      <c r="AL15" s="14"/>
-      <c r="AM15" s="14"/>
-      <c r="AN15" s="14"/>
-      <c r="AO15" s="14"/>
-      <c r="AP15" s="14"/>
+      <c r="AI15" s="49"/>
+      <c r="AJ15" s="49"/>
+      <c r="AK15" s="49"/>
+      <c r="AL15" s="49"/>
+      <c r="AM15" s="49"/>
+      <c r="AN15" s="49"/>
+      <c r="AO15" s="49"/>
+      <c r="AP15" s="49"/>
       <c r="AQ15" s="14"/>
       <c r="AR15" s="14"/>
       <c r="AS15" s="14"/>
       <c r="AT15" s="14"/>
       <c r="AU15" s="14"/>
       <c r="AV15" s="50"/>
-      <c r="AW15" s="134"/>
-      <c r="AX15" s="120"/>
-      <c r="AY15" s="120"/>
-      <c r="AZ15" s="120" t="s">
-        <v>161</v>
-      </c>
-      <c r="BA15" s="120"/>
-      <c r="BB15" s="120"/>
-      <c r="BC15" s="135"/>
+      <c r="AW15" s="123"/>
+      <c r="AX15" s="111"/>
+      <c r="AY15" s="111"/>
+      <c r="AZ15" s="111" t="s">
+        <v>160</v>
+      </c>
+      <c r="BA15" s="111"/>
+      <c r="BB15" s="111"/>
+      <c r="BC15" s="124"/>
       <c r="BD15" s="41"/>
       <c r="BE15" s="7"/>
       <c r="BF15" s="22"/>
@@ -3678,12 +3726,12 @@
       <c r="E16" s="7"/>
       <c r="F16" s="7"/>
       <c r="G16" s="37"/>
-      <c r="H16" s="144"/>
-      <c r="I16" s="145"/>
-      <c r="J16" s="145"/>
-      <c r="K16" s="145"/>
-      <c r="L16" s="145"/>
-      <c r="M16" s="146"/>
+      <c r="H16" s="133"/>
+      <c r="I16" s="134"/>
+      <c r="J16" s="134"/>
+      <c r="K16" s="134"/>
+      <c r="L16" s="134"/>
+      <c r="M16" s="135"/>
       <c r="N16" s="41"/>
       <c r="O16" s="7"/>
       <c r="P16" s="7"/>
@@ -3704,34 +3752,34 @@
       <c r="AE16" s="7"/>
       <c r="AF16" s="7"/>
       <c r="AG16" s="7"/>
-      <c r="AH16" s="7"/>
-      <c r="AI16" s="7"/>
-      <c r="AJ16" s="7"/>
-      <c r="AK16" s="7"/>
-      <c r="AL16" s="7"/>
-      <c r="AM16" s="7"/>
-      <c r="AN16" s="7"/>
-      <c r="AO16" s="7"/>
-      <c r="AP16" s="7"/>
-      <c r="AQ16" s="7"/>
+      <c r="AH16" s="37"/>
+      <c r="AI16" s="90"/>
+      <c r="AJ16" s="91"/>
+      <c r="AK16" s="91"/>
+      <c r="AL16" s="91"/>
+      <c r="AM16" s="91"/>
+      <c r="AN16" s="91"/>
+      <c r="AO16" s="91"/>
+      <c r="AP16" s="54"/>
+      <c r="AQ16" s="41"/>
       <c r="AR16" s="7"/>
       <c r="AS16" s="7"/>
       <c r="AT16" s="7"/>
       <c r="AU16" s="7"/>
       <c r="AV16" s="37"/>
-      <c r="AW16" s="134"/>
-      <c r="AX16" s="120"/>
-      <c r="AY16" s="120"/>
-      <c r="AZ16" s="120"/>
-      <c r="BA16" s="120"/>
-      <c r="BB16" s="120"/>
-      <c r="BC16" s="135"/>
+      <c r="AW16" s="123"/>
+      <c r="AX16" s="111"/>
+      <c r="AY16" s="111"/>
+      <c r="AZ16" s="111"/>
+      <c r="BA16" s="111"/>
+      <c r="BB16" s="111"/>
+      <c r="BC16" s="124"/>
       <c r="BD16" s="41"/>
       <c r="BE16" s="7"/>
-      <c r="BF16" s="22"/>
-      <c r="BG16" s="22"/>
-      <c r="BH16" s="22"/>
-      <c r="BI16" s="22"/>
+      <c r="BF16" s="15"/>
+      <c r="BG16" s="15"/>
+      <c r="BH16" s="15"/>
+      <c r="BI16" s="15"/>
     </row>
     <row r="17" spans="1:61" ht="18" customHeight="1" thickTop="1" x14ac:dyDescent="0.25">
       <c r="A17" s="6">
@@ -3769,34 +3817,34 @@
       <c r="AE17" s="7"/>
       <c r="AF17" s="7"/>
       <c r="AG17" s="7"/>
-      <c r="AH17" s="7"/>
-      <c r="AI17" s="7"/>
-      <c r="AJ17" s="7"/>
-      <c r="AK17" s="7"/>
-      <c r="AL17" s="7"/>
-      <c r="AM17" s="7"/>
-      <c r="AN17" s="7"/>
-      <c r="AO17" s="7"/>
-      <c r="AP17" s="7"/>
-      <c r="AQ17" s="7"/>
+      <c r="AH17" s="37"/>
+      <c r="AI17" s="92"/>
+      <c r="AJ17" s="170"/>
+      <c r="AK17" s="170"/>
+      <c r="AL17" s="170"/>
+      <c r="AM17" s="170"/>
+      <c r="AN17" s="170"/>
+      <c r="AO17" s="170"/>
+      <c r="AP17" s="59"/>
+      <c r="AQ17" s="41"/>
       <c r="AR17" s="7"/>
       <c r="AS17" s="7"/>
       <c r="AT17" s="7"/>
       <c r="AU17" s="7"/>
       <c r="AV17" s="37"/>
-      <c r="AW17" s="134"/>
-      <c r="AX17" s="120"/>
-      <c r="AY17" s="120"/>
-      <c r="AZ17" s="120"/>
-      <c r="BA17" s="120"/>
-      <c r="BB17" s="120"/>
-      <c r="BC17" s="135"/>
+      <c r="AW17" s="123"/>
+      <c r="AX17" s="111"/>
+      <c r="AY17" s="111"/>
+      <c r="AZ17" s="111"/>
+      <c r="BA17" s="111"/>
+      <c r="BB17" s="111"/>
+      <c r="BC17" s="124"/>
       <c r="BD17" s="41"/>
       <c r="BE17" s="7"/>
-      <c r="BF17" s="22"/>
-      <c r="BG17" s="22"/>
-      <c r="BH17" s="22"/>
-      <c r="BI17" s="22"/>
+      <c r="BF17" s="15"/>
+      <c r="BG17" s="15"/>
+      <c r="BH17" s="15"/>
+      <c r="BI17" s="15"/>
     </row>
     <row r="18" spans="1:61" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A18" s="6">
@@ -3834,34 +3882,36 @@
       <c r="AE18" s="14"/>
       <c r="AF18" s="14"/>
       <c r="AG18" s="7"/>
-      <c r="AH18" s="7"/>
-      <c r="AI18" s="7"/>
-      <c r="AJ18" s="7"/>
-      <c r="AK18" s="7"/>
-      <c r="AL18" s="7"/>
-      <c r="AM18" s="7"/>
-      <c r="AN18" s="7"/>
-      <c r="AO18" s="7"/>
-      <c r="AP18" s="7"/>
-      <c r="AQ18" s="7"/>
+      <c r="AH18" s="37"/>
+      <c r="AI18" s="92"/>
+      <c r="AJ18" s="170"/>
+      <c r="AK18" s="170" t="s">
+        <v>162</v>
+      </c>
+      <c r="AL18" s="170"/>
+      <c r="AM18" s="170"/>
+      <c r="AN18" s="170"/>
+      <c r="AO18" s="170"/>
+      <c r="AP18" s="59"/>
+      <c r="AQ18" s="41"/>
       <c r="AR18" s="7"/>
       <c r="AS18" s="7"/>
       <c r="AT18" s="7"/>
       <c r="AU18" s="7"/>
       <c r="AV18" s="37"/>
-      <c r="AW18" s="136"/>
-      <c r="AX18" s="137"/>
-      <c r="AY18" s="137"/>
-      <c r="AZ18" s="137"/>
-      <c r="BA18" s="137"/>
-      <c r="BB18" s="137"/>
-      <c r="BC18" s="138"/>
+      <c r="AW18" s="125"/>
+      <c r="AX18" s="126"/>
+      <c r="AY18" s="126"/>
+      <c r="AZ18" s="126"/>
+      <c r="BA18" s="126"/>
+      <c r="BB18" s="126"/>
+      <c r="BC18" s="127"/>
       <c r="BD18" s="41"/>
       <c r="BE18" s="7"/>
-      <c r="BF18" s="22"/>
-      <c r="BG18" s="22"/>
-      <c r="BH18" s="22"/>
-      <c r="BI18" s="22"/>
+      <c r="BF18" s="15"/>
+      <c r="BG18" s="15"/>
+      <c r="BH18" s="15"/>
+      <c r="BI18" s="15"/>
     </row>
     <row r="19" spans="1:61" ht="18" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A19" s="6">
@@ -3899,16 +3949,16 @@
       <c r="AE19" s="14"/>
       <c r="AF19" s="14"/>
       <c r="AG19" s="7"/>
-      <c r="AH19" s="7"/>
-      <c r="AI19" s="7"/>
-      <c r="AJ19" s="7"/>
-      <c r="AK19" s="7"/>
-      <c r="AL19" s="7"/>
-      <c r="AM19" s="7"/>
-      <c r="AN19" s="7"/>
-      <c r="AO19" s="7"/>
-      <c r="AP19" s="7"/>
-      <c r="AQ19" s="7"/>
+      <c r="AH19" s="37"/>
+      <c r="AI19" s="92"/>
+      <c r="AJ19" s="170"/>
+      <c r="AK19" s="170"/>
+      <c r="AL19" s="170"/>
+      <c r="AM19" s="170"/>
+      <c r="AN19" s="170"/>
+      <c r="AO19" s="170"/>
+      <c r="AP19" s="59"/>
+      <c r="AQ19" s="41"/>
       <c r="AR19" s="7"/>
       <c r="AS19" s="7"/>
       <c r="AT19" s="7"/>
@@ -3921,14 +3971,14 @@
       <c r="BA19" s="48"/>
       <c r="BB19" s="48"/>
       <c r="BC19" s="48"/>
-      <c r="BD19" s="7"/>
-      <c r="BE19" s="7"/>
-      <c r="BF19" s="22"/>
-      <c r="BG19" s="22"/>
-      <c r="BH19" s="22"/>
-      <c r="BI19" s="22"/>
-    </row>
-    <row r="20" spans="1:61" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="BD19" s="15"/>
+      <c r="BE19" s="15"/>
+      <c r="BF19" s="15"/>
+      <c r="BG19" s="15"/>
+      <c r="BH19" s="15"/>
+      <c r="BI19" s="15"/>
+    </row>
+    <row r="20" spans="1:61" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A20" s="6">
         <v>19</v>
       </c>
@@ -3964,16 +4014,16 @@
       <c r="AE20" s="55"/>
       <c r="AF20" s="14"/>
       <c r="AG20" s="7"/>
-      <c r="AH20" s="7"/>
-      <c r="AI20" s="7"/>
-      <c r="AJ20" s="7"/>
-      <c r="AK20" s="7"/>
-      <c r="AL20" s="7"/>
-      <c r="AM20" s="7"/>
-      <c r="AN20" s="7"/>
-      <c r="AO20" s="7"/>
-      <c r="AP20" s="7"/>
-      <c r="AQ20" s="7"/>
+      <c r="AH20" s="37"/>
+      <c r="AI20" s="94"/>
+      <c r="AJ20" s="95"/>
+      <c r="AK20" s="95"/>
+      <c r="AL20" s="95"/>
+      <c r="AM20" s="95"/>
+      <c r="AN20" s="95"/>
+      <c r="AO20" s="95"/>
+      <c r="AP20" s="67"/>
+      <c r="AQ20" s="41"/>
       <c r="AR20" s="7"/>
       <c r="AS20" s="7"/>
       <c r="AT20" s="7"/>
@@ -3986,7 +4036,7 @@
       <c r="BA20" s="7"/>
       <c r="BB20" s="7"/>
       <c r="BC20" s="7"/>
-      <c r="BD20" s="7"/>
+      <c r="BD20" s="15"/>
       <c r="BE20" s="7"/>
       <c r="BF20" s="22"/>
       <c r="BG20" s="22"/>
@@ -4030,35 +4080,35 @@
       <c r="AD21" s="59"/>
       <c r="AE21" s="55"/>
       <c r="AF21" s="14"/>
-      <c r="AG21" s="7"/>
-      <c r="AH21" s="7"/>
-      <c r="AI21" s="7"/>
-      <c r="AJ21" s="7"/>
-      <c r="AK21" s="7"/>
-      <c r="AL21" s="7"/>
-      <c r="AM21" s="7"/>
-      <c r="AN21" s="7"/>
-      <c r="AO21" s="7"/>
-      <c r="AP21" s="7"/>
-      <c r="AQ21" s="7"/>
-      <c r="AR21" s="7"/>
-      <c r="AS21" s="7"/>
-      <c r="AT21" s="7"/>
-      <c r="AU21" s="7"/>
-      <c r="AV21" s="7"/>
-      <c r="AW21" s="7"/>
-      <c r="AX21" s="7"/>
-      <c r="AY21" s="7"/>
-      <c r="AZ21" s="7"/>
-      <c r="BA21" s="7"/>
-      <c r="BB21" s="7"/>
-      <c r="BC21" s="7"/>
-      <c r="BD21" s="7"/>
-      <c r="BE21" s="7"/>
-      <c r="BF21" s="22"/>
-      <c r="BG21" s="22"/>
-      <c r="BH21" s="22"/>
-      <c r="BI21" s="22"/>
+      <c r="AG21" s="55"/>
+      <c r="AH21" s="55"/>
+      <c r="AI21" s="169"/>
+      <c r="AJ21" s="169"/>
+      <c r="AK21" s="169"/>
+      <c r="AL21" s="169"/>
+      <c r="AM21" s="169"/>
+      <c r="AN21" s="169"/>
+      <c r="AO21" s="169"/>
+      <c r="AP21" s="169"/>
+      <c r="AQ21" s="55"/>
+      <c r="AR21" s="55"/>
+      <c r="AS21" s="55"/>
+      <c r="AT21" s="55"/>
+      <c r="AU21" s="55"/>
+      <c r="AV21" s="55"/>
+      <c r="AW21" s="55"/>
+      <c r="AX21" s="55"/>
+      <c r="AY21" s="55"/>
+      <c r="AZ21" s="55"/>
+      <c r="BA21" s="55"/>
+      <c r="BB21" s="55"/>
+      <c r="BC21" s="55"/>
+      <c r="BD21" s="55"/>
+      <c r="BE21" s="55"/>
+      <c r="BF21" s="55"/>
+      <c r="BG21" s="55"/>
+      <c r="BH21" s="55"/>
+      <c r="BI21" s="55"/>
     </row>
     <row r="22" spans="1:61" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A22" s="6">
@@ -4105,30 +4155,30 @@
       <c r="AD22" s="59"/>
       <c r="AE22" s="55"/>
       <c r="AF22" s="14"/>
-      <c r="AG22" s="7"/>
-      <c r="AH22" s="7"/>
-      <c r="AI22" s="7"/>
-      <c r="AJ22" s="7"/>
-      <c r="AK22" s="7"/>
-      <c r="AL22" s="7"/>
-      <c r="AM22" s="7"/>
-      <c r="AN22" s="7"/>
-      <c r="AO22" s="7"/>
-      <c r="AP22" s="7"/>
-      <c r="AQ22" s="7"/>
-      <c r="AR22" s="7"/>
-      <c r="AS22" s="7"/>
-      <c r="AT22" s="7"/>
-      <c r="AU22" s="7"/>
-      <c r="AV22" s="7"/>
-      <c r="AW22" s="7"/>
-      <c r="AX22" s="7"/>
-      <c r="AY22" s="7"/>
-      <c r="AZ22" s="7"/>
-      <c r="BA22" s="7"/>
-      <c r="BB22" s="7"/>
-      <c r="BC22" s="7"/>
-      <c r="BD22" s="7"/>
+      <c r="AG22" s="173"/>
+      <c r="AH22" s="173"/>
+      <c r="AI22" s="85"/>
+      <c r="AJ22" s="85"/>
+      <c r="AK22" s="173"/>
+      <c r="AL22" s="173"/>
+      <c r="AM22" s="173"/>
+      <c r="AN22" s="173"/>
+      <c r="AO22" s="173"/>
+      <c r="AP22" s="173"/>
+      <c r="AQ22" s="85"/>
+      <c r="AR22" s="85"/>
+      <c r="AS22" s="85"/>
+      <c r="AT22" s="85"/>
+      <c r="AU22" s="86"/>
+      <c r="AV22" s="85"/>
+      <c r="AW22" s="85"/>
+      <c r="AX22" s="85"/>
+      <c r="AY22" s="85"/>
+      <c r="AZ22" s="85"/>
+      <c r="BA22" s="85"/>
+      <c r="BB22" s="85"/>
+      <c r="BC22" s="86"/>
+      <c r="BD22" s="15"/>
       <c r="BE22" s="7"/>
       <c r="BF22" s="22"/>
       <c r="BG22" s="22"/>
@@ -4179,38 +4229,38 @@
       <c r="AC23" s="66"/>
       <c r="AD23" s="67"/>
       <c r="AE23" s="55"/>
-      <c r="AF23" s="14"/>
-      <c r="AG23" s="7"/>
-      <c r="AH23" s="7"/>
-      <c r="AI23" s="7"/>
-      <c r="AJ23" s="7"/>
-      <c r="AK23" s="7"/>
-      <c r="AL23" s="7"/>
-      <c r="AM23" s="7"/>
-      <c r="AN23" s="7"/>
-      <c r="AO23" s="7"/>
-      <c r="AP23" s="7"/>
-      <c r="AQ23" s="7"/>
-      <c r="AR23" s="7"/>
-      <c r="AS23" s="7"/>
-      <c r="AT23" s="7"/>
-      <c r="AU23" s="7"/>
-      <c r="AV23" s="7"/>
-      <c r="AW23" s="7"/>
-      <c r="AX23" s="7"/>
-      <c r="AY23" s="7"/>
-      <c r="AZ23" s="7"/>
-      <c r="BA23" s="7"/>
-      <c r="BB23" s="7"/>
-      <c r="BC23" s="7"/>
-      <c r="BD23" s="7"/>
+      <c r="AF23" s="50"/>
+      <c r="AG23" s="90"/>
+      <c r="AH23" s="54"/>
+      <c r="AI23" s="172"/>
+      <c r="AJ23" s="171"/>
+      <c r="AK23" s="90"/>
+      <c r="AL23" s="91"/>
+      <c r="AM23" s="91"/>
+      <c r="AN23" s="91"/>
+      <c r="AO23" s="91"/>
+      <c r="AP23" s="54"/>
+      <c r="AQ23" s="172"/>
+      <c r="AR23" s="85"/>
+      <c r="AS23" s="85"/>
+      <c r="AT23" s="85"/>
+      <c r="AU23" s="86"/>
+      <c r="AV23" s="85"/>
+      <c r="AW23" s="173"/>
+      <c r="AX23" s="173"/>
+      <c r="AY23" s="85"/>
+      <c r="AZ23" s="85"/>
+      <c r="BA23" s="85"/>
+      <c r="BB23" s="85"/>
+      <c r="BC23" s="86"/>
+      <c r="BD23" s="15"/>
       <c r="BE23" s="7"/>
       <c r="BF23" s="22"/>
       <c r="BG23" s="22"/>
       <c r="BH23" s="22"/>
       <c r="BI23" s="22"/>
     </row>
-    <row r="24" spans="1:61" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:61" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A24" s="6">
         <v>23</v>
       </c>
@@ -4244,38 +4294,38 @@
       <c r="AC24" s="69"/>
       <c r="AD24" s="14"/>
       <c r="AE24" s="14"/>
-      <c r="AF24" s="14"/>
-      <c r="AG24" s="7"/>
-      <c r="AH24" s="7"/>
-      <c r="AI24" s="7"/>
-      <c r="AJ24" s="7"/>
-      <c r="AK24" s="7"/>
-      <c r="AL24" s="7"/>
-      <c r="AM24" s="7"/>
-      <c r="AN24" s="7"/>
-      <c r="AO24" s="7"/>
-      <c r="AP24" s="7"/>
-      <c r="AQ24" s="7"/>
-      <c r="AR24" s="7"/>
-      <c r="AS24" s="7"/>
-      <c r="AT24" s="7"/>
-      <c r="AU24" s="7"/>
-      <c r="AV24" s="7"/>
-      <c r="AW24" s="7"/>
-      <c r="AX24" s="7"/>
-      <c r="AY24" s="7"/>
-      <c r="AZ24" s="7"/>
-      <c r="BA24" s="7"/>
-      <c r="BB24" s="7"/>
-      <c r="BC24" s="7"/>
-      <c r="BD24" s="7"/>
+      <c r="AF24" s="50"/>
+      <c r="AG24" s="92"/>
+      <c r="AH24" s="59"/>
+      <c r="AI24" s="172"/>
+      <c r="AJ24" s="171"/>
+      <c r="AK24" s="94"/>
+      <c r="AL24" s="95"/>
+      <c r="AM24" s="95"/>
+      <c r="AN24" s="95"/>
+      <c r="AO24" s="95"/>
+      <c r="AP24" s="67"/>
+      <c r="AQ24" s="172"/>
+      <c r="AR24" s="85"/>
+      <c r="AS24" s="85"/>
+      <c r="AT24" s="85"/>
+      <c r="AU24" s="86"/>
+      <c r="AV24" s="171"/>
+      <c r="AW24" s="90"/>
+      <c r="AX24" s="54"/>
+      <c r="AY24" s="172"/>
+      <c r="AZ24" s="85"/>
+      <c r="BA24" s="85"/>
+      <c r="BB24" s="85"/>
+      <c r="BC24" s="86"/>
+      <c r="BD24" s="15"/>
       <c r="BE24" s="7"/>
       <c r="BF24" s="22"/>
       <c r="BG24" s="22"/>
       <c r="BH24" s="22"/>
       <c r="BI24" s="22"/>
     </row>
-    <row r="25" spans="1:61" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:61" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A25" s="6">
         <v>24</v>
       </c>
@@ -4309,31 +4359,31 @@
       <c r="AC25" s="14"/>
       <c r="AD25" s="14"/>
       <c r="AE25" s="15"/>
-      <c r="AF25" s="15"/>
-      <c r="AG25" s="7"/>
-      <c r="AH25" s="7"/>
-      <c r="AI25" s="7"/>
-      <c r="AJ25" s="7"/>
-      <c r="AK25" s="7"/>
-      <c r="AL25" s="7"/>
-      <c r="AM25" s="7"/>
-      <c r="AN25" s="7"/>
-      <c r="AO25" s="7"/>
-      <c r="AP25" s="7"/>
-      <c r="AQ25" s="7"/>
-      <c r="AR25" s="7"/>
-      <c r="AS25" s="7"/>
-      <c r="AT25" s="7"/>
-      <c r="AU25" s="7"/>
-      <c r="AV25" s="7"/>
-      <c r="AW25" s="7"/>
-      <c r="AX25" s="7"/>
-      <c r="AY25" s="7"/>
-      <c r="AZ25" s="7"/>
-      <c r="BA25" s="7"/>
-      <c r="BB25" s="7"/>
-      <c r="BC25" s="7"/>
-      <c r="BD25" s="7"/>
+      <c r="AF25" s="44"/>
+      <c r="AG25" s="92"/>
+      <c r="AH25" s="59"/>
+      <c r="AI25" s="172"/>
+      <c r="AJ25" s="85"/>
+      <c r="AK25" s="85"/>
+      <c r="AL25" s="85"/>
+      <c r="AM25" s="85"/>
+      <c r="AN25" s="85"/>
+      <c r="AO25" s="85"/>
+      <c r="AP25" s="85"/>
+      <c r="AQ25" s="85"/>
+      <c r="AR25" s="85"/>
+      <c r="AS25" s="85"/>
+      <c r="AT25" s="85"/>
+      <c r="AU25" s="86"/>
+      <c r="AV25" s="171"/>
+      <c r="AW25" s="92"/>
+      <c r="AX25" s="59"/>
+      <c r="AY25" s="172"/>
+      <c r="AZ25" s="85"/>
+      <c r="BA25" s="85"/>
+      <c r="BB25" s="85"/>
+      <c r="BC25" s="86"/>
+      <c r="BD25" s="15"/>
       <c r="BE25" s="7"/>
       <c r="BF25" s="22"/>
       <c r="BG25" s="22"/>
@@ -4374,31 +4424,31 @@
       <c r="AC26" s="14"/>
       <c r="AD26" s="14"/>
       <c r="AE26" s="15"/>
-      <c r="AF26" s="15"/>
-      <c r="AG26" s="7"/>
-      <c r="AH26" s="7"/>
-      <c r="AI26" s="7"/>
-      <c r="AJ26" s="7"/>
-      <c r="AK26" s="7"/>
-      <c r="AL26" s="7"/>
-      <c r="AM26" s="7"/>
-      <c r="AN26" s="7"/>
-      <c r="AO26" s="7"/>
-      <c r="AP26" s="7"/>
-      <c r="AQ26" s="7"/>
-      <c r="AR26" s="7"/>
-      <c r="AS26" s="7"/>
-      <c r="AT26" s="7"/>
-      <c r="AU26" s="7"/>
-      <c r="AV26" s="7"/>
-      <c r="AW26" s="7"/>
-      <c r="AX26" s="7"/>
-      <c r="AY26" s="7"/>
-      <c r="AZ26" s="7"/>
-      <c r="BA26" s="7"/>
-      <c r="BB26" s="7"/>
-      <c r="BC26" s="7"/>
-      <c r="BD26" s="7"/>
+      <c r="AF26" s="44"/>
+      <c r="AG26" s="94"/>
+      <c r="AH26" s="67"/>
+      <c r="AI26" s="172"/>
+      <c r="AJ26" s="85"/>
+      <c r="AK26" s="85"/>
+      <c r="AL26" s="85"/>
+      <c r="AM26" s="85"/>
+      <c r="AN26" s="85"/>
+      <c r="AO26" s="85"/>
+      <c r="AP26" s="85"/>
+      <c r="AQ26" s="85"/>
+      <c r="AR26" s="85"/>
+      <c r="AS26" s="85"/>
+      <c r="AT26" s="85"/>
+      <c r="AU26" s="86"/>
+      <c r="AV26" s="171"/>
+      <c r="AW26" s="94"/>
+      <c r="AX26" s="67"/>
+      <c r="AY26" s="172"/>
+      <c r="AZ26" s="85"/>
+      <c r="BA26" s="85"/>
+      <c r="BB26" s="85"/>
+      <c r="BC26" s="86"/>
+      <c r="BD26" s="15"/>
       <c r="BE26" s="7"/>
       <c r="BF26" s="22"/>
       <c r="BG26" s="22"/>
@@ -4440,30 +4490,30 @@
       <c r="AD27" s="14"/>
       <c r="AE27" s="14"/>
       <c r="AF27" s="14"/>
-      <c r="AG27" s="14"/>
-      <c r="AH27" s="14"/>
+      <c r="AG27" s="69"/>
+      <c r="AH27" s="69"/>
       <c r="AI27" s="14"/>
-      <c r="AJ27" s="7"/>
-      <c r="AK27" s="7"/>
-      <c r="AL27" s="7"/>
-      <c r="AM27" s="7"/>
-      <c r="AN27" s="7"/>
-      <c r="AO27" s="7"/>
-      <c r="AP27" s="7"/>
-      <c r="AQ27" s="7"/>
-      <c r="AR27" s="7"/>
-      <c r="AS27" s="7"/>
-      <c r="AT27" s="7"/>
-      <c r="AU27" s="7"/>
-      <c r="AV27" s="7"/>
-      <c r="AW27" s="7"/>
-      <c r="AX27" s="7"/>
-      <c r="AY27" s="7"/>
-      <c r="AZ27" s="7"/>
-      <c r="BA27" s="7"/>
-      <c r="BB27" s="7"/>
-      <c r="BC27" s="7"/>
-      <c r="BD27" s="7"/>
+      <c r="AJ27" s="86"/>
+      <c r="AK27" s="86"/>
+      <c r="AL27" s="86"/>
+      <c r="AM27" s="86"/>
+      <c r="AN27" s="86"/>
+      <c r="AO27" s="86"/>
+      <c r="AP27" s="86"/>
+      <c r="AQ27" s="86"/>
+      <c r="AR27" s="86"/>
+      <c r="AS27" s="86"/>
+      <c r="AT27" s="86"/>
+      <c r="AU27" s="86"/>
+      <c r="AV27" s="86"/>
+      <c r="AW27" s="86"/>
+      <c r="AX27" s="86"/>
+      <c r="AY27" s="86"/>
+      <c r="AZ27" s="86"/>
+      <c r="BA27" s="86"/>
+      <c r="BB27" s="86"/>
+      <c r="BC27" s="86"/>
+      <c r="BD27" s="15"/>
       <c r="BE27" s="7"/>
       <c r="BF27" s="22"/>
       <c r="BG27" s="22"/>
@@ -4508,10 +4558,10 @@
       <c r="AG28" s="49"/>
       <c r="AH28" s="14"/>
       <c r="AI28" s="14"/>
-      <c r="AJ28" s="7"/>
-      <c r="AK28" s="7"/>
-      <c r="AL28" s="7"/>
-      <c r="AM28" s="7"/>
+      <c r="AJ28" s="86"/>
+      <c r="AK28" s="86"/>
+      <c r="AL28" s="86"/>
+      <c r="AM28" s="86"/>
       <c r="AN28" s="14"/>
       <c r="AO28" s="49"/>
       <c r="AP28" s="49"/>
@@ -4522,13 +4572,13 @@
       <c r="AU28" s="49"/>
       <c r="AV28" s="49"/>
       <c r="AW28" s="14"/>
-      <c r="AX28" s="7"/>
-      <c r="AY28" s="7"/>
-      <c r="AZ28" s="7"/>
-      <c r="BA28" s="7"/>
-      <c r="BB28" s="7"/>
-      <c r="BC28" s="7"/>
-      <c r="BD28" s="7"/>
+      <c r="AX28" s="86"/>
+      <c r="AY28" s="86"/>
+      <c r="AZ28" s="86"/>
+      <c r="BA28" s="86"/>
+      <c r="BB28" s="86"/>
+      <c r="BC28" s="86"/>
+      <c r="BD28" s="15"/>
       <c r="BE28" s="7"/>
       <c r="BF28" s="22"/>
       <c r="BG28" s="22"/>
@@ -4566,34 +4616,34 @@
       <c r="Z29" s="16"/>
       <c r="AA29" s="14"/>
       <c r="AB29" s="50"/>
-      <c r="AC29" s="164"/>
-      <c r="AD29" s="165"/>
-      <c r="AE29" s="165"/>
-      <c r="AF29" s="165"/>
-      <c r="AG29" s="166"/>
+      <c r="AC29" s="152"/>
+      <c r="AD29" s="153"/>
+      <c r="AE29" s="153"/>
+      <c r="AF29" s="153"/>
+      <c r="AG29" s="154"/>
       <c r="AH29" s="55"/>
       <c r="AI29" s="14"/>
-      <c r="AJ29" s="7"/>
-      <c r="AK29" s="7"/>
-      <c r="AL29" s="7"/>
-      <c r="AM29" s="7"/>
+      <c r="AJ29" s="86"/>
+      <c r="AK29" s="86"/>
+      <c r="AL29" s="86"/>
+      <c r="AM29" s="86"/>
       <c r="AN29" s="50"/>
-      <c r="AO29" s="155"/>
-      <c r="AP29" s="156"/>
-      <c r="AQ29" s="156"/>
-      <c r="AR29" s="156"/>
-      <c r="AS29" s="156"/>
-      <c r="AT29" s="156"/>
-      <c r="AU29" s="156"/>
-      <c r="AV29" s="157"/>
+      <c r="AO29" s="144"/>
+      <c r="AP29" s="145"/>
+      <c r="AQ29" s="145"/>
+      <c r="AR29" s="145"/>
+      <c r="AS29" s="145"/>
+      <c r="AT29" s="145"/>
+      <c r="AU29" s="145"/>
+      <c r="AV29" s="146"/>
       <c r="AW29" s="55"/>
-      <c r="AX29" s="7"/>
-      <c r="AY29" s="7"/>
-      <c r="AZ29" s="7"/>
-      <c r="BA29" s="7"/>
-      <c r="BB29" s="7"/>
-      <c r="BC29" s="7"/>
-      <c r="BD29" s="7"/>
+      <c r="AX29" s="86"/>
+      <c r="AY29" s="86"/>
+      <c r="AZ29" s="86"/>
+      <c r="BA29" s="86"/>
+      <c r="BB29" s="86"/>
+      <c r="BC29" s="86"/>
+      <c r="BD29" s="15"/>
       <c r="BE29" s="7"/>
       <c r="BF29" s="22"/>
       <c r="BG29" s="22"/>
@@ -4631,11 +4681,11 @@
       <c r="Z30" s="16"/>
       <c r="AA30" s="14"/>
       <c r="AB30" s="50"/>
-      <c r="AC30" s="167"/>
-      <c r="AD30" s="122"/>
-      <c r="AE30" s="122"/>
-      <c r="AF30" s="122"/>
-      <c r="AG30" s="168"/>
+      <c r="AC30" s="155"/>
+      <c r="AD30" s="93"/>
+      <c r="AE30" s="93"/>
+      <c r="AF30" s="93"/>
+      <c r="AG30" s="156"/>
       <c r="AH30" s="55"/>
       <c r="AI30" s="14"/>
       <c r="AJ30" s="15"/>
@@ -4643,14 +4693,14 @@
       <c r="AL30" s="15"/>
       <c r="AM30" s="15"/>
       <c r="AN30" s="50"/>
-      <c r="AO30" s="158"/>
-      <c r="AP30" s="117"/>
-      <c r="AQ30" s="117"/>
-      <c r="AR30" s="117"/>
-      <c r="AS30" s="117"/>
-      <c r="AT30" s="117"/>
-      <c r="AU30" s="117"/>
-      <c r="AV30" s="159"/>
+      <c r="AO30" s="147"/>
+      <c r="AP30" s="108"/>
+      <c r="AQ30" s="108"/>
+      <c r="AR30" s="108"/>
+      <c r="AS30" s="108"/>
+      <c r="AT30" s="108"/>
+      <c r="AU30" s="108"/>
+      <c r="AV30" s="148"/>
       <c r="AW30" s="55"/>
       <c r="AX30" s="15"/>
       <c r="AY30" s="15"/>
@@ -4696,13 +4746,13 @@
       <c r="Z31" s="16"/>
       <c r="AA31" s="14"/>
       <c r="AB31" s="50"/>
-      <c r="AC31" s="167"/>
-      <c r="AD31" s="122"/>
-      <c r="AE31" s="122" t="s">
-        <v>151</v>
-      </c>
-      <c r="AF31" s="122"/>
-      <c r="AG31" s="168"/>
+      <c r="AC31" s="155"/>
+      <c r="AD31" s="93"/>
+      <c r="AE31" s="93" t="s">
+        <v>161</v>
+      </c>
+      <c r="AF31" s="93"/>
+      <c r="AG31" s="156"/>
       <c r="AH31" s="55"/>
       <c r="AI31" s="14"/>
       <c r="AJ31" s="16"/>
@@ -4710,16 +4760,16 @@
       <c r="AL31" s="16"/>
       <c r="AM31" s="7"/>
       <c r="AN31" s="50"/>
-      <c r="AO31" s="158"/>
-      <c r="AP31" s="117"/>
-      <c r="AQ31" s="117" t="s">
-        <v>160</v>
-      </c>
-      <c r="AR31" s="117"/>
-      <c r="AS31" s="117"/>
-      <c r="AT31" s="117"/>
-      <c r="AU31" s="117"/>
-      <c r="AV31" s="159"/>
+      <c r="AO31" s="147"/>
+      <c r="AP31" s="108"/>
+      <c r="AQ31" s="108" t="s">
+        <v>159</v>
+      </c>
+      <c r="AR31" s="108"/>
+      <c r="AS31" s="108"/>
+      <c r="AT31" s="108"/>
+      <c r="AU31" s="108"/>
+      <c r="AV31" s="148"/>
       <c r="AW31" s="55"/>
       <c r="AX31" s="7"/>
       <c r="AY31" s="7"/>
@@ -4765,13 +4815,13 @@
       <c r="Z32" s="16"/>
       <c r="AA32" s="14"/>
       <c r="AB32" s="50"/>
-      <c r="AC32" s="167"/>
-      <c r="AD32" s="122" t="s">
-        <v>161</v>
-      </c>
-      <c r="AE32" s="122"/>
-      <c r="AF32" s="122"/>
-      <c r="AG32" s="168"/>
+      <c r="AC32" s="155"/>
+      <c r="AD32" s="93" t="s">
+        <v>160</v>
+      </c>
+      <c r="AE32" s="93"/>
+      <c r="AF32" s="93"/>
+      <c r="AG32" s="156"/>
       <c r="AH32" s="55"/>
       <c r="AI32" s="14"/>
       <c r="AJ32" s="16"/>
@@ -4779,14 +4829,14 @@
       <c r="AL32" s="16"/>
       <c r="AM32" s="7"/>
       <c r="AN32" s="50"/>
-      <c r="AO32" s="158"/>
-      <c r="AP32" s="117"/>
-      <c r="AQ32" s="117"/>
-      <c r="AR32" s="117"/>
-      <c r="AS32" s="117"/>
-      <c r="AT32" s="117"/>
-      <c r="AU32" s="117"/>
-      <c r="AV32" s="159"/>
+      <c r="AO32" s="147"/>
+      <c r="AP32" s="108"/>
+      <c r="AQ32" s="108"/>
+      <c r="AR32" s="108"/>
+      <c r="AS32" s="108"/>
+      <c r="AT32" s="108"/>
+      <c r="AU32" s="108"/>
+      <c r="AV32" s="148"/>
       <c r="AW32" s="55"/>
       <c r="AX32" s="7"/>
       <c r="AY32" s="7"/>
@@ -4832,11 +4882,11 @@
       <c r="Z33" s="16"/>
       <c r="AA33" s="14"/>
       <c r="AB33" s="50"/>
-      <c r="AC33" s="169"/>
-      <c r="AD33" s="170"/>
-      <c r="AE33" s="170"/>
-      <c r="AF33" s="170"/>
-      <c r="AG33" s="171"/>
+      <c r="AC33" s="157"/>
+      <c r="AD33" s="158"/>
+      <c r="AE33" s="158"/>
+      <c r="AF33" s="158"/>
+      <c r="AG33" s="159"/>
       <c r="AH33" s="55"/>
       <c r="AI33" s="14"/>
       <c r="AJ33" s="16"/>
@@ -4844,14 +4894,14 @@
       <c r="AL33" s="16"/>
       <c r="AM33" s="7"/>
       <c r="AN33" s="50"/>
-      <c r="AO33" s="160"/>
-      <c r="AP33" s="161"/>
-      <c r="AQ33" s="161"/>
-      <c r="AR33" s="161"/>
-      <c r="AS33" s="161"/>
-      <c r="AT33" s="161"/>
-      <c r="AU33" s="161"/>
-      <c r="AV33" s="162"/>
+      <c r="AO33" s="149"/>
+      <c r="AP33" s="150"/>
+      <c r="AQ33" s="150"/>
+      <c r="AR33" s="150"/>
+      <c r="AS33" s="150"/>
+      <c r="AT33" s="150"/>
+      <c r="AU33" s="150"/>
+      <c r="AV33" s="151"/>
       <c r="AW33" s="55"/>
       <c r="AX33" s="7"/>
       <c r="AY33" s="7"/>
@@ -5043,15 +5093,15 @@
       <c r="AP36" s="15"/>
       <c r="AQ36" s="14"/>
       <c r="AR36" s="50"/>
-      <c r="AS36" s="147"/>
-      <c r="AT36" s="148"/>
-      <c r="AU36" s="148"/>
-      <c r="AV36" s="148"/>
-      <c r="AW36" s="148"/>
-      <c r="AX36" s="148"/>
-      <c r="AY36" s="148"/>
-      <c r="AZ36" s="148"/>
-      <c r="BA36" s="149"/>
+      <c r="AS36" s="136"/>
+      <c r="AT36" s="137"/>
+      <c r="AU36" s="137"/>
+      <c r="AV36" s="137"/>
+      <c r="AW36" s="137"/>
+      <c r="AX36" s="137"/>
+      <c r="AY36" s="137"/>
+      <c r="AZ36" s="137"/>
+      <c r="BA36" s="138"/>
       <c r="BB36" s="55"/>
       <c r="BC36" s="14"/>
       <c r="BD36" s="15"/>
@@ -5096,7 +5146,7 @@
       <c r="AD37" s="93"/>
       <c r="AE37" s="93"/>
       <c r="AF37" s="93" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="AG37" s="93"/>
       <c r="AH37" s="59"/>
@@ -5110,15 +5160,15 @@
       <c r="AP37" s="15"/>
       <c r="AQ37" s="14"/>
       <c r="AR37" s="50"/>
-      <c r="AS37" s="150"/>
-      <c r="AT37" s="118"/>
-      <c r="AU37" s="118"/>
-      <c r="AV37" s="118"/>
-      <c r="AW37" s="118"/>
-      <c r="AX37" s="118"/>
-      <c r="AY37" s="118"/>
-      <c r="AZ37" s="118"/>
-      <c r="BA37" s="151"/>
+      <c r="AS37" s="139"/>
+      <c r="AT37" s="109"/>
+      <c r="AU37" s="109"/>
+      <c r="AV37" s="109"/>
+      <c r="AW37" s="109"/>
+      <c r="AX37" s="109"/>
+      <c r="AY37" s="109"/>
+      <c r="AZ37" s="109"/>
+      <c r="BA37" s="140"/>
       <c r="BB37" s="55"/>
       <c r="BC37" s="14"/>
       <c r="BD37" s="15"/>
@@ -5175,15 +5225,15 @@
       <c r="AP38" s="15"/>
       <c r="AQ38" s="14"/>
       <c r="AR38" s="50"/>
-      <c r="AS38" s="150"/>
-      <c r="AT38" s="118"/>
-      <c r="AU38" s="118"/>
-      <c r="AV38" s="118"/>
-      <c r="AW38" s="118"/>
-      <c r="AX38" s="118"/>
-      <c r="AY38" s="118"/>
-      <c r="AZ38" s="118"/>
-      <c r="BA38" s="151"/>
+      <c r="AS38" s="139"/>
+      <c r="AT38" s="109"/>
+      <c r="AU38" s="109"/>
+      <c r="AV38" s="109"/>
+      <c r="AW38" s="109"/>
+      <c r="AX38" s="109"/>
+      <c r="AY38" s="109"/>
+      <c r="AZ38" s="109"/>
+      <c r="BA38" s="140"/>
       <c r="BB38" s="55"/>
       <c r="BC38" s="14"/>
       <c r="BD38" s="15"/>
@@ -5240,17 +5290,17 @@
       <c r="AP39" s="15"/>
       <c r="AQ39" s="14"/>
       <c r="AR39" s="50"/>
-      <c r="AS39" s="150"/>
-      <c r="AT39" s="118"/>
-      <c r="AU39" s="118"/>
-      <c r="AV39" s="118" t="s">
-        <v>159</v>
-      </c>
-      <c r="AW39" s="118"/>
-      <c r="AX39" s="118"/>
-      <c r="AY39" s="118"/>
-      <c r="AZ39" s="118"/>
-      <c r="BA39" s="151"/>
+      <c r="AS39" s="139"/>
+      <c r="AT39" s="109"/>
+      <c r="AU39" s="109"/>
+      <c r="AV39" s="109" t="s">
+        <v>158</v>
+      </c>
+      <c r="AW39" s="109"/>
+      <c r="AX39" s="109"/>
+      <c r="AY39" s="109"/>
+      <c r="AZ39" s="109"/>
+      <c r="BA39" s="140"/>
       <c r="BB39" s="55"/>
       <c r="BC39" s="14"/>
       <c r="BD39" s="15"/>
@@ -5307,15 +5357,15 @@
       <c r="AP40" s="15"/>
       <c r="AQ40" s="14"/>
       <c r="AR40" s="50"/>
-      <c r="AS40" s="150"/>
-      <c r="AT40" s="118"/>
-      <c r="AU40" s="118"/>
-      <c r="AV40" s="118"/>
-      <c r="AW40" s="118"/>
-      <c r="AX40" s="118"/>
-      <c r="AY40" s="118"/>
-      <c r="AZ40" s="118"/>
-      <c r="BA40" s="151"/>
+      <c r="AS40" s="139"/>
+      <c r="AT40" s="109"/>
+      <c r="AU40" s="109"/>
+      <c r="AV40" s="109"/>
+      <c r="AW40" s="109"/>
+      <c r="AX40" s="109"/>
+      <c r="AY40" s="109"/>
+      <c r="AZ40" s="109"/>
+      <c r="BA40" s="140"/>
       <c r="BB40" s="55"/>
       <c r="BC40" s="14"/>
       <c r="BD40" s="15"/>
@@ -5372,15 +5422,15 @@
       <c r="AP41" s="15"/>
       <c r="AQ41" s="14"/>
       <c r="AR41" s="50"/>
-      <c r="AS41" s="150"/>
-      <c r="AT41" s="118"/>
-      <c r="AU41" s="118"/>
-      <c r="AV41" s="118"/>
-      <c r="AW41" s="118"/>
-      <c r="AX41" s="118"/>
-      <c r="AY41" s="118"/>
-      <c r="AZ41" s="118"/>
-      <c r="BA41" s="151"/>
+      <c r="AS41" s="139"/>
+      <c r="AT41" s="109"/>
+      <c r="AU41" s="109"/>
+      <c r="AV41" s="109"/>
+      <c r="AW41" s="109"/>
+      <c r="AX41" s="109"/>
+      <c r="AY41" s="109"/>
+      <c r="AZ41" s="109"/>
+      <c r="BA41" s="140"/>
       <c r="BB41" s="55"/>
       <c r="BC41" s="14"/>
       <c r="BD41" s="15"/>
@@ -5437,15 +5487,15 @@
       <c r="AP42" s="15"/>
       <c r="AQ42" s="14"/>
       <c r="AR42" s="50"/>
-      <c r="AS42" s="152"/>
-      <c r="AT42" s="153"/>
-      <c r="AU42" s="153"/>
-      <c r="AV42" s="153"/>
-      <c r="AW42" s="153"/>
-      <c r="AX42" s="153"/>
-      <c r="AY42" s="153"/>
-      <c r="AZ42" s="153"/>
-      <c r="BA42" s="154"/>
+      <c r="AS42" s="141"/>
+      <c r="AT42" s="142"/>
+      <c r="AU42" s="142"/>
+      <c r="AV42" s="142"/>
+      <c r="AW42" s="142"/>
+      <c r="AX42" s="142"/>
+      <c r="AY42" s="142"/>
+      <c r="AZ42" s="142"/>
+      <c r="BA42" s="143"/>
       <c r="BB42" s="55"/>
       <c r="BC42" s="14"/>
       <c r="BD42" s="15"/>
@@ -5725,10 +5775,10 @@
       <c r="E47" s="7"/>
       <c r="F47" s="7"/>
       <c r="G47" s="37"/>
-      <c r="H47" s="123"/>
-      <c r="I47" s="124"/>
-      <c r="J47" s="124"/>
-      <c r="K47" s="125"/>
+      <c r="H47" s="112"/>
+      <c r="I47" s="113"/>
+      <c r="J47" s="113"/>
+      <c r="K47" s="114"/>
       <c r="L47" s="41"/>
       <c r="M47" s="7"/>
       <c r="N47" s="7"/>
@@ -5790,10 +5840,10 @@
       <c r="E48" s="7"/>
       <c r="F48" s="7"/>
       <c r="G48" s="37"/>
-      <c r="H48" s="126"/>
-      <c r="I48" s="121"/>
-      <c r="J48" s="121"/>
-      <c r="K48" s="127"/>
+      <c r="H48" s="115"/>
+      <c r="I48" s="98"/>
+      <c r="J48" s="98"/>
+      <c r="K48" s="116"/>
       <c r="L48" s="41"/>
       <c r="M48" s="7"/>
       <c r="N48" s="7"/>
@@ -5855,12 +5905,12 @@
       <c r="E49" s="7"/>
       <c r="F49" s="7"/>
       <c r="G49" s="37"/>
-      <c r="H49" s="126"/>
-      <c r="I49" s="121" t="s">
-        <v>161</v>
-      </c>
-      <c r="J49" s="121"/>
-      <c r="K49" s="127"/>
+      <c r="H49" s="115"/>
+      <c r="I49" s="98" t="s">
+        <v>160</v>
+      </c>
+      <c r="J49" s="98"/>
+      <c r="K49" s="116"/>
       <c r="L49" s="55"/>
       <c r="M49" s="14"/>
       <c r="N49" s="14"/>
@@ -5922,10 +5972,10 @@
       <c r="E50" s="7"/>
       <c r="F50" s="7"/>
       <c r="G50" s="37"/>
-      <c r="H50" s="126"/>
-      <c r="I50" s="121"/>
-      <c r="J50" s="121"/>
-      <c r="K50" s="127"/>
+      <c r="H50" s="115"/>
+      <c r="I50" s="98"/>
+      <c r="J50" s="98"/>
+      <c r="K50" s="116"/>
       <c r="L50" s="55"/>
       <c r="M50" s="14"/>
       <c r="N50" s="14"/>
@@ -5987,10 +6037,10 @@
       <c r="E51" s="7"/>
       <c r="F51" s="7"/>
       <c r="G51" s="37"/>
-      <c r="H51" s="126"/>
-      <c r="I51" s="121"/>
-      <c r="J51" s="121"/>
-      <c r="K51" s="127"/>
+      <c r="H51" s="115"/>
+      <c r="I51" s="98"/>
+      <c r="J51" s="98"/>
+      <c r="K51" s="116"/>
       <c r="L51" s="41"/>
       <c r="M51" s="7"/>
       <c r="N51" s="7"/>
@@ -6052,10 +6102,10 @@
       <c r="E52" s="7"/>
       <c r="F52" s="7"/>
       <c r="G52" s="37"/>
-      <c r="H52" s="126"/>
-      <c r="I52" s="121"/>
-      <c r="J52" s="121"/>
-      <c r="K52" s="127"/>
+      <c r="H52" s="115"/>
+      <c r="I52" s="98"/>
+      <c r="J52" s="98"/>
+      <c r="K52" s="116"/>
       <c r="L52" s="41"/>
       <c r="M52" s="7"/>
       <c r="N52" s="7"/>
@@ -6117,10 +6167,10 @@
       <c r="E53" s="7"/>
       <c r="F53" s="7"/>
       <c r="G53" s="37"/>
-      <c r="H53" s="126"/>
-      <c r="I53" s="121"/>
-      <c r="J53" s="121"/>
-      <c r="K53" s="127"/>
+      <c r="H53" s="115"/>
+      <c r="I53" s="98"/>
+      <c r="J53" s="98"/>
+      <c r="K53" s="116"/>
       <c r="L53" s="41"/>
       <c r="M53" s="7"/>
       <c r="N53" s="37"/>
@@ -6182,10 +6232,10 @@
       <c r="E54" s="7"/>
       <c r="F54" s="7"/>
       <c r="G54" s="37"/>
-      <c r="H54" s="128"/>
-      <c r="I54" s="129"/>
-      <c r="J54" s="129"/>
-      <c r="K54" s="130"/>
+      <c r="H54" s="117"/>
+      <c r="I54" s="118"/>
+      <c r="J54" s="118"/>
+      <c r="K54" s="119"/>
       <c r="L54" s="41"/>
       <c r="M54" s="7"/>
       <c r="N54" s="37"/>
@@ -10799,50 +10849,50 @@
       <c r="BI61" s="8"/>
     </row>
     <row r="63" spans="1:61" x14ac:dyDescent="0.25">
-      <c r="A63" s="111" t="s">
+      <c r="A63" s="168" t="s">
         <v>15</v>
       </c>
-      <c r="B63" s="109"/>
-      <c r="C63" s="109"/>
-      <c r="D63" s="109"/>
-      <c r="E63" s="109"/>
-      <c r="F63" s="109"/>
-      <c r="G63" s="109"/>
-      <c r="H63" s="109"/>
-      <c r="I63" s="109"/>
-      <c r="J63" s="109"/>
-      <c r="K63" s="109"/>
-      <c r="L63" s="109"/>
-      <c r="M63" s="109"/>
-      <c r="N63" s="109"/>
-      <c r="O63" s="109"/>
-      <c r="P63" s="109"/>
-      <c r="Q63" s="109"/>
-      <c r="R63" s="109"/>
-      <c r="S63" s="109"/>
-      <c r="T63" s="109"/>
+      <c r="B63" s="161"/>
+      <c r="C63" s="161"/>
+      <c r="D63" s="161"/>
+      <c r="E63" s="161"/>
+      <c r="F63" s="161"/>
+      <c r="G63" s="161"/>
+      <c r="H63" s="161"/>
+      <c r="I63" s="161"/>
+      <c r="J63" s="161"/>
+      <c r="K63" s="161"/>
+      <c r="L63" s="161"/>
+      <c r="M63" s="161"/>
+      <c r="N63" s="161"/>
+      <c r="O63" s="161"/>
+      <c r="P63" s="161"/>
+      <c r="Q63" s="161"/>
+      <c r="R63" s="161"/>
+      <c r="S63" s="161"/>
+      <c r="T63" s="161"/>
     </row>
     <row r="64" spans="1:61" x14ac:dyDescent="0.25">
-      <c r="A64" s="109"/>
-      <c r="B64" s="109"/>
-      <c r="C64" s="109"/>
-      <c r="D64" s="109"/>
-      <c r="E64" s="109"/>
-      <c r="F64" s="109"/>
-      <c r="G64" s="109"/>
-      <c r="H64" s="109"/>
-      <c r="I64" s="109"/>
-      <c r="J64" s="109"/>
-      <c r="K64" s="109"/>
-      <c r="L64" s="109"/>
-      <c r="M64" s="109"/>
-      <c r="N64" s="109"/>
-      <c r="O64" s="109"/>
-      <c r="P64" s="109"/>
-      <c r="Q64" s="109"/>
-      <c r="R64" s="109"/>
-      <c r="S64" s="109"/>
-      <c r="T64" s="109"/>
+      <c r="A64" s="161"/>
+      <c r="B64" s="161"/>
+      <c r="C64" s="161"/>
+      <c r="D64" s="161"/>
+      <c r="E64" s="161"/>
+      <c r="F64" s="161"/>
+      <c r="G64" s="161"/>
+      <c r="H64" s="161"/>
+      <c r="I64" s="161"/>
+      <c r="J64" s="161"/>
+      <c r="K64" s="161"/>
+      <c r="L64" s="161"/>
+      <c r="M64" s="161"/>
+      <c r="N64" s="161"/>
+      <c r="O64" s="161"/>
+      <c r="P64" s="161"/>
+      <c r="Q64" s="161"/>
+      <c r="R64" s="161"/>
+      <c r="S64" s="161"/>
+      <c r="T64" s="161"/>
     </row>
     <row r="66" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B66" s="9"/>
@@ -10868,33 +10918,33 @@
   <dimension ref="A1:E74"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="6" customWidth="1"/>
+    <col min="1" max="1" width="8.140625" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="20" customWidth="1"/>
     <col min="3" max="3" width="12" customWidth="1"/>
     <col min="4" max="4" width="60" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:4" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="A1" s="108" t="s">
+      <c r="A1" s="164" t="s">
         <v>16</v>
       </c>
-      <c r="B1" s="109"/>
-      <c r="C1" s="109"/>
-      <c r="D1" s="109"/>
+      <c r="B1" s="161"/>
+      <c r="C1" s="161"/>
+      <c r="D1" s="161"/>
     </row>
     <row r="3" spans="1:4" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="116" t="s">
+      <c r="A3" s="166" t="s">
         <v>17</v>
       </c>
-      <c r="B3" s="109"/>
-      <c r="C3" s="109"/>
-      <c r="D3" s="109"/>
+      <c r="B3" s="161"/>
+      <c r="C3" s="161"/>
+      <c r="D3" s="161"/>
     </row>
     <row r="4" spans="1:4" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="109"/>
-      <c r="B4" s="109"/>
-      <c r="C4" s="109"/>
-      <c r="D4" s="109"/>
+      <c r="A4" s="161"/>
+      <c r="B4" s="161"/>
+      <c r="C4" s="161"/>
+      <c r="D4" s="161"/>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A6" s="1" t="s">
@@ -10911,12 +10961,12 @@
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A7" s="115" t="s">
+      <c r="A7" s="165" t="s">
         <v>22</v>
       </c>
-      <c r="B7" s="109"/>
-      <c r="C7" s="109"/>
-      <c r="D7" s="109"/>
+      <c r="B7" s="161"/>
+      <c r="C7" s="161"/>
+      <c r="D7" s="161"/>
     </row>
     <row r="8" spans="1:4" ht="24" x14ac:dyDescent="0.25">
       <c r="A8" s="12"/>
@@ -11051,20 +11101,20 @@
       </c>
     </row>
     <row r="19" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A19" s="113" t="s">
+      <c r="A19" s="163" t="s">
         <v>46</v>
       </c>
-      <c r="B19" s="109"/>
-      <c r="C19" s="109"/>
-      <c r="D19" s="109"/>
+      <c r="B19" s="161"/>
+      <c r="C19" s="161"/>
+      <c r="D19" s="161"/>
     </row>
     <row r="21" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A21" s="115" t="s">
+      <c r="A21" s="165" t="s">
         <v>47</v>
       </c>
-      <c r="B21" s="109"/>
-      <c r="C21" s="109"/>
-      <c r="D21" s="109"/>
+      <c r="B21" s="161"/>
+      <c r="C21" s="161"/>
+      <c r="D21" s="161"/>
     </row>
     <row r="22" spans="1:5" ht="24" x14ac:dyDescent="0.25">
       <c r="A22" s="23"/>
@@ -11078,7 +11128,7 @@
         <v>50</v>
       </c>
       <c r="E22" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
     </row>
     <row r="23" spans="1:5" ht="24" x14ac:dyDescent="0.25">
@@ -11093,7 +11143,7 @@
         <v>52</v>
       </c>
       <c r="E23" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
     </row>
     <row r="24" spans="1:5" ht="24" x14ac:dyDescent="0.25">
@@ -11108,7 +11158,7 @@
         <v>54</v>
       </c>
       <c r="E24" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
     </row>
     <row r="25" spans="1:5" ht="24" x14ac:dyDescent="0.25">
@@ -11123,7 +11173,7 @@
         <v>56</v>
       </c>
       <c r="E25" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
     </row>
     <row r="26" spans="1:5" ht="24" x14ac:dyDescent="0.25">
@@ -11138,7 +11188,7 @@
         <v>58</v>
       </c>
       <c r="E26" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
     </row>
     <row r="27" spans="1:5" ht="24" x14ac:dyDescent="0.25">
@@ -11153,352 +11203,352 @@
         <v>60</v>
       </c>
       <c r="E27" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
     </row>
     <row r="28" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A28" s="113" t="s">
+      <c r="A28" s="163" t="s">
         <v>61</v>
       </c>
-      <c r="B28" s="109"/>
-      <c r="C28" s="109"/>
-      <c r="D28" s="109"/>
+      <c r="B28" s="161"/>
+      <c r="C28" s="161"/>
+      <c r="D28" s="161"/>
     </row>
     <row r="32" spans="1:5" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A32" s="114" t="s">
+      <c r="A32" s="160" t="s">
         <v>62</v>
       </c>
-      <c r="B32" s="109"/>
-      <c r="C32" s="109"/>
-      <c r="D32" s="109"/>
+      <c r="B32" s="161"/>
+      <c r="C32" s="161"/>
+      <c r="D32" s="161"/>
     </row>
     <row r="33" spans="1:4" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A33" s="112" t="s">
+      <c r="A33" s="162" t="s">
         <v>63</v>
       </c>
-      <c r="B33" s="109"/>
-      <c r="C33" s="109"/>
-      <c r="D33" s="109"/>
+      <c r="B33" s="161"/>
+      <c r="C33" s="161"/>
+      <c r="D33" s="161"/>
     </row>
     <row r="34" spans="1:4" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A34" s="112" t="s">
+      <c r="A34" s="162" t="s">
         <v>64</v>
       </c>
-      <c r="B34" s="109"/>
-      <c r="C34" s="109"/>
-      <c r="D34" s="109"/>
+      <c r="B34" s="161"/>
+      <c r="C34" s="161"/>
+      <c r="D34" s="161"/>
     </row>
     <row r="35" spans="1:4" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A35" s="112" t="s">
+      <c r="A35" s="162" t="s">
         <v>65</v>
       </c>
-      <c r="B35" s="109"/>
-      <c r="C35" s="109"/>
-      <c r="D35" s="109"/>
+      <c r="B35" s="161"/>
+      <c r="C35" s="161"/>
+      <c r="D35" s="161"/>
     </row>
     <row r="36" spans="1:4" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A36" s="112" t="s">
+      <c r="A36" s="162" t="s">
         <v>66</v>
       </c>
-      <c r="B36" s="109"/>
-      <c r="C36" s="109"/>
-      <c r="D36" s="109"/>
+      <c r="B36" s="161"/>
+      <c r="C36" s="161"/>
+      <c r="D36" s="161"/>
     </row>
     <row r="37" spans="1:4" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A37" s="112" t="s">
+      <c r="A37" s="162" t="s">
         <v>67</v>
       </c>
-      <c r="B37" s="109"/>
-      <c r="C37" s="109"/>
-      <c r="D37" s="109"/>
+      <c r="B37" s="161"/>
+      <c r="C37" s="161"/>
+      <c r="D37" s="161"/>
     </row>
     <row r="38" spans="1:4" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A38" s="112" t="s">
+      <c r="A38" s="162" t="s">
         <v>68</v>
       </c>
-      <c r="B38" s="109"/>
-      <c r="C38" s="109"/>
-      <c r="D38" s="109"/>
+      <c r="B38" s="161"/>
+      <c r="C38" s="161"/>
+      <c r="D38" s="161"/>
     </row>
     <row r="39" spans="1:4" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A39" s="112" t="s">
+      <c r="A39" s="162" t="s">
         <v>69</v>
       </c>
-      <c r="B39" s="109"/>
-      <c r="C39" s="109"/>
-      <c r="D39" s="109"/>
+      <c r="B39" s="161"/>
+      <c r="C39" s="161"/>
+      <c r="D39" s="161"/>
     </row>
     <row r="40" spans="1:4" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A40" s="112" t="s">
+      <c r="A40" s="162" t="s">
         <v>70</v>
       </c>
-      <c r="B40" s="109"/>
-      <c r="C40" s="109"/>
-      <c r="D40" s="109"/>
+      <c r="B40" s="161"/>
+      <c r="C40" s="161"/>
+      <c r="D40" s="161"/>
     </row>
     <row r="41" spans="1:4" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A41" s="112" t="s">
+      <c r="A41" s="162" t="s">
         <v>71</v>
       </c>
-      <c r="B41" s="109"/>
-      <c r="C41" s="109"/>
-      <c r="D41" s="109"/>
+      <c r="B41" s="161"/>
+      <c r="C41" s="161"/>
+      <c r="D41" s="161"/>
     </row>
     <row r="42" spans="1:4" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A42" s="112" t="s">
+      <c r="A42" s="162" t="s">
         <v>72</v>
       </c>
-      <c r="B42" s="109"/>
-      <c r="C42" s="109"/>
-      <c r="D42" s="109"/>
+      <c r="B42" s="161"/>
+      <c r="C42" s="161"/>
+      <c r="D42" s="161"/>
     </row>
     <row r="43" spans="1:4" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A43" s="112" t="s">
+      <c r="A43" s="162" t="s">
         <v>73</v>
       </c>
-      <c r="B43" s="109"/>
-      <c r="C43" s="109"/>
-      <c r="D43" s="109"/>
+      <c r="B43" s="161"/>
+      <c r="C43" s="161"/>
+      <c r="D43" s="161"/>
     </row>
     <row r="44" spans="1:4" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A44" s="112"/>
-      <c r="B44" s="109"/>
-      <c r="C44" s="109"/>
-      <c r="D44" s="109"/>
+      <c r="A44" s="162"/>
+      <c r="B44" s="161"/>
+      <c r="C44" s="161"/>
+      <c r="D44" s="161"/>
     </row>
     <row r="45" spans="1:4" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A45" s="114" t="s">
+      <c r="A45" s="160" t="s">
         <v>74</v>
       </c>
-      <c r="B45" s="109"/>
-      <c r="C45" s="109"/>
-      <c r="D45" s="109"/>
+      <c r="B45" s="161"/>
+      <c r="C45" s="161"/>
+      <c r="D45" s="161"/>
     </row>
     <row r="46" spans="1:4" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A46" s="112" t="s">
+      <c r="A46" s="162" t="s">
         <v>75</v>
       </c>
-      <c r="B46" s="109"/>
-      <c r="C46" s="109"/>
-      <c r="D46" s="109"/>
+      <c r="B46" s="161"/>
+      <c r="C46" s="161"/>
+      <c r="D46" s="161"/>
     </row>
     <row r="47" spans="1:4" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A47" s="112" t="s">
+      <c r="A47" s="162" t="s">
         <v>76</v>
       </c>
-      <c r="B47" s="109"/>
-      <c r="C47" s="109"/>
-      <c r="D47" s="109"/>
+      <c r="B47" s="161"/>
+      <c r="C47" s="161"/>
+      <c r="D47" s="161"/>
     </row>
     <row r="48" spans="1:4" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A48" s="112" t="s">
+      <c r="A48" s="162" t="s">
         <v>77</v>
       </c>
-      <c r="B48" s="109"/>
-      <c r="C48" s="109"/>
-      <c r="D48" s="109"/>
+      <c r="B48" s="161"/>
+      <c r="C48" s="161"/>
+      <c r="D48" s="161"/>
     </row>
     <row r="49" spans="1:4" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A49" s="112" t="s">
+      <c r="A49" s="162" t="s">
         <v>78</v>
       </c>
-      <c r="B49" s="109"/>
-      <c r="C49" s="109"/>
-      <c r="D49" s="109"/>
+      <c r="B49" s="161"/>
+      <c r="C49" s="161"/>
+      <c r="D49" s="161"/>
     </row>
     <row r="50" spans="1:4" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A50" s="112" t="s">
+      <c r="A50" s="162" t="s">
         <v>79</v>
       </c>
-      <c r="B50" s="109"/>
-      <c r="C50" s="109"/>
-      <c r="D50" s="109"/>
+      <c r="B50" s="161"/>
+      <c r="C50" s="161"/>
+      <c r="D50" s="161"/>
     </row>
     <row r="51" spans="1:4" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A51" s="112" t="s">
+      <c r="A51" s="162" t="s">
         <v>80</v>
       </c>
-      <c r="B51" s="109"/>
-      <c r="C51" s="109"/>
-      <c r="D51" s="109"/>
+      <c r="B51" s="161"/>
+      <c r="C51" s="161"/>
+      <c r="D51" s="161"/>
     </row>
     <row r="52" spans="1:4" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A52" s="112"/>
-      <c r="B52" s="109"/>
-      <c r="C52" s="109"/>
-      <c r="D52" s="109"/>
+      <c r="A52" s="162"/>
+      <c r="B52" s="161"/>
+      <c r="C52" s="161"/>
+      <c r="D52" s="161"/>
     </row>
     <row r="53" spans="1:4" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A53" s="114" t="s">
+      <c r="A53" s="160" t="s">
         <v>81</v>
       </c>
-      <c r="B53" s="109"/>
-      <c r="C53" s="109"/>
-      <c r="D53" s="109"/>
+      <c r="B53" s="161"/>
+      <c r="C53" s="161"/>
+      <c r="D53" s="161"/>
     </row>
     <row r="54" spans="1:4" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A54" s="112" t="s">
+      <c r="A54" s="162" t="s">
         <v>82</v>
       </c>
-      <c r="B54" s="109"/>
-      <c r="C54" s="109"/>
-      <c r="D54" s="109"/>
+      <c r="B54" s="161"/>
+      <c r="C54" s="161"/>
+      <c r="D54" s="161"/>
     </row>
     <row r="55" spans="1:4" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A55" s="112" t="s">
+      <c r="A55" s="162" t="s">
         <v>83</v>
       </c>
-      <c r="B55" s="109"/>
-      <c r="C55" s="109"/>
-      <c r="D55" s="109"/>
+      <c r="B55" s="161"/>
+      <c r="C55" s="161"/>
+      <c r="D55" s="161"/>
     </row>
     <row r="56" spans="1:4" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A56" s="112" t="s">
+      <c r="A56" s="162" t="s">
         <v>84</v>
       </c>
-      <c r="B56" s="109"/>
-      <c r="C56" s="109"/>
-      <c r="D56" s="109"/>
+      <c r="B56" s="161"/>
+      <c r="C56" s="161"/>
+      <c r="D56" s="161"/>
     </row>
     <row r="57" spans="1:4" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A57" s="112" t="s">
+      <c r="A57" s="162" t="s">
         <v>85</v>
       </c>
-      <c r="B57" s="109"/>
-      <c r="C57" s="109"/>
-      <c r="D57" s="109"/>
+      <c r="B57" s="161"/>
+      <c r="C57" s="161"/>
+      <c r="D57" s="161"/>
     </row>
     <row r="58" spans="1:4" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A58" s="112"/>
-      <c r="B58" s="109"/>
-      <c r="C58" s="109"/>
-      <c r="D58" s="109"/>
+      <c r="A58" s="162"/>
+      <c r="B58" s="161"/>
+      <c r="C58" s="161"/>
+      <c r="D58" s="161"/>
     </row>
     <row r="59" spans="1:4" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A59" s="114" t="s">
+      <c r="A59" s="160" t="s">
         <v>86</v>
       </c>
-      <c r="B59" s="109"/>
-      <c r="C59" s="109"/>
-      <c r="D59" s="109"/>
+      <c r="B59" s="161"/>
+      <c r="C59" s="161"/>
+      <c r="D59" s="161"/>
     </row>
     <row r="60" spans="1:4" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A60" s="112" t="s">
+      <c r="A60" s="162" t="s">
         <v>87</v>
       </c>
-      <c r="B60" s="109"/>
-      <c r="C60" s="109"/>
-      <c r="D60" s="109"/>
+      <c r="B60" s="161"/>
+      <c r="C60" s="161"/>
+      <c r="D60" s="161"/>
     </row>
     <row r="61" spans="1:4" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A61" s="112" t="s">
+      <c r="A61" s="162" t="s">
         <v>88</v>
       </c>
-      <c r="B61" s="109"/>
-      <c r="C61" s="109"/>
-      <c r="D61" s="109"/>
+      <c r="B61" s="161"/>
+      <c r="C61" s="161"/>
+      <c r="D61" s="161"/>
     </row>
     <row r="62" spans="1:4" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A62" s="112" t="s">
+      <c r="A62" s="162" t="s">
         <v>89</v>
       </c>
-      <c r="B62" s="109"/>
-      <c r="C62" s="109"/>
-      <c r="D62" s="109"/>
+      <c r="B62" s="161"/>
+      <c r="C62" s="161"/>
+      <c r="D62" s="161"/>
     </row>
     <row r="63" spans="1:4" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A63" s="112" t="s">
+      <c r="A63" s="162" t="s">
         <v>90</v>
       </c>
-      <c r="B63" s="109"/>
-      <c r="C63" s="109"/>
-      <c r="D63" s="109"/>
+      <c r="B63" s="161"/>
+      <c r="C63" s="161"/>
+      <c r="D63" s="161"/>
     </row>
     <row r="64" spans="1:4" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A64" s="112" t="s">
+      <c r="A64" s="162" t="s">
         <v>91</v>
       </c>
-      <c r="B64" s="109"/>
-      <c r="C64" s="109"/>
-      <c r="D64" s="109"/>
+      <c r="B64" s="161"/>
+      <c r="C64" s="161"/>
+      <c r="D64" s="161"/>
     </row>
     <row r="65" spans="1:4" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A65" s="112" t="s">
+      <c r="A65" s="162" t="s">
         <v>92</v>
       </c>
-      <c r="B65" s="109"/>
-      <c r="C65" s="109"/>
-      <c r="D65" s="109"/>
+      <c r="B65" s="161"/>
+      <c r="C65" s="161"/>
+      <c r="D65" s="161"/>
     </row>
     <row r="66" spans="1:4" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A66" s="112" t="s">
+      <c r="A66" s="162" t="s">
         <v>93</v>
       </c>
-      <c r="B66" s="109"/>
-      <c r="C66" s="109"/>
-      <c r="D66" s="109"/>
+      <c r="B66" s="161"/>
+      <c r="C66" s="161"/>
+      <c r="D66" s="161"/>
     </row>
     <row r="67" spans="1:4" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A67" s="112"/>
-      <c r="B67" s="109"/>
-      <c r="C67" s="109"/>
-      <c r="D67" s="109"/>
+      <c r="A67" s="162"/>
+      <c r="B67" s="161"/>
+      <c r="C67" s="161"/>
+      <c r="D67" s="161"/>
     </row>
     <row r="68" spans="1:4" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A68" s="114" t="s">
+      <c r="A68" s="160" t="s">
         <v>94</v>
       </c>
-      <c r="B68" s="109"/>
-      <c r="C68" s="109"/>
-      <c r="D68" s="109"/>
+      <c r="B68" s="161"/>
+      <c r="C68" s="161"/>
+      <c r="D68" s="161"/>
     </row>
     <row r="69" spans="1:4" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A69" s="112" t="s">
+      <c r="A69" s="162" t="s">
         <v>95</v>
       </c>
-      <c r="B69" s="109"/>
-      <c r="C69" s="109"/>
-      <c r="D69" s="109"/>
+      <c r="B69" s="161"/>
+      <c r="C69" s="161"/>
+      <c r="D69" s="161"/>
     </row>
     <row r="70" spans="1:4" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A70" s="112" t="s">
+      <c r="A70" s="162" t="s">
         <v>96</v>
       </c>
-      <c r="B70" s="109"/>
-      <c r="C70" s="109"/>
-      <c r="D70" s="109"/>
+      <c r="B70" s="161"/>
+      <c r="C70" s="161"/>
+      <c r="D70" s="161"/>
     </row>
     <row r="71" spans="1:4" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A71" s="112" t="s">
+      <c r="A71" s="162" t="s">
         <v>97</v>
       </c>
-      <c r="B71" s="109"/>
-      <c r="C71" s="109"/>
-      <c r="D71" s="109"/>
+      <c r="B71" s="161"/>
+      <c r="C71" s="161"/>
+      <c r="D71" s="161"/>
     </row>
     <row r="72" spans="1:4" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A72" s="112" t="s">
+      <c r="A72" s="162" t="s">
         <v>98</v>
       </c>
-      <c r="B72" s="109"/>
-      <c r="C72" s="109"/>
-      <c r="D72" s="109"/>
+      <c r="B72" s="161"/>
+      <c r="C72" s="161"/>
+      <c r="D72" s="161"/>
     </row>
     <row r="73" spans="1:4" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A73" s="112" t="s">
+      <c r="A73" s="162" t="s">
         <v>99</v>
       </c>
-      <c r="B73" s="109"/>
-      <c r="C73" s="109"/>
-      <c r="D73" s="109"/>
+      <c r="B73" s="161"/>
+      <c r="C73" s="161"/>
+      <c r="D73" s="161"/>
     </row>
     <row r="74" spans="1:4" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A74" s="112" t="s">
+      <c r="A74" s="162" t="s">
         <v>100</v>
       </c>
-      <c r="B74" s="109"/>
-      <c r="C74" s="109"/>
-      <c r="D74" s="109"/>
+      <c r="B74" s="161"/>
+      <c r="C74" s="161"/>
+      <c r="D74" s="161"/>
     </row>
   </sheetData>
   <mergeCells count="49">
@@ -11518,8 +11568,6 @@
     <mergeCell ref="A49:D49"/>
     <mergeCell ref="A51:D51"/>
     <mergeCell ref="A60:D60"/>
-    <mergeCell ref="A36:D36"/>
-    <mergeCell ref="A52:D52"/>
     <mergeCell ref="A1:D1"/>
     <mergeCell ref="A45:D45"/>
     <mergeCell ref="A70:D70"/>
@@ -11534,23 +11582,25 @@
     <mergeCell ref="A37:D37"/>
     <mergeCell ref="A56:D56"/>
     <mergeCell ref="A3:D4"/>
-    <mergeCell ref="A64:D64"/>
-    <mergeCell ref="A43:D43"/>
     <mergeCell ref="A19:D19"/>
     <mergeCell ref="A63:D63"/>
     <mergeCell ref="A28:D28"/>
+    <mergeCell ref="A34:D34"/>
+    <mergeCell ref="A39:D39"/>
+    <mergeCell ref="A35:D35"/>
+    <mergeCell ref="A38:D38"/>
+    <mergeCell ref="A36:D36"/>
+    <mergeCell ref="A52:D52"/>
     <mergeCell ref="A68:D68"/>
     <mergeCell ref="A44:D44"/>
     <mergeCell ref="A40:D40"/>
     <mergeCell ref="A67:D67"/>
     <mergeCell ref="A58:D58"/>
-    <mergeCell ref="A34:D34"/>
     <mergeCell ref="A48:D48"/>
-    <mergeCell ref="A39:D39"/>
     <mergeCell ref="A53:D53"/>
-    <mergeCell ref="A35:D35"/>
     <mergeCell ref="A62:D62"/>
-    <mergeCell ref="A38:D38"/>
+    <mergeCell ref="A64:D64"/>
+    <mergeCell ref="A43:D43"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -12116,42 +12166,42 @@
       <c r="J39" s="35"/>
     </row>
     <row r="41" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A41" s="111" t="s">
+      <c r="A41" s="168" t="s">
         <v>131</v>
       </c>
-      <c r="B41" s="109"/>
-      <c r="C41" s="109"/>
-      <c r="D41" s="109"/>
-      <c r="E41" s="109"/>
-      <c r="F41" s="109"/>
-      <c r="G41" s="109"/>
-      <c r="H41" s="109"/>
-      <c r="I41" s="109"/>
-      <c r="J41" s="109"/>
+      <c r="B41" s="161"/>
+      <c r="C41" s="161"/>
+      <c r="D41" s="161"/>
+      <c r="E41" s="161"/>
+      <c r="F41" s="161"/>
+      <c r="G41" s="161"/>
+      <c r="H41" s="161"/>
+      <c r="I41" s="161"/>
+      <c r="J41" s="161"/>
     </row>
     <row r="42" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A42" s="109"/>
-      <c r="B42" s="109"/>
-      <c r="C42" s="109"/>
-      <c r="D42" s="109"/>
-      <c r="E42" s="109"/>
-      <c r="F42" s="109"/>
-      <c r="G42" s="109"/>
-      <c r="H42" s="109"/>
-      <c r="I42" s="109"/>
-      <c r="J42" s="109"/>
+      <c r="A42" s="161"/>
+      <c r="B42" s="161"/>
+      <c r="C42" s="161"/>
+      <c r="D42" s="161"/>
+      <c r="E42" s="161"/>
+      <c r="F42" s="161"/>
+      <c r="G42" s="161"/>
+      <c r="H42" s="161"/>
+      <c r="I42" s="161"/>
+      <c r="J42" s="161"/>
     </row>
     <row r="43" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A43" s="109"/>
-      <c r="B43" s="109"/>
-      <c r="C43" s="109"/>
-      <c r="D43" s="109"/>
-      <c r="E43" s="109"/>
-      <c r="F43" s="109"/>
-      <c r="G43" s="109"/>
-      <c r="H43" s="109"/>
-      <c r="I43" s="109"/>
-      <c r="J43" s="109"/>
+      <c r="A43" s="161"/>
+      <c r="B43" s="161"/>
+      <c r="C43" s="161"/>
+      <c r="D43" s="161"/>
+      <c r="E43" s="161"/>
+      <c r="F43" s="161"/>
+      <c r="G43" s="161"/>
+      <c r="H43" s="161"/>
+      <c r="I43" s="161"/>
+      <c r="J43" s="161"/>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -12447,24 +12497,24 @@
       <c r="G24" s="35"/>
     </row>
     <row r="26" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A26" s="111" t="s">
+      <c r="A26" s="168" t="s">
         <v>148</v>
       </c>
-      <c r="B26" s="109"/>
-      <c r="C26" s="109"/>
-      <c r="D26" s="109"/>
-      <c r="E26" s="109"/>
-      <c r="F26" s="109"/>
-      <c r="G26" s="109"/>
+      <c r="B26" s="161"/>
+      <c r="C26" s="161"/>
+      <c r="D26" s="161"/>
+      <c r="E26" s="161"/>
+      <c r="F26" s="161"/>
+      <c r="G26" s="161"/>
     </row>
     <row r="27" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A27" s="109"/>
-      <c r="B27" s="109"/>
-      <c r="C27" s="109"/>
-      <c r="D27" s="109"/>
-      <c r="E27" s="109"/>
-      <c r="F27" s="109"/>
-      <c r="G27" s="109"/>
+      <c r="A27" s="161"/>
+      <c r="B27" s="161"/>
+      <c r="C27" s="161"/>
+      <c r="D27" s="161"/>
+      <c r="E27" s="161"/>
+      <c r="F27" s="161"/>
+      <c r="G27" s="161"/>
     </row>
   </sheetData>
   <mergeCells count="1">

</xml_diff>

<commit_message>
content(holomap): gabarit de carte mis à jour (retrait des spots par l'auteur)
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Carte Holo/carte_holomap.xlsx
+++ b/Carte Holo/carte_holomap.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\b.consol\Downloads\Divers\ecole\Dossier UE9\IdleEvolution\Carte Holo\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Projets\IdleEvolution\Carte Holo\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{75579294-7778-4076-90C2-020B8CF5B36F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FE8F05C0-D73A-45E5-B48F-68DF6116C6DA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Paramètres" sheetId="1" r:id="rId1"/>
@@ -2081,26 +2081,26 @@
     <xf numFmtId="0" fontId="0" fillId="5" borderId="4" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="9" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="27" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -2417,7 +2417,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="A1" s="176" t="s">
+      <c r="A1" s="174" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="175"/>
@@ -2479,7 +2479,7 @@
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A9" s="177" t="s">
+      <c r="A9" s="176" t="s">
         <v>13</v>
       </c>
       <c r="B9" s="175"/>
@@ -6648,7 +6648,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:4" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="A1" s="176" t="s">
+      <c r="A1" s="174" t="s">
         <v>42</v>
       </c>
       <c r="B1" s="175"/>
@@ -6690,7 +6690,7 @@
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A8" s="182" t="s">
+      <c r="A8" s="179" t="s">
         <v>46</v>
       </c>
       <c r="B8" s="175"/>
@@ -6854,7 +6854,7 @@
       </c>
     </row>
     <row r="22" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A22" s="183" t="s">
+      <c r="A22" s="182" t="s">
         <v>74</v>
       </c>
       <c r="B22" s="175"/>
@@ -6862,7 +6862,7 @@
       <c r="D22" s="175"/>
     </row>
     <row r="24" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A24" s="182" t="s">
+      <c r="A24" s="179" t="s">
         <v>75</v>
       </c>
       <c r="B24" s="175"/>
@@ -6907,7 +6907,7 @@
       <c r="D28" s="175"/>
     </row>
     <row r="30" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A30" s="182" t="s">
+      <c r="A30" s="179" t="s">
         <v>83</v>
       </c>
       <c r="B30" s="175"/>
@@ -7018,7 +7018,7 @@
       <c r="D48" s="175"/>
     </row>
     <row r="52" spans="1:4" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A52" s="179" t="s">
+      <c r="A52" s="177" t="s">
         <v>90</v>
       </c>
       <c r="B52" s="175"/>
@@ -7120,7 +7120,7 @@
       <c r="D64" s="175"/>
     </row>
     <row r="65" spans="1:4" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A65" s="179" t="s">
+      <c r="A65" s="177" t="s">
         <v>102</v>
       </c>
       <c r="B65" s="175"/>
@@ -7182,7 +7182,7 @@
       <c r="D72" s="175"/>
     </row>
     <row r="73" spans="1:4" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A73" s="179" t="s">
+      <c r="A73" s="177" t="s">
         <v>109</v>
       </c>
       <c r="B73" s="175"/>
@@ -7236,7 +7236,7 @@
       <c r="D79" s="175"/>
     </row>
     <row r="80" spans="1:4" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A80" s="179" t="s">
+      <c r="A80" s="177" t="s">
         <v>115</v>
       </c>
       <c r="B80" s="175"/>
@@ -7306,7 +7306,7 @@
       <c r="D88" s="175"/>
     </row>
     <row r="89" spans="1:4" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A89" s="179" t="s">
+      <c r="A89" s="177" t="s">
         <v>123</v>
       </c>
       <c r="B89" s="175"/>
@@ -7363,31 +7363,17 @@
     </row>
   </sheetData>
   <mergeCells count="52">
-    <mergeCell ref="A52:D52"/>
-    <mergeCell ref="A81:D81"/>
-    <mergeCell ref="A63:D63"/>
-    <mergeCell ref="A24:D24"/>
-    <mergeCell ref="A89:D89"/>
-    <mergeCell ref="A74:D74"/>
-    <mergeCell ref="A30:D30"/>
-    <mergeCell ref="A64:D64"/>
-    <mergeCell ref="A59:D59"/>
-    <mergeCell ref="A82:D82"/>
-    <mergeCell ref="A60:D60"/>
-    <mergeCell ref="A75:D75"/>
-    <mergeCell ref="A56:D56"/>
-    <mergeCell ref="A1:D1"/>
-    <mergeCell ref="A47:D48"/>
-    <mergeCell ref="A54:D54"/>
-    <mergeCell ref="A3:D5"/>
-    <mergeCell ref="A55:D55"/>
-    <mergeCell ref="A57:D57"/>
-    <mergeCell ref="A27:D28"/>
-    <mergeCell ref="A58:D58"/>
-    <mergeCell ref="A8:D8"/>
-    <mergeCell ref="A22:D22"/>
-    <mergeCell ref="A53:D53"/>
-    <mergeCell ref="A62:D62"/>
+    <mergeCell ref="A95:D95"/>
+    <mergeCell ref="A71:D71"/>
+    <mergeCell ref="A85:D85"/>
+    <mergeCell ref="A76:D76"/>
+    <mergeCell ref="A93:D93"/>
+    <mergeCell ref="A77:D77"/>
+    <mergeCell ref="A83:D83"/>
+    <mergeCell ref="A92:D92"/>
+    <mergeCell ref="A94:D94"/>
+    <mergeCell ref="A90:D90"/>
+    <mergeCell ref="A91:D91"/>
     <mergeCell ref="A72:D72"/>
     <mergeCell ref="A70:D70"/>
     <mergeCell ref="A79:D79"/>
@@ -7404,17 +7390,31 @@
     <mergeCell ref="A68:D68"/>
     <mergeCell ref="A67:D67"/>
     <mergeCell ref="A73:D73"/>
-    <mergeCell ref="A95:D95"/>
-    <mergeCell ref="A71:D71"/>
-    <mergeCell ref="A85:D85"/>
-    <mergeCell ref="A76:D76"/>
-    <mergeCell ref="A93:D93"/>
-    <mergeCell ref="A77:D77"/>
-    <mergeCell ref="A83:D83"/>
-    <mergeCell ref="A92:D92"/>
-    <mergeCell ref="A94:D94"/>
-    <mergeCell ref="A90:D90"/>
-    <mergeCell ref="A91:D91"/>
+    <mergeCell ref="A1:D1"/>
+    <mergeCell ref="A47:D48"/>
+    <mergeCell ref="A54:D54"/>
+    <mergeCell ref="A3:D5"/>
+    <mergeCell ref="A55:D55"/>
+    <mergeCell ref="A27:D28"/>
+    <mergeCell ref="A8:D8"/>
+    <mergeCell ref="A22:D22"/>
+    <mergeCell ref="A53:D53"/>
+    <mergeCell ref="A52:D52"/>
+    <mergeCell ref="A81:D81"/>
+    <mergeCell ref="A63:D63"/>
+    <mergeCell ref="A24:D24"/>
+    <mergeCell ref="A89:D89"/>
+    <mergeCell ref="A74:D74"/>
+    <mergeCell ref="A30:D30"/>
+    <mergeCell ref="A64:D64"/>
+    <mergeCell ref="A59:D59"/>
+    <mergeCell ref="A82:D82"/>
+    <mergeCell ref="A60:D60"/>
+    <mergeCell ref="A75:D75"/>
+    <mergeCell ref="A56:D56"/>
+    <mergeCell ref="A57:D57"/>
+    <mergeCell ref="A58:D58"/>
+    <mergeCell ref="A62:D62"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -10925,17 +10925,13 @@
       <c r="AU52" s="8"/>
       <c r="AV52" s="8"/>
       <c r="AW52" s="8"/>
-      <c r="AX52" s="173">
-        <v>1</v>
-      </c>
+      <c r="AX52" s="8"/>
       <c r="AY52" s="8"/>
       <c r="AZ52" s="8"/>
       <c r="BA52" s="8"/>
       <c r="BB52" s="8"/>
       <c r="BC52" s="8"/>
-      <c r="BD52" s="15">
-        <v>1</v>
-      </c>
+      <c r="BD52" s="8"/>
       <c r="BE52" s="8"/>
       <c r="BF52" s="8"/>
       <c r="BG52" s="8"/>
@@ -11254,17 +11250,13 @@
       <c r="AU57" s="8"/>
       <c r="AV57" s="8"/>
       <c r="AW57" s="8"/>
-      <c r="AX57" s="15">
-        <v>1</v>
-      </c>
+      <c r="AX57" s="8"/>
       <c r="AY57" s="8"/>
       <c r="AZ57" s="8"/>
       <c r="BA57" s="8"/>
       <c r="BB57" s="8"/>
       <c r="BC57" s="8"/>
-      <c r="BD57" s="15">
-        <v>1</v>
-      </c>
+      <c r="BD57" s="8"/>
       <c r="BE57" s="8"/>
       <c r="BF57" s="8"/>
       <c r="BG57" s="8"/>
@@ -11532,7 +11524,7 @@
       <c r="BI61" s="8"/>
     </row>
     <row r="63" spans="1:61" x14ac:dyDescent="0.25">
-      <c r="A63" s="174" t="s">
+      <c r="A63" s="183" t="s">
         <v>15</v>
       </c>
       <c r="B63" s="175"/>
@@ -11631,7 +11623,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:4" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="A1" s="176" t="s">
+      <c r="A1" s="174" t="s">
         <v>16</v>
       </c>
       <c r="B1" s="175"/>
@@ -11761,7 +11753,7 @@
       </c>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A14" s="174" t="s">
+      <c r="A14" s="183" t="s">
         <v>41</v>
       </c>
       <c r="B14" s="175"/>
@@ -12058,7 +12050,7 @@
       <c r="G24" s="34"/>
     </row>
     <row r="26" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A26" s="174" t="s">
+      <c r="A26" s="183" t="s">
         <v>147</v>
       </c>
       <c r="B26" s="175"/>

</xml_diff>

<commit_message>
feat(holomap): tailles minimales DURES des apparences (croix rouge)
Un bloc d'apparence specifique peint sous sa taille min (feuille
« Contraintes tailles » du gabarit / _TAILLES_MIN) n'est plus rendu :
_valider_tailles_min le retire de sa famille et pose une croix rouge
au centre de la zone (convention universelle, comme le Surelevé).
Formes dures en plus : prison rectangulaire PLEINE obligatoire (fin
des miradors flottants), stade ratio max 3:2. Les autres conseils de
forme restent souples. Carte reelle conforme (0 croix), snapshot
inchangé.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Carte Holo/carte_holomap.xlsx
+++ b/Carte Holo/carte_holomap.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Projets\IdleEvolution\Carte Holo\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AFC39C11-4481-45C6-87BD-F549FAAB1160}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9ACAEED3-5A76-4511-BF7D-C8D8030C8471}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-105" yWindow="0" windowWidth="14610" windowHeight="15585" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Paramètres" sheetId="1" r:id="rId1"/>
@@ -18,14 +18,28 @@
     <sheet name="Légende" sheetId="5" r:id="rId3"/>
     <sheet name="Surélevé" sheetId="3" r:id="rId4"/>
     <sheet name="Légende Surélevé" sheetId="4" r:id="rId5"/>
-    <sheet name="Ouvrages d'art" sheetId="6" r:id="rId6"/>
+    <sheet name="Contraintes tailles" sheetId="7" r:id="rId6"/>
+    <sheet name="Ouvrages d'art" sheetId="6" r:id="rId7"/>
   </sheets>
-  <calcPr calcId="162913"/>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="187" uniqueCount="161">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="243" uniqueCount="201">
   <si>
     <t>Paramètres globaux — HoloMap</t>
   </si>
@@ -508,6 +522,126 @@
   </si>
   <si>
     <t>Institution culturelle : façade monumentale, colonnades/verrière, hologrammes d'exposition, éclairage soigné (motif libre).</t>
+  </si>
+  <si>
+    <t>Bâtiment requis dessous, toit forcé plat. Croix rouge si pas de bâtiment (déjà codé).</t>
+  </si>
+  <si>
+    <t>Carré obligatoire</t>
+  </si>
+  <si>
+    <t>4×4</t>
+  </si>
+  <si>
+    <t>Héliport (Surélevé)</t>
+  </si>
+  <si>
+    <t>Colonnade 8 colonnes + fronton (L ≥ 4), 3 marches (P ≥ 4), parvis (P ≥ 4), verrière en berceau 5 arches, hologrammes.</t>
+  </si>
+  <si>
+    <t>Plus large que profond conseillé</t>
+  </si>
+  <si>
+    <t>Amphi-dôme (illisible &lt; 4), esplanade (P ≥ 4), corps + 2 ailes + colonnade 8 colonnes (L ≥ 4), panneaux.</t>
+  </si>
+  <si>
+    <t>Plus large que profond conseillé (5×4)</t>
+  </si>
+  <si>
+    <t>Bassin central (seuil ≥ 3), kiosques-dômes (seuil ≥ 4), arbres sur cases intérieures (≥ 3/axe), allées en croix.</t>
+  </si>
+  <si>
+    <t>Aucune stricte (≤ 2:1 conseillé)</t>
+  </si>
+  <si>
+    <t>Portique d'entrée + écusson, bandeau bleu, antenne haubanée au coin de toit, gyrophares près de l'entrée.</t>
+  </si>
+  <si>
+    <t>Aucune</t>
+  </si>
+  <si>
+    <t>2×2</t>
+  </si>
+  <si>
+    <t>Commissariat</t>
+  </si>
+  <si>
+    <t>4 miradors d'angle + faisceaux, enceinte crénelée, champ de force sur la cour, portail. Non-rectangulaire → miradors flottants.</t>
+  </si>
+  <si>
+    <t>RECTANGULAIRE OBLIGATOIRE (croix rouge si en L)</t>
+  </si>
+  <si>
+    <t>3×3</t>
+  </si>
+  <si>
+    <t>Chapelle centrale (seuil codé ≥ 4 cases), 2 stèles/case, mur d'enceinte + portail, cyprès.</t>
+  </si>
+  <si>
+    <t>Aucune (formes en L acceptées)</t>
+  </si>
+  <si>
+    <t>Losange d'infield (bases lisibles ≥ 4×4), clôture elliptique, tribunes en fer à cheval, projecteurs, tableau.</t>
+  </si>
+  <si>
+    <t>Proche du carré (ratio ≤ ~3:2)</t>
+  </si>
+  <si>
+    <t>Stade / arène</t>
+  </si>
+  <si>
+    <t>Billboard de toit (déborde à 1×1), marquee périmétrique, verrières, atrium d'entrée, totem sur route.</t>
+  </si>
+  <si>
+    <t>Léger allongement conseillé (2×3)</t>
+  </si>
+  <si>
+    <t>Grue à aimant (seuil codé ≥ 6 cases), 2ᵉ grue ≥ 10 ; murs de carcasses en frontière ; épaves intérieures dès 3×3.</t>
+  </si>
+  <si>
+    <t>≥ 3 sur un axe (allées intérieures)</t>
+  </si>
+  <si>
+    <t>2×3</t>
+  </si>
+  <si>
+    <t>Casse auto</t>
+  </si>
+  <si>
+    <t>3 cheminées réparties sur le grand axe + dents de scie (min 2) ; cheminées à 28 % du petit axe → largeur ≥ 2.</t>
+  </si>
+  <si>
+    <t>Allongée (grand axe ≥ 2× petit)</t>
+  </si>
+  <si>
+    <t>2×4</t>
+  </si>
+  <si>
+    <t>Usine désaffectée</t>
+  </si>
+  <si>
+    <t>Attributs déterminants</t>
+  </si>
+  <si>
+    <t>Contrainte de forme</t>
+  </si>
+  <si>
+    <t>Taille min</t>
+  </si>
+  <si>
+    <t>Apparence</t>
+  </si>
+  <si>
+    <t>Sous la taille min OU forme non respectée → CROIX ROUGE (contrainte dure). Échelle : 1 case = 10 m. L×P = Largeur×Profondeur.</t>
+  </si>
+  <si>
+    <t>Contraintes de taille/forme minimales par apparence</t>
+  </si>
+  <si>
+    <t>Casse / épaves de voitures empilées (motif libre).</t>
+  </si>
+  <si>
+    <t>Bâtiment industriel à l'abandon, métal corrodé (motif libre).</t>
   </si>
 </sst>
 </file>
@@ -1804,7 +1938,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="211">
+  <cellXfs count="210">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -1994,13 +2128,34 @@
     <xf numFmtId="0" fontId="0" fillId="28" borderId="41" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="28" borderId="42" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="28" borderId="43" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="29" borderId="5" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="29" borderId="2" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="30" borderId="2" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="31" borderId="2" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="31" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="31" borderId="30" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="31" borderId="31" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="31" borderId="32" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="31" borderId="33" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="31" borderId="34" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="31" borderId="41" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="31" borderId="42" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="31" borderId="43" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="30" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="30" borderId="30" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="30" borderId="31" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="30" borderId="32" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="30" borderId="33" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="30" borderId="34" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="30" borderId="41" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="30" borderId="42" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="30" borderId="43" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
@@ -2010,40 +2165,20 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="29" borderId="5" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="2" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="2" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="16" borderId="2" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="29" borderId="2" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="30" borderId="2" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="31" borderId="2" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="31" borderId="0" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="31" borderId="30" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="31" borderId="31" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="31" borderId="32" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="31" borderId="33" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="31" borderId="34" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="31" borderId="41" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="31" borderId="42" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="31" borderId="43" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="30" borderId="0" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="30" borderId="30" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="30" borderId="31" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="30" borderId="32" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="30" borderId="33" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="30" borderId="34" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="30" borderId="41" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="30" borderId="42" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="30" borderId="43" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="21" borderId="2" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="20" borderId="2" xfId="0" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -2360,11 +2495,11 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="A1" s="173" t="s">
+      <c r="A1" s="195" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="174"/>
-      <c r="C1" s="174"/>
+      <c r="B1" s="196"/>
+      <c r="C1" s="196"/>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
@@ -2422,11 +2557,11 @@
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A9" s="175" t="s">
+      <c r="A9" s="197" t="s">
         <v>13</v>
       </c>
-      <c r="B9" s="174"/>
-      <c r="C9" s="174"/>
+      <c r="B9" s="196"/>
+      <c r="C9" s="196"/>
     </row>
   </sheetData>
   <mergeCells count="2">
@@ -3239,9 +3374,9 @@
       <c r="Q11" s="7"/>
       <c r="R11" s="7"/>
       <c r="S11" s="7"/>
-      <c r="T11" s="189"/>
-      <c r="U11" s="189"/>
-      <c r="V11" s="189"/>
+      <c r="T11" s="22"/>
+      <c r="U11" s="22"/>
+      <c r="V11" s="22"/>
       <c r="W11" s="163"/>
       <c r="X11" s="35"/>
       <c r="Y11" s="35"/>
@@ -3304,14 +3439,14 @@
       <c r="Q12" s="7"/>
       <c r="R12" s="7"/>
       <c r="S12" s="7"/>
-      <c r="T12" s="189"/>
+      <c r="T12" s="22"/>
       <c r="U12" s="36"/>
-      <c r="V12" s="203"/>
-      <c r="W12" s="204"/>
-      <c r="X12" s="204"/>
-      <c r="Y12" s="204"/>
-      <c r="Z12" s="204"/>
-      <c r="AA12" s="205"/>
+      <c r="V12" s="187"/>
+      <c r="W12" s="188"/>
+      <c r="X12" s="188"/>
+      <c r="Y12" s="188"/>
+      <c r="Z12" s="188"/>
+      <c r="AA12" s="189"/>
       <c r="AB12" s="40"/>
       <c r="AC12" s="36"/>
       <c r="AD12" s="168"/>
@@ -3373,14 +3508,14 @@
       <c r="Q13" s="7"/>
       <c r="R13" s="7"/>
       <c r="S13" s="7"/>
-      <c r="T13" s="189"/>
+      <c r="T13" s="22"/>
       <c r="U13" s="36"/>
-      <c r="V13" s="206"/>
-      <c r="W13" s="202"/>
-      <c r="X13" s="202"/>
-      <c r="Y13" s="202"/>
-      <c r="Z13" s="202"/>
-      <c r="AA13" s="207"/>
+      <c r="V13" s="190"/>
+      <c r="W13" s="186"/>
+      <c r="X13" s="186"/>
+      <c r="Y13" s="186"/>
+      <c r="Z13" s="186"/>
+      <c r="AA13" s="191"/>
       <c r="AB13" s="40"/>
       <c r="AC13" s="36"/>
       <c r="AD13" s="170"/>
@@ -3438,14 +3573,14 @@
       <c r="Q14" s="61"/>
       <c r="R14" s="7"/>
       <c r="S14" s="7"/>
-      <c r="T14" s="189"/>
+      <c r="T14" s="22"/>
       <c r="U14" s="36"/>
-      <c r="V14" s="206"/>
-      <c r="W14" s="202"/>
-      <c r="X14" s="202"/>
-      <c r="Y14" s="202"/>
-      <c r="Z14" s="202"/>
-      <c r="AA14" s="207"/>
+      <c r="V14" s="190"/>
+      <c r="W14" s="186"/>
+      <c r="X14" s="186"/>
+      <c r="Y14" s="186"/>
+      <c r="Z14" s="186"/>
+      <c r="AA14" s="191"/>
       <c r="AB14" s="40"/>
       <c r="AC14" s="7"/>
       <c r="AD14" s="50"/>
@@ -3503,15 +3638,15 @@
       <c r="Q15" s="61"/>
       <c r="R15" s="7"/>
       <c r="S15" s="7"/>
-      <c r="T15" s="189"/>
+      <c r="T15" s="22"/>
       <c r="U15" s="36"/>
-      <c r="V15" s="206"/>
-      <c r="W15" s="202"/>
-      <c r="X15" s="202"/>
-      <c r="Y15" s="202"/>
-      <c r="Z15" s="202"/>
-      <c r="AA15" s="207"/>
-      <c r="AB15" s="187"/>
+      <c r="V15" s="190"/>
+      <c r="W15" s="186"/>
+      <c r="X15" s="186"/>
+      <c r="Y15" s="186"/>
+      <c r="Z15" s="186"/>
+      <c r="AA15" s="191"/>
+      <c r="AB15" s="10"/>
       <c r="AC15" s="10"/>
       <c r="AD15" s="10"/>
       <c r="AE15" s="10"/>
@@ -3570,14 +3705,14 @@
       <c r="Q16" s="61"/>
       <c r="R16" s="7"/>
       <c r="S16" s="7"/>
-      <c r="T16" s="189"/>
+      <c r="T16" s="22"/>
       <c r="U16" s="36"/>
-      <c r="V16" s="208"/>
-      <c r="W16" s="209"/>
-      <c r="X16" s="209"/>
-      <c r="Y16" s="209"/>
-      <c r="Z16" s="209"/>
-      <c r="AA16" s="210"/>
+      <c r="V16" s="192"/>
+      <c r="W16" s="193"/>
+      <c r="X16" s="193"/>
+      <c r="Y16" s="193"/>
+      <c r="Z16" s="193"/>
+      <c r="AA16" s="194"/>
       <c r="AB16" s="40"/>
       <c r="AC16" s="10"/>
       <c r="AD16" s="7"/>
@@ -3636,9 +3771,9 @@
       <c r="R17" s="7"/>
       <c r="S17" s="22"/>
       <c r="T17" s="22"/>
-      <c r="U17" s="186"/>
-      <c r="V17" s="186"/>
-      <c r="W17" s="186"/>
+      <c r="U17" s="7"/>
+      <c r="V17" s="7"/>
+      <c r="W17" s="7"/>
       <c r="X17" s="50"/>
       <c r="Y17" s="50"/>
       <c r="Z17" s="50"/>
@@ -4177,15 +4312,15 @@
       <c r="O25" s="20"/>
       <c r="P25" s="98"/>
       <c r="Q25" s="10"/>
-      <c r="R25" s="190"/>
-      <c r="S25" s="190"/>
-      <c r="T25" s="190"/>
-      <c r="U25" s="190"/>
-      <c r="V25" s="190"/>
-      <c r="W25" s="190"/>
-      <c r="X25" s="190"/>
-      <c r="Y25" s="190"/>
-      <c r="Z25" s="183"/>
+      <c r="R25" s="174"/>
+      <c r="S25" s="174"/>
+      <c r="T25" s="174"/>
+      <c r="U25" s="174"/>
+      <c r="V25" s="174"/>
+      <c r="W25" s="174"/>
+      <c r="X25" s="174"/>
+      <c r="Y25" s="174"/>
+      <c r="Z25" s="173"/>
       <c r="AA25" s="66"/>
       <c r="AB25" s="68"/>
       <c r="AC25" s="78"/>
@@ -4242,15 +4377,15 @@
       <c r="O26" s="61"/>
       <c r="P26" s="61"/>
       <c r="Q26" s="10"/>
-      <c r="R26" s="190"/>
-      <c r="S26" s="190"/>
-      <c r="T26" s="190"/>
-      <c r="U26" s="190"/>
-      <c r="V26" s="190"/>
-      <c r="W26" s="190"/>
-      <c r="X26" s="190"/>
-      <c r="Y26" s="190"/>
-      <c r="Z26" s="183"/>
+      <c r="R26" s="174"/>
+      <c r="S26" s="174"/>
+      <c r="T26" s="174"/>
+      <c r="U26" s="174"/>
+      <c r="V26" s="174"/>
+      <c r="W26" s="174"/>
+      <c r="X26" s="174"/>
+      <c r="Y26" s="174"/>
+      <c r="Z26" s="173"/>
       <c r="AA26" s="79">
         <v>8</v>
       </c>
@@ -4309,15 +4444,15 @@
       <c r="O27" s="67"/>
       <c r="P27" s="68"/>
       <c r="Q27" s="78"/>
-      <c r="R27" s="190"/>
-      <c r="S27" s="190"/>
-      <c r="T27" s="190"/>
-      <c r="U27" s="190"/>
-      <c r="V27" s="190"/>
-      <c r="W27" s="190"/>
-      <c r="X27" s="190"/>
-      <c r="Y27" s="190"/>
-      <c r="Z27" s="190"/>
+      <c r="R27" s="174"/>
+      <c r="S27" s="174"/>
+      <c r="T27" s="174"/>
+      <c r="U27" s="174"/>
+      <c r="V27" s="174"/>
+      <c r="W27" s="174"/>
+      <c r="X27" s="174"/>
+      <c r="Y27" s="174"/>
+      <c r="Z27" s="174"/>
       <c r="AA27" s="85"/>
       <c r="AB27" s="99"/>
       <c r="AC27" s="10"/>
@@ -4376,15 +4511,15 @@
       </c>
       <c r="P28" s="71"/>
       <c r="Q28" s="78"/>
-      <c r="R28" s="190"/>
-      <c r="S28" s="190"/>
-      <c r="T28" s="190"/>
-      <c r="U28" s="190"/>
-      <c r="V28" s="190"/>
-      <c r="W28" s="190"/>
-      <c r="X28" s="190"/>
-      <c r="Y28" s="190"/>
-      <c r="Z28" s="190"/>
+      <c r="R28" s="174"/>
+      <c r="S28" s="174"/>
+      <c r="T28" s="174"/>
+      <c r="U28" s="174"/>
+      <c r="V28" s="174"/>
+      <c r="W28" s="174"/>
+      <c r="X28" s="174"/>
+      <c r="Y28" s="174"/>
+      <c r="Z28" s="174"/>
       <c r="AA28" s="10"/>
       <c r="AB28" s="10"/>
       <c r="AC28" s="61"/>
@@ -4441,15 +4576,15 @@
       <c r="O29" s="70"/>
       <c r="P29" s="71"/>
       <c r="Q29" s="78"/>
-      <c r="R29" s="190"/>
-      <c r="S29" s="190"/>
-      <c r="T29" s="190"/>
-      <c r="U29" s="190"/>
-      <c r="V29" s="190"/>
-      <c r="W29" s="190"/>
-      <c r="X29" s="190"/>
-      <c r="Y29" s="190"/>
-      <c r="Z29" s="190"/>
+      <c r="R29" s="174"/>
+      <c r="S29" s="174"/>
+      <c r="T29" s="174"/>
+      <c r="U29" s="174"/>
+      <c r="V29" s="174"/>
+      <c r="W29" s="174"/>
+      <c r="X29" s="174"/>
+      <c r="Y29" s="174"/>
+      <c r="Z29" s="174"/>
       <c r="AA29" s="10"/>
       <c r="AB29" s="62"/>
       <c r="AC29" s="103"/>
@@ -4506,15 +4641,15 @@
       <c r="O30" s="80"/>
       <c r="P30" s="81"/>
       <c r="Q30" s="78"/>
-      <c r="R30" s="190"/>
-      <c r="S30" s="190"/>
-      <c r="T30" s="190"/>
-      <c r="U30" s="190"/>
-      <c r="V30" s="190"/>
-      <c r="W30" s="190"/>
-      <c r="X30" s="190"/>
-      <c r="Y30" s="190"/>
-      <c r="Z30" s="190"/>
+      <c r="R30" s="174"/>
+      <c r="S30" s="174"/>
+      <c r="T30" s="174"/>
+      <c r="U30" s="174"/>
+      <c r="V30" s="174"/>
+      <c r="W30" s="174"/>
+      <c r="X30" s="174"/>
+      <c r="Y30" s="174"/>
+      <c r="Z30" s="174"/>
       <c r="AA30" s="10"/>
       <c r="AB30" s="62"/>
       <c r="AC30" s="109"/>
@@ -4571,15 +4706,15 @@
       <c r="O31" s="99"/>
       <c r="P31" s="99"/>
       <c r="Q31" s="10"/>
-      <c r="R31" s="190"/>
-      <c r="S31" s="190"/>
-      <c r="T31" s="190"/>
-      <c r="U31" s="190"/>
-      <c r="V31" s="190"/>
-      <c r="W31" s="190"/>
-      <c r="X31" s="190"/>
-      <c r="Y31" s="190"/>
-      <c r="Z31" s="190"/>
+      <c r="R31" s="174"/>
+      <c r="S31" s="174"/>
+      <c r="T31" s="174"/>
+      <c r="U31" s="174"/>
+      <c r="V31" s="174"/>
+      <c r="W31" s="174"/>
+      <c r="X31" s="174"/>
+      <c r="Y31" s="174"/>
+      <c r="Z31" s="174"/>
       <c r="AA31" s="10"/>
       <c r="AB31" s="62"/>
       <c r="AC31" s="109"/>
@@ -4640,15 +4775,15 @@
       <c r="O32" s="102"/>
       <c r="P32" s="102"/>
       <c r="Q32" s="10"/>
-      <c r="R32" s="190"/>
-      <c r="S32" s="190"/>
-      <c r="T32" s="190"/>
-      <c r="U32" s="190"/>
-      <c r="V32" s="190"/>
-      <c r="W32" s="190"/>
-      <c r="X32" s="190"/>
-      <c r="Y32" s="190"/>
-      <c r="Z32" s="190"/>
+      <c r="R32" s="174"/>
+      <c r="S32" s="174"/>
+      <c r="T32" s="174"/>
+      <c r="U32" s="174"/>
+      <c r="V32" s="174"/>
+      <c r="W32" s="174"/>
+      <c r="X32" s="174"/>
+      <c r="Y32" s="174"/>
+      <c r="Z32" s="174"/>
       <c r="AA32" s="10"/>
       <c r="AB32" s="62"/>
       <c r="AC32" s="109"/>
@@ -4707,15 +4842,15 @@
       <c r="O33" s="102"/>
       <c r="P33" s="102"/>
       <c r="Q33" s="10"/>
-      <c r="R33" s="190"/>
-      <c r="S33" s="190"/>
-      <c r="T33" s="190"/>
-      <c r="U33" s="190"/>
-      <c r="V33" s="190"/>
-      <c r="W33" s="190"/>
-      <c r="X33" s="190"/>
-      <c r="Y33" s="190"/>
-      <c r="Z33" s="190"/>
+      <c r="R33" s="174"/>
+      <c r="S33" s="174"/>
+      <c r="T33" s="174"/>
+      <c r="U33" s="174"/>
+      <c r="V33" s="174"/>
+      <c r="W33" s="174"/>
+      <c r="X33" s="174"/>
+      <c r="Y33" s="174"/>
+      <c r="Z33" s="174"/>
       <c r="AA33" s="10"/>
       <c r="AB33" s="62"/>
       <c r="AC33" s="114"/>
@@ -5707,7 +5842,7 @@
       <c r="AJ48" s="35"/>
       <c r="AK48" s="35"/>
       <c r="AL48" s="35"/>
-      <c r="AM48" s="187"/>
+      <c r="AM48" s="10"/>
       <c r="AN48" s="35"/>
       <c r="AO48" s="35"/>
       <c r="AP48" s="7"/>
@@ -5771,12 +5906,12 @@
       <c r="AG49" s="22"/>
       <c r="AH49" s="22"/>
       <c r="AI49" s="36"/>
-      <c r="AJ49" s="194"/>
-      <c r="AK49" s="195"/>
-      <c r="AL49" s="195"/>
-      <c r="AM49" s="195"/>
-      <c r="AN49" s="195"/>
-      <c r="AO49" s="196"/>
+      <c r="AJ49" s="178"/>
+      <c r="AK49" s="179"/>
+      <c r="AL49" s="179"/>
+      <c r="AM49" s="179"/>
+      <c r="AN49" s="179"/>
+      <c r="AO49" s="180"/>
       <c r="AP49" s="40"/>
       <c r="AQ49" s="10"/>
       <c r="AR49" s="10"/>
@@ -5836,12 +5971,12 @@
       <c r="AG50" s="7"/>
       <c r="AH50" s="22"/>
       <c r="AI50" s="36"/>
-      <c r="AJ50" s="197"/>
-      <c r="AK50" s="193"/>
-      <c r="AL50" s="193"/>
-      <c r="AM50" s="193"/>
-      <c r="AN50" s="193"/>
-      <c r="AO50" s="198"/>
+      <c r="AJ50" s="181"/>
+      <c r="AK50" s="177"/>
+      <c r="AL50" s="177"/>
+      <c r="AM50" s="177"/>
+      <c r="AN50" s="177"/>
+      <c r="AO50" s="182"/>
       <c r="AP50" s="40"/>
       <c r="AQ50" s="10"/>
       <c r="AR50" s="10"/>
@@ -5901,13 +6036,13 @@
       <c r="AG51" s="7"/>
       <c r="AH51" s="22"/>
       <c r="AI51" s="36"/>
-      <c r="AJ51" s="197"/>
-      <c r="AK51" s="193"/>
-      <c r="AL51" s="193"/>
-      <c r="AM51" s="193"/>
-      <c r="AN51" s="193"/>
-      <c r="AO51" s="198"/>
-      <c r="AP51" s="187"/>
+      <c r="AJ51" s="181"/>
+      <c r="AK51" s="177"/>
+      <c r="AL51" s="177"/>
+      <c r="AM51" s="177"/>
+      <c r="AN51" s="177"/>
+      <c r="AO51" s="182"/>
+      <c r="AP51" s="10"/>
       <c r="AQ51" s="10"/>
       <c r="AR51" s="10"/>
       <c r="AS51" s="7"/>
@@ -5966,12 +6101,12 @@
       <c r="AG52" s="40"/>
       <c r="AH52" s="22"/>
       <c r="AI52" s="36"/>
-      <c r="AJ52" s="197"/>
-      <c r="AK52" s="193"/>
-      <c r="AL52" s="193"/>
-      <c r="AM52" s="193"/>
-      <c r="AN52" s="193"/>
-      <c r="AO52" s="198"/>
+      <c r="AJ52" s="181"/>
+      <c r="AK52" s="177"/>
+      <c r="AL52" s="177"/>
+      <c r="AM52" s="177"/>
+      <c r="AN52" s="177"/>
+      <c r="AO52" s="182"/>
       <c r="AP52" s="40"/>
       <c r="AQ52" s="10"/>
       <c r="AR52" s="10"/>
@@ -6031,12 +6166,12 @@
       <c r="AG53" s="40"/>
       <c r="AH53" s="22"/>
       <c r="AI53" s="36"/>
-      <c r="AJ53" s="199"/>
-      <c r="AK53" s="200"/>
-      <c r="AL53" s="200"/>
-      <c r="AM53" s="200"/>
-      <c r="AN53" s="200"/>
-      <c r="AO53" s="201"/>
+      <c r="AJ53" s="183"/>
+      <c r="AK53" s="184"/>
+      <c r="AL53" s="184"/>
+      <c r="AM53" s="184"/>
+      <c r="AN53" s="184"/>
+      <c r="AO53" s="185"/>
       <c r="AP53" s="40"/>
       <c r="AQ53" s="10"/>
       <c r="AR53" s="10"/>
@@ -6585,7 +6720,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
-  <dimension ref="A1:D97"/>
+  <dimension ref="A1:D99"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="6" customWidth="1"/>
@@ -6595,32 +6730,32 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:4" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="A1" s="173" t="s">
+      <c r="A1" s="195" t="s">
         <v>42</v>
       </c>
-      <c r="B1" s="174"/>
-      <c r="C1" s="174"/>
-      <c r="D1" s="174"/>
+      <c r="B1" s="196"/>
+      <c r="C1" s="196"/>
+      <c r="D1" s="196"/>
     </row>
     <row r="3" spans="1:4" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="180" t="s">
+      <c r="A3" s="201" t="s">
         <v>43</v>
       </c>
-      <c r="B3" s="174"/>
-      <c r="C3" s="174"/>
-      <c r="D3" s="174"/>
+      <c r="B3" s="196"/>
+      <c r="C3" s="196"/>
+      <c r="D3" s="196"/>
     </row>
     <row r="4" spans="1:4" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="174"/>
-      <c r="B4" s="174"/>
-      <c r="C4" s="174"/>
-      <c r="D4" s="174"/>
+      <c r="A4" s="196"/>
+      <c r="B4" s="196"/>
+      <c r="C4" s="196"/>
+      <c r="D4" s="196"/>
     </row>
     <row r="5" spans="1:4" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="174"/>
-      <c r="B5" s="174"/>
-      <c r="C5" s="174"/>
-      <c r="D5" s="174"/>
+      <c r="A5" s="196"/>
+      <c r="B5" s="196"/>
+      <c r="C5" s="196"/>
+      <c r="D5" s="196"/>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A7" s="1" t="s">
@@ -6637,12 +6772,12 @@
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A8" s="177" t="s">
+      <c r="A8" s="202" t="s">
         <v>46</v>
       </c>
-      <c r="B8" s="174"/>
-      <c r="C8" s="174"/>
-      <c r="D8" s="174"/>
+      <c r="B8" s="196"/>
+      <c r="C8" s="196"/>
+      <c r="D8" s="196"/>
     </row>
     <row r="9" spans="1:4" ht="24" x14ac:dyDescent="0.25">
       <c r="A9" s="20"/>
@@ -6716,676 +6851,700 @@
         <v>59</v>
       </c>
     </row>
-    <row r="15" spans="1:4" ht="36" x14ac:dyDescent="0.25">
-      <c r="A15" s="190"/>
-      <c r="B15" s="184" t="s">
+    <row r="15" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A15" s="209"/>
+      <c r="B15" s="2" t="s">
+        <v>192</v>
+      </c>
+      <c r="C15" s="21" t="s">
+        <v>48</v>
+      </c>
+      <c r="D15" s="4" t="s">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="16" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A16" s="208"/>
+      <c r="B16" s="2" t="s">
+        <v>188</v>
+      </c>
+      <c r="C16" s="21" t="s">
+        <v>48</v>
+      </c>
+      <c r="D16" s="4" t="s">
+        <v>199</v>
+      </c>
+    </row>
+    <row r="17" spans="1:4" ht="36" x14ac:dyDescent="0.25">
+      <c r="A17" s="174"/>
+      <c r="B17" s="2" t="s">
         <v>155</v>
       </c>
-      <c r="C15" s="188" t="s">
+      <c r="C17" s="21" t="s">
         <v>48</v>
       </c>
-      <c r="D15" s="185" t="s">
+      <c r="D17" s="4" t="s">
         <v>156</v>
       </c>
     </row>
-    <row r="16" spans="1:4" ht="24" x14ac:dyDescent="0.25">
-      <c r="A16" s="191"/>
-      <c r="B16" s="184" t="s">
+    <row r="18" spans="1:4" ht="24" x14ac:dyDescent="0.25">
+      <c r="A18" s="175"/>
+      <c r="B18" s="2" t="s">
         <v>157</v>
-      </c>
-      <c r="C16" s="188" t="s">
-        <v>48</v>
-      </c>
-      <c r="D16" s="185" t="s">
-        <v>158</v>
-      </c>
-    </row>
-    <row r="17" spans="1:4" ht="24" x14ac:dyDescent="0.25">
-      <c r="A17" s="192"/>
-      <c r="B17" s="184" t="s">
-        <v>159</v>
-      </c>
-      <c r="C17" s="188" t="s">
-        <v>48</v>
-      </c>
-      <c r="D17" s="185" t="s">
-        <v>160</v>
-      </c>
-    </row>
-    <row r="18" spans="1:4" ht="24" x14ac:dyDescent="0.25">
-      <c r="A18" s="26"/>
-      <c r="B18" s="2" t="s">
-        <v>60</v>
       </c>
       <c r="C18" s="21" t="s">
         <v>48</v>
       </c>
       <c r="D18" s="4" t="s">
-        <v>61</v>
+        <v>158</v>
       </c>
     </row>
     <row r="19" spans="1:4" ht="24" x14ac:dyDescent="0.25">
-      <c r="A19" s="27"/>
+      <c r="A19" s="176"/>
       <c r="B19" s="2" t="s">
-        <v>62</v>
+        <v>159</v>
       </c>
       <c r="C19" s="21" t="s">
         <v>48</v>
       </c>
       <c r="D19" s="4" t="s">
-        <v>63</v>
-      </c>
-    </row>
-    <row r="20" spans="1:4" ht="36" x14ac:dyDescent="0.25">
-      <c r="A20" s="162"/>
+        <v>160</v>
+      </c>
+    </row>
+    <row r="20" spans="1:4" ht="24" x14ac:dyDescent="0.25">
+      <c r="A20" s="26"/>
       <c r="B20" s="2" t="s">
-        <v>153</v>
+        <v>60</v>
       </c>
       <c r="C20" s="21" t="s">
         <v>48</v>
       </c>
       <c r="D20" s="4" t="s">
-        <v>154</v>
-      </c>
-    </row>
-    <row r="21" spans="1:4" ht="36" x14ac:dyDescent="0.25">
-      <c r="A21" s="28"/>
+        <v>61</v>
+      </c>
+    </row>
+    <row r="21" spans="1:4" ht="24" x14ac:dyDescent="0.25">
+      <c r="A21" s="27"/>
       <c r="B21" s="2" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="C21" s="21" t="s">
         <v>48</v>
       </c>
       <c r="D21" s="4" t="s">
-        <v>65</v>
-      </c>
-    </row>
-    <row r="22" spans="1:4" ht="24" x14ac:dyDescent="0.25">
-      <c r="A22" s="29"/>
+        <v>63</v>
+      </c>
+    </row>
+    <row r="22" spans="1:4" ht="36" x14ac:dyDescent="0.25">
+      <c r="A22" s="162"/>
       <c r="B22" s="2" t="s">
-        <v>66</v>
+        <v>153</v>
       </c>
       <c r="C22" s="21" t="s">
         <v>48</v>
       </c>
       <c r="D22" s="4" t="s">
-        <v>67</v>
-      </c>
-    </row>
-    <row r="23" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A23" s="7"/>
+        <v>154</v>
+      </c>
+    </row>
+    <row r="23" spans="1:4" ht="36" x14ac:dyDescent="0.25">
+      <c r="A23" s="28"/>
       <c r="B23" s="2" t="s">
-        <v>68</v>
+        <v>64</v>
       </c>
       <c r="C23" s="21" t="s">
         <v>48</v>
       </c>
       <c r="D23" s="4" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="24" spans="1:4" ht="24" x14ac:dyDescent="0.25">
+      <c r="A24" s="29"/>
+      <c r="B24" s="2" t="s">
+        <v>66</v>
+      </c>
+      <c r="C24" s="21" t="s">
+        <v>48</v>
+      </c>
+      <c r="D24" s="4" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="25" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A25" s="7"/>
+      <c r="B25" s="2" t="s">
+        <v>68</v>
+      </c>
+      <c r="C25" s="21" t="s">
+        <v>48</v>
+      </c>
+      <c r="D25" s="4" t="s">
         <v>69</v>
       </c>
     </row>
-    <row r="24" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A24" s="181" t="s">
+    <row r="26" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A26" s="203" t="s">
         <v>70</v>
       </c>
-      <c r="B24" s="174"/>
-      <c r="C24" s="174"/>
-      <c r="D24" s="174"/>
-    </row>
-    <row r="26" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A26" s="177" t="s">
+      <c r="B26" s="196"/>
+      <c r="C26" s="196"/>
+      <c r="D26" s="196"/>
+    </row>
+    <row r="28" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A28" s="202" t="s">
         <v>71</v>
       </c>
-      <c r="B26" s="174"/>
-      <c r="C26" s="174"/>
-      <c r="D26" s="174"/>
-    </row>
-    <row r="27" spans="1:4" ht="36" x14ac:dyDescent="0.25">
-      <c r="A27" s="30"/>
-      <c r="B27" s="2" t="s">
+      <c r="B28" s="196"/>
+      <c r="C28" s="196"/>
+      <c r="D28" s="196"/>
+    </row>
+    <row r="29" spans="1:4" ht="36" x14ac:dyDescent="0.25">
+      <c r="A29" s="30"/>
+      <c r="B29" s="2" t="s">
         <v>72</v>
       </c>
-      <c r="C27" s="21" t="s">
+      <c r="C29" s="21" t="s">
         <v>73</v>
       </c>
-      <c r="D27" s="4" t="s">
+      <c r="D29" s="4" t="s">
         <v>74</v>
       </c>
     </row>
-    <row r="28" spans="1:4" ht="36" x14ac:dyDescent="0.25">
-      <c r="B28" s="2" t="s">
+    <row r="30" spans="1:4" ht="36" x14ac:dyDescent="0.25">
+      <c r="B30" s="2" t="s">
         <v>75</v>
       </c>
-      <c r="C28" s="21" t="s">
+      <c r="C30" s="21" t="s">
         <v>76</v>
       </c>
-      <c r="D28" s="4" t="s">
+      <c r="D30" s="4" t="s">
         <v>77</v>
       </c>
     </row>
-    <row r="29" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A29" s="179" t="s">
+    <row r="31" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A31" s="200" t="s">
         <v>78</v>
       </c>
-      <c r="B29" s="174"/>
-      <c r="C29" s="174"/>
-      <c r="D29" s="174"/>
-    </row>
-    <row r="30" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A30" s="174"/>
-      <c r="B30" s="174"/>
-      <c r="C30" s="174"/>
-      <c r="D30" s="174"/>
+      <c r="B31" s="196"/>
+      <c r="C31" s="196"/>
+      <c r="D31" s="196"/>
     </row>
     <row r="32" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A32" s="177" t="s">
+      <c r="A32" s="196"/>
+      <c r="B32" s="196"/>
+      <c r="C32" s="196"/>
+      <c r="D32" s="196"/>
+    </row>
+    <row r="34" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A34" s="202" t="s">
         <v>79</v>
       </c>
-      <c r="B32" s="174"/>
-      <c r="C32" s="174"/>
-      <c r="D32" s="174"/>
-    </row>
-    <row r="33" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A33" s="1" t="s">
+      <c r="B34" s="196"/>
+      <c r="C34" s="196"/>
+      <c r="D34" s="196"/>
+    </row>
+    <row r="35" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A35" s="1" t="s">
         <v>80</v>
       </c>
-      <c r="B33" s="1" t="s">
+      <c r="B35" s="1" t="s">
         <v>81</v>
       </c>
-      <c r="C33" s="1" t="s">
+      <c r="C35" s="1" t="s">
         <v>82</v>
       </c>
     </row>
-    <row r="34" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A34" s="31" t="s">
+    <row r="36" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A36" s="31" t="s">
         <v>83</v>
       </c>
-      <c r="B34" s="31" t="s">
+      <c r="B36" s="31" t="s">
         <v>84</v>
       </c>
     </row>
-    <row r="35" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A35" s="32"/>
-      <c r="B35" s="32"/>
-      <c r="C35" s="32"/>
-    </row>
-    <row r="36" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A36" s="32"/>
-      <c r="B36" s="32"/>
-      <c r="C36" s="32"/>
-    </row>
-    <row r="37" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A37" s="32"/>
       <c r="B37" s="32"/>
       <c r="C37" s="32"/>
     </row>
-    <row r="38" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A38" s="32"/>
       <c r="B38" s="32"/>
       <c r="C38" s="32"/>
     </row>
-    <row r="39" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A39" s="32"/>
       <c r="B39" s="32"/>
       <c r="C39" s="32"/>
     </row>
-    <row r="40" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A40" s="32"/>
       <c r="B40" s="32"/>
       <c r="C40" s="32"/>
     </row>
-    <row r="41" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A41" s="32"/>
       <c r="B41" s="32"/>
       <c r="C41" s="32"/>
     </row>
-    <row r="42" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A42" s="32"/>
       <c r="B42" s="32"/>
       <c r="C42" s="32"/>
     </row>
-    <row r="43" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A43" s="32"/>
       <c r="B43" s="32"/>
       <c r="C43" s="32"/>
     </row>
-    <row r="44" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A44" s="32"/>
       <c r="B44" s="32"/>
       <c r="C44" s="32"/>
     </row>
-    <row r="45" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A45" s="32"/>
       <c r="B45" s="32"/>
       <c r="C45" s="32"/>
     </row>
-    <row r="46" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A46" s="32"/>
       <c r="B46" s="32"/>
       <c r="C46" s="32"/>
     </row>
-    <row r="47" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A47" s="32"/>
       <c r="B47" s="32"/>
       <c r="C47" s="32"/>
     </row>
-    <row r="48" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A48" s="32"/>
       <c r="B48" s="32"/>
       <c r="C48" s="32"/>
     </row>
     <row r="49" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A49" s="179" t="s">
+      <c r="A49" s="32"/>
+      <c r="B49" s="32"/>
+      <c r="C49" s="32"/>
+    </row>
+    <row r="50" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A50" s="32"/>
+      <c r="B50" s="32"/>
+      <c r="C50" s="32"/>
+    </row>
+    <row r="51" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A51" s="200" t="s">
         <v>85</v>
       </c>
-      <c r="B49" s="174"/>
-      <c r="C49" s="174"/>
-      <c r="D49" s="174"/>
-    </row>
-    <row r="50" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A50" s="174"/>
-      <c r="B50" s="174"/>
-      <c r="C50" s="174"/>
-      <c r="D50" s="174"/>
-    </row>
-    <row r="54" spans="1:4" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A54" s="178" t="s">
+      <c r="B51" s="196"/>
+      <c r="C51" s="196"/>
+      <c r="D51" s="196"/>
+    </row>
+    <row r="52" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A52" s="196"/>
+      <c r="B52" s="196"/>
+      <c r="C52" s="196"/>
+      <c r="D52" s="196"/>
+    </row>
+    <row r="56" spans="1:4" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A56" s="199" t="s">
         <v>86</v>
       </c>
-      <c r="B54" s="174"/>
-      <c r="C54" s="174"/>
-      <c r="D54" s="174"/>
-    </row>
-    <row r="55" spans="1:4" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A55" s="176" t="s">
+      <c r="B56" s="196"/>
+      <c r="C56" s="196"/>
+      <c r="D56" s="196"/>
+    </row>
+    <row r="57" spans="1:4" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A57" s="198" t="s">
         <v>87</v>
       </c>
-      <c r="B55" s="174"/>
-      <c r="C55" s="174"/>
-      <c r="D55" s="174"/>
-    </row>
-    <row r="56" spans="1:4" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A56" s="176" t="s">
+      <c r="B57" s="196"/>
+      <c r="C57" s="196"/>
+      <c r="D57" s="196"/>
+    </row>
+    <row r="58" spans="1:4" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A58" s="198" t="s">
         <v>88</v>
       </c>
-      <c r="B56" s="174"/>
-      <c r="C56" s="174"/>
-      <c r="D56" s="174"/>
-    </row>
-    <row r="57" spans="1:4" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A57" s="176" t="s">
+      <c r="B58" s="196"/>
+      <c r="C58" s="196"/>
+      <c r="D58" s="196"/>
+    </row>
+    <row r="59" spans="1:4" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A59" s="198" t="s">
         <v>89</v>
       </c>
-      <c r="B57" s="174"/>
-      <c r="C57" s="174"/>
-      <c r="D57" s="174"/>
-    </row>
-    <row r="58" spans="1:4" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A58" s="176" t="s">
+      <c r="B59" s="196"/>
+      <c r="C59" s="196"/>
+      <c r="D59" s="196"/>
+    </row>
+    <row r="60" spans="1:4" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A60" s="198" t="s">
         <v>90</v>
       </c>
-      <c r="B58" s="174"/>
-      <c r="C58" s="174"/>
-      <c r="D58" s="174"/>
-    </row>
-    <row r="59" spans="1:4" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A59" s="176" t="s">
+      <c r="B60" s="196"/>
+      <c r="C60" s="196"/>
+      <c r="D60" s="196"/>
+    </row>
+    <row r="61" spans="1:4" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A61" s="198" t="s">
         <v>91</v>
       </c>
-      <c r="B59" s="174"/>
-      <c r="C59" s="174"/>
-      <c r="D59" s="174"/>
-    </row>
-    <row r="60" spans="1:4" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A60" s="176" t="s">
+      <c r="B61" s="196"/>
+      <c r="C61" s="196"/>
+      <c r="D61" s="196"/>
+    </row>
+    <row r="62" spans="1:4" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A62" s="198" t="s">
         <v>92</v>
       </c>
-      <c r="B60" s="174"/>
-      <c r="C60" s="174"/>
-      <c r="D60" s="174"/>
-    </row>
-    <row r="61" spans="1:4" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A61" s="176" t="s">
+      <c r="B62" s="196"/>
+      <c r="C62" s="196"/>
+      <c r="D62" s="196"/>
+    </row>
+    <row r="63" spans="1:4" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A63" s="198" t="s">
         <v>93</v>
       </c>
-      <c r="B61" s="174"/>
-      <c r="C61" s="174"/>
-      <c r="D61" s="174"/>
-    </row>
-    <row r="62" spans="1:4" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A62" s="176" t="s">
+      <c r="B63" s="196"/>
+      <c r="C63" s="196"/>
+      <c r="D63" s="196"/>
+    </row>
+    <row r="64" spans="1:4" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A64" s="198" t="s">
         <v>94</v>
       </c>
-      <c r="B62" s="174"/>
-      <c r="C62" s="174"/>
-      <c r="D62" s="174"/>
-    </row>
-    <row r="63" spans="1:4" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A63" s="176" t="s">
+      <c r="B64" s="196"/>
+      <c r="C64" s="196"/>
+      <c r="D64" s="196"/>
+    </row>
+    <row r="65" spans="1:4" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A65" s="198" t="s">
         <v>95</v>
       </c>
-      <c r="B63" s="174"/>
-      <c r="C63" s="174"/>
-      <c r="D63" s="174"/>
-    </row>
-    <row r="64" spans="1:4" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A64" s="176" t="s">
+      <c r="B65" s="196"/>
+      <c r="C65" s="196"/>
+      <c r="D65" s="196"/>
+    </row>
+    <row r="66" spans="1:4" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A66" s="198" t="s">
         <v>96</v>
       </c>
-      <c r="B64" s="174"/>
-      <c r="C64" s="174"/>
-      <c r="D64" s="174"/>
-    </row>
-    <row r="65" spans="1:4" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A65" s="176" t="s">
+      <c r="B66" s="196"/>
+      <c r="C66" s="196"/>
+      <c r="D66" s="196"/>
+    </row>
+    <row r="67" spans="1:4" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A67" s="198" t="s">
         <v>97</v>
       </c>
-      <c r="B65" s="174"/>
-      <c r="C65" s="174"/>
-      <c r="D65" s="174"/>
-    </row>
-    <row r="66" spans="1:4" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A66" s="176"/>
-      <c r="B66" s="174"/>
-      <c r="C66" s="174"/>
-      <c r="D66" s="174"/>
-    </row>
-    <row r="67" spans="1:4" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A67" s="178" t="s">
+      <c r="B67" s="196"/>
+      <c r="C67" s="196"/>
+      <c r="D67" s="196"/>
+    </row>
+    <row r="68" spans="1:4" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A68" s="198"/>
+      <c r="B68" s="196"/>
+      <c r="C68" s="196"/>
+      <c r="D68" s="196"/>
+    </row>
+    <row r="69" spans="1:4" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A69" s="199" t="s">
         <v>98</v>
       </c>
-      <c r="B67" s="174"/>
-      <c r="C67" s="174"/>
-      <c r="D67" s="174"/>
-    </row>
-    <row r="68" spans="1:4" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A68" s="176" t="s">
+      <c r="B69" s="196"/>
+      <c r="C69" s="196"/>
+      <c r="D69" s="196"/>
+    </row>
+    <row r="70" spans="1:4" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A70" s="198" t="s">
         <v>99</v>
       </c>
-      <c r="B68" s="174"/>
-      <c r="C68" s="174"/>
-      <c r="D68" s="174"/>
-    </row>
-    <row r="69" spans="1:4" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A69" s="176" t="s">
+      <c r="B70" s="196"/>
+      <c r="C70" s="196"/>
+      <c r="D70" s="196"/>
+    </row>
+    <row r="71" spans="1:4" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A71" s="198" t="s">
         <v>100</v>
       </c>
-      <c r="B69" s="174"/>
-      <c r="C69" s="174"/>
-      <c r="D69" s="174"/>
-    </row>
-    <row r="70" spans="1:4" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A70" s="176" t="s">
+      <c r="B71" s="196"/>
+      <c r="C71" s="196"/>
+      <c r="D71" s="196"/>
+    </row>
+    <row r="72" spans="1:4" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A72" s="198" t="s">
         <v>101</v>
       </c>
-      <c r="B70" s="174"/>
-      <c r="C70" s="174"/>
-      <c r="D70" s="174"/>
-    </row>
-    <row r="71" spans="1:4" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A71" s="176" t="s">
+      <c r="B72" s="196"/>
+      <c r="C72" s="196"/>
+      <c r="D72" s="196"/>
+    </row>
+    <row r="73" spans="1:4" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A73" s="198" t="s">
         <v>102</v>
       </c>
-      <c r="B71" s="174"/>
-      <c r="C71" s="174"/>
-      <c r="D71" s="174"/>
-    </row>
-    <row r="72" spans="1:4" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A72" s="176" t="s">
+      <c r="B73" s="196"/>
+      <c r="C73" s="196"/>
+      <c r="D73" s="196"/>
+    </row>
+    <row r="74" spans="1:4" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A74" s="198" t="s">
         <v>103</v>
       </c>
-      <c r="B72" s="174"/>
-      <c r="C72" s="174"/>
-      <c r="D72" s="174"/>
-    </row>
-    <row r="73" spans="1:4" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A73" s="176" t="s">
+      <c r="B74" s="196"/>
+      <c r="C74" s="196"/>
+      <c r="D74" s="196"/>
+    </row>
+    <row r="75" spans="1:4" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A75" s="198" t="s">
         <v>104</v>
       </c>
-      <c r="B73" s="174"/>
-      <c r="C73" s="174"/>
-      <c r="D73" s="174"/>
-    </row>
-    <row r="74" spans="1:4" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A74" s="176"/>
-      <c r="B74" s="174"/>
-      <c r="C74" s="174"/>
-      <c r="D74" s="174"/>
-    </row>
-    <row r="75" spans="1:4" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A75" s="178" t="s">
+      <c r="B75" s="196"/>
+      <c r="C75" s="196"/>
+      <c r="D75" s="196"/>
+    </row>
+    <row r="76" spans="1:4" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A76" s="198"/>
+      <c r="B76" s="196"/>
+      <c r="C76" s="196"/>
+      <c r="D76" s="196"/>
+    </row>
+    <row r="77" spans="1:4" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A77" s="199" t="s">
         <v>105</v>
       </c>
-      <c r="B75" s="174"/>
-      <c r="C75" s="174"/>
-      <c r="D75" s="174"/>
-    </row>
-    <row r="76" spans="1:4" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A76" s="176" t="s">
+      <c r="B77" s="196"/>
+      <c r="C77" s="196"/>
+      <c r="D77" s="196"/>
+    </row>
+    <row r="78" spans="1:4" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A78" s="198" t="s">
         <v>106</v>
       </c>
-      <c r="B76" s="174"/>
-      <c r="C76" s="174"/>
-      <c r="D76" s="174"/>
-    </row>
-    <row r="77" spans="1:4" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A77" s="176" t="s">
+      <c r="B78" s="196"/>
+      <c r="C78" s="196"/>
+      <c r="D78" s="196"/>
+    </row>
+    <row r="79" spans="1:4" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A79" s="198" t="s">
         <v>107</v>
       </c>
-      <c r="B77" s="174"/>
-      <c r="C77" s="174"/>
-      <c r="D77" s="174"/>
-    </row>
-    <row r="78" spans="1:4" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A78" s="176" t="s">
+      <c r="B79" s="196"/>
+      <c r="C79" s="196"/>
+      <c r="D79" s="196"/>
+    </row>
+    <row r="80" spans="1:4" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A80" s="198" t="s">
         <v>108</v>
       </c>
-      <c r="B78" s="174"/>
-      <c r="C78" s="174"/>
-      <c r="D78" s="174"/>
-    </row>
-    <row r="79" spans="1:4" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A79" s="176" t="s">
+      <c r="B80" s="196"/>
+      <c r="C80" s="196"/>
+      <c r="D80" s="196"/>
+    </row>
+    <row r="81" spans="1:4" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A81" s="198" t="s">
         <v>109</v>
       </c>
-      <c r="B79" s="174"/>
-      <c r="C79" s="174"/>
-      <c r="D79" s="174"/>
-    </row>
-    <row r="80" spans="1:4" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A80" s="176" t="s">
+      <c r="B81" s="196"/>
+      <c r="C81" s="196"/>
+      <c r="D81" s="196"/>
+    </row>
+    <row r="82" spans="1:4" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A82" s="198" t="s">
         <v>110</v>
       </c>
-      <c r="B80" s="174"/>
-      <c r="C80" s="174"/>
-      <c r="D80" s="174"/>
-    </row>
-    <row r="81" spans="1:4" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A81" s="176"/>
-      <c r="B81" s="174"/>
-      <c r="C81" s="174"/>
-      <c r="D81" s="174"/>
-    </row>
-    <row r="82" spans="1:4" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A82" s="178" t="s">
+      <c r="B82" s="196"/>
+      <c r="C82" s="196"/>
+      <c r="D82" s="196"/>
+    </row>
+    <row r="83" spans="1:4" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A83" s="198"/>
+      <c r="B83" s="196"/>
+      <c r="C83" s="196"/>
+      <c r="D83" s="196"/>
+    </row>
+    <row r="84" spans="1:4" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A84" s="199" t="s">
         <v>111</v>
       </c>
-      <c r="B82" s="174"/>
-      <c r="C82" s="174"/>
-      <c r="D82" s="174"/>
-    </row>
-    <row r="83" spans="1:4" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A83" s="176" t="s">
+      <c r="B84" s="196"/>
+      <c r="C84" s="196"/>
+      <c r="D84" s="196"/>
+    </row>
+    <row r="85" spans="1:4" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A85" s="198" t="s">
         <v>112</v>
       </c>
-      <c r="B83" s="174"/>
-      <c r="C83" s="174"/>
-      <c r="D83" s="174"/>
-    </row>
-    <row r="84" spans="1:4" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A84" s="176" t="s">
+      <c r="B85" s="196"/>
+      <c r="C85" s="196"/>
+      <c r="D85" s="196"/>
+    </row>
+    <row r="86" spans="1:4" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A86" s="198" t="s">
         <v>113</v>
       </c>
-      <c r="B84" s="174"/>
-      <c r="C84" s="174"/>
-      <c r="D84" s="174"/>
-    </row>
-    <row r="85" spans="1:4" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A85" s="176" t="s">
+      <c r="B86" s="196"/>
+      <c r="C86" s="196"/>
+      <c r="D86" s="196"/>
+    </row>
+    <row r="87" spans="1:4" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A87" s="198" t="s">
         <v>114</v>
       </c>
-      <c r="B85" s="174"/>
-      <c r="C85" s="174"/>
-      <c r="D85" s="174"/>
-    </row>
-    <row r="86" spans="1:4" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A86" s="176" t="s">
+      <c r="B87" s="196"/>
+      <c r="C87" s="196"/>
+      <c r="D87" s="196"/>
+    </row>
+    <row r="88" spans="1:4" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A88" s="198" t="s">
         <v>115</v>
       </c>
-      <c r="B86" s="174"/>
-      <c r="C86" s="174"/>
-      <c r="D86" s="174"/>
-    </row>
-    <row r="87" spans="1:4" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A87" s="176" t="s">
+      <c r="B88" s="196"/>
+      <c r="C88" s="196"/>
+      <c r="D88" s="196"/>
+    </row>
+    <row r="89" spans="1:4" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A89" s="198" t="s">
         <v>116</v>
       </c>
-      <c r="B87" s="174"/>
-      <c r="C87" s="174"/>
-      <c r="D87" s="174"/>
-    </row>
-    <row r="88" spans="1:4" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A88" s="176" t="s">
+      <c r="B89" s="196"/>
+      <c r="C89" s="196"/>
+      <c r="D89" s="196"/>
+    </row>
+    <row r="90" spans="1:4" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A90" s="198" t="s">
         <v>117</v>
       </c>
-      <c r="B88" s="174"/>
-      <c r="C88" s="174"/>
-      <c r="D88" s="174"/>
-    </row>
-    <row r="89" spans="1:4" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A89" s="176" t="s">
+      <c r="B90" s="196"/>
+      <c r="C90" s="196"/>
+      <c r="D90" s="196"/>
+    </row>
+    <row r="91" spans="1:4" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A91" s="198" t="s">
         <v>118</v>
       </c>
-      <c r="B89" s="174"/>
-      <c r="C89" s="174"/>
-      <c r="D89" s="174"/>
-    </row>
-    <row r="90" spans="1:4" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A90" s="176"/>
-      <c r="B90" s="174"/>
-      <c r="C90" s="174"/>
-      <c r="D90" s="174"/>
-    </row>
-    <row r="91" spans="1:4" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A91" s="178" t="s">
+      <c r="B91" s="196"/>
+      <c r="C91" s="196"/>
+      <c r="D91" s="196"/>
+    </row>
+    <row r="92" spans="1:4" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A92" s="198"/>
+      <c r="B92" s="196"/>
+      <c r="C92" s="196"/>
+      <c r="D92" s="196"/>
+    </row>
+    <row r="93" spans="1:4" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A93" s="199" t="s">
         <v>119</v>
       </c>
-      <c r="B91" s="174"/>
-      <c r="C91" s="174"/>
-      <c r="D91" s="174"/>
-    </row>
-    <row r="92" spans="1:4" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A92" s="176" t="s">
+      <c r="B93" s="196"/>
+      <c r="C93" s="196"/>
+      <c r="D93" s="196"/>
+    </row>
+    <row r="94" spans="1:4" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A94" s="198" t="s">
         <v>120</v>
       </c>
-      <c r="B92" s="174"/>
-      <c r="C92" s="174"/>
-      <c r="D92" s="174"/>
-    </row>
-    <row r="93" spans="1:4" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A93" s="176" t="s">
+      <c r="B94" s="196"/>
+      <c r="C94" s="196"/>
+      <c r="D94" s="196"/>
+    </row>
+    <row r="95" spans="1:4" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A95" s="198" t="s">
         <v>121</v>
       </c>
-      <c r="B93" s="174"/>
-      <c r="C93" s="174"/>
-      <c r="D93" s="174"/>
-    </row>
-    <row r="94" spans="1:4" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A94" s="176" t="s">
+      <c r="B95" s="196"/>
+      <c r="C95" s="196"/>
+      <c r="D95" s="196"/>
+    </row>
+    <row r="96" spans="1:4" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A96" s="198" t="s">
         <v>122</v>
       </c>
-      <c r="B94" s="174"/>
-      <c r="C94" s="174"/>
-      <c r="D94" s="174"/>
-    </row>
-    <row r="95" spans="1:4" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A95" s="176" t="s">
+      <c r="B96" s="196"/>
+      <c r="C96" s="196"/>
+      <c r="D96" s="196"/>
+    </row>
+    <row r="97" spans="1:4" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A97" s="198" t="s">
         <v>123</v>
       </c>
-      <c r="B95" s="174"/>
-      <c r="C95" s="174"/>
-      <c r="D95" s="174"/>
-    </row>
-    <row r="96" spans="1:4" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A96" s="176" t="s">
+      <c r="B97" s="196"/>
+      <c r="C97" s="196"/>
+      <c r="D97" s="196"/>
+    </row>
+    <row r="98" spans="1:4" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A98" s="198" t="s">
         <v>124</v>
       </c>
-      <c r="B96" s="174"/>
-      <c r="C96" s="174"/>
-      <c r="D96" s="174"/>
-    </row>
-    <row r="97" spans="1:4" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A97" s="176" t="s">
+      <c r="B98" s="196"/>
+      <c r="C98" s="196"/>
+      <c r="D98" s="196"/>
+    </row>
+    <row r="99" spans="1:4" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A99" s="198" t="s">
         <v>125</v>
       </c>
-      <c r="B97" s="174"/>
-      <c r="C97" s="174"/>
-      <c r="D97" s="174"/>
+      <c r="B99" s="196"/>
+      <c r="C99" s="196"/>
+      <c r="D99" s="196"/>
     </row>
   </sheetData>
   <mergeCells count="52">
-    <mergeCell ref="A97:D97"/>
+    <mergeCell ref="A60:D60"/>
+    <mergeCell ref="A61:D61"/>
+    <mergeCell ref="A62:D62"/>
+    <mergeCell ref="A66:D66"/>
+    <mergeCell ref="A74:D74"/>
+    <mergeCell ref="A68:D68"/>
+    <mergeCell ref="A63:D63"/>
+    <mergeCell ref="A86:D86"/>
+    <mergeCell ref="A64:D64"/>
+    <mergeCell ref="A79:D79"/>
+    <mergeCell ref="A83:D83"/>
+    <mergeCell ref="A1:D1"/>
+    <mergeCell ref="A51:D52"/>
+    <mergeCell ref="A58:D58"/>
+    <mergeCell ref="A3:D5"/>
+    <mergeCell ref="A59:D59"/>
+    <mergeCell ref="A31:D32"/>
+    <mergeCell ref="A8:D8"/>
+    <mergeCell ref="A26:D26"/>
+    <mergeCell ref="A57:D57"/>
+    <mergeCell ref="A56:D56"/>
+    <mergeCell ref="A28:D28"/>
+    <mergeCell ref="A34:D34"/>
+    <mergeCell ref="A65:D65"/>
+    <mergeCell ref="A92:D92"/>
     <mergeCell ref="A73:D73"/>
-    <mergeCell ref="A87:D87"/>
-    <mergeCell ref="A78:D78"/>
-    <mergeCell ref="A95:D95"/>
-    <mergeCell ref="A79:D79"/>
-    <mergeCell ref="A85:D85"/>
-    <mergeCell ref="A94:D94"/>
-    <mergeCell ref="A96:D96"/>
-    <mergeCell ref="A92:D92"/>
-    <mergeCell ref="A93:D93"/>
-    <mergeCell ref="A74:D74"/>
-    <mergeCell ref="A63:D63"/>
-    <mergeCell ref="A90:D90"/>
-    <mergeCell ref="A71:D71"/>
-    <mergeCell ref="A80:D80"/>
-    <mergeCell ref="A89:D89"/>
-    <mergeCell ref="A67:D67"/>
-    <mergeCell ref="A86:D86"/>
-    <mergeCell ref="A68:D68"/>
     <mergeCell ref="A82:D82"/>
+    <mergeCell ref="A91:D91"/>
+    <mergeCell ref="A69:D69"/>
     <mergeCell ref="A88:D88"/>
     <mergeCell ref="A70:D70"/>
-    <mergeCell ref="A69:D69"/>
+    <mergeCell ref="A84:D84"/>
+    <mergeCell ref="A90:D90"/>
+    <mergeCell ref="A72:D72"/>
+    <mergeCell ref="A71:D71"/>
+    <mergeCell ref="A77:D77"/>
+    <mergeCell ref="A85:D85"/>
+    <mergeCell ref="A67:D67"/>
+    <mergeCell ref="A78:D78"/>
+    <mergeCell ref="A99:D99"/>
     <mergeCell ref="A75:D75"/>
-    <mergeCell ref="A83:D83"/>
-    <mergeCell ref="A1:D1"/>
-    <mergeCell ref="A49:D50"/>
-    <mergeCell ref="A56:D56"/>
-    <mergeCell ref="A3:D5"/>
-    <mergeCell ref="A57:D57"/>
-    <mergeCell ref="A29:D30"/>
-    <mergeCell ref="A8:D8"/>
-    <mergeCell ref="A24:D24"/>
-    <mergeCell ref="A55:D55"/>
-    <mergeCell ref="A54:D54"/>
-    <mergeCell ref="A65:D65"/>
-    <mergeCell ref="A26:D26"/>
-    <mergeCell ref="A91:D91"/>
+    <mergeCell ref="A89:D89"/>
+    <mergeCell ref="A80:D80"/>
+    <mergeCell ref="A97:D97"/>
+    <mergeCell ref="A81:D81"/>
+    <mergeCell ref="A87:D87"/>
+    <mergeCell ref="A96:D96"/>
+    <mergeCell ref="A98:D98"/>
+    <mergeCell ref="A94:D94"/>
+    <mergeCell ref="A95:D95"/>
     <mergeCell ref="A76:D76"/>
-    <mergeCell ref="A32:D32"/>
-    <mergeCell ref="A66:D66"/>
-    <mergeCell ref="A61:D61"/>
-    <mergeCell ref="A84:D84"/>
-    <mergeCell ref="A62:D62"/>
-    <mergeCell ref="A77:D77"/>
-    <mergeCell ref="A58:D58"/>
-    <mergeCell ref="A59:D59"/>
-    <mergeCell ref="A60:D60"/>
-    <mergeCell ref="A64:D64"/>
-    <mergeCell ref="A72:D72"/>
-    <mergeCell ref="A81:D81"/>
+    <mergeCell ref="A93:D93"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -11495,84 +11654,84 @@
       <c r="BI61" s="8"/>
     </row>
     <row r="63" spans="1:61" x14ac:dyDescent="0.25">
-      <c r="A63" s="182" t="s">
+      <c r="A63" s="204" t="s">
         <v>15</v>
       </c>
-      <c r="B63" s="174"/>
-      <c r="C63" s="174"/>
-      <c r="D63" s="174"/>
-      <c r="E63" s="174"/>
-      <c r="F63" s="174"/>
-      <c r="G63" s="174"/>
-      <c r="H63" s="174"/>
-      <c r="I63" s="174"/>
-      <c r="J63" s="174"/>
-      <c r="K63" s="174"/>
-      <c r="L63" s="174"/>
-      <c r="M63" s="174"/>
-      <c r="N63" s="174"/>
-      <c r="O63" s="174"/>
-      <c r="P63" s="174"/>
-      <c r="Q63" s="174"/>
-      <c r="R63" s="174"/>
-      <c r="S63" s="174"/>
-      <c r="T63" s="174"/>
-      <c r="U63" s="174"/>
-      <c r="V63" s="174"/>
-      <c r="W63" s="174"/>
-      <c r="X63" s="174"/>
+      <c r="B63" s="196"/>
+      <c r="C63" s="196"/>
+      <c r="D63" s="196"/>
+      <c r="E63" s="196"/>
+      <c r="F63" s="196"/>
+      <c r="G63" s="196"/>
+      <c r="H63" s="196"/>
+      <c r="I63" s="196"/>
+      <c r="J63" s="196"/>
+      <c r="K63" s="196"/>
+      <c r="L63" s="196"/>
+      <c r="M63" s="196"/>
+      <c r="N63" s="196"/>
+      <c r="O63" s="196"/>
+      <c r="P63" s="196"/>
+      <c r="Q63" s="196"/>
+      <c r="R63" s="196"/>
+      <c r="S63" s="196"/>
+      <c r="T63" s="196"/>
+      <c r="U63" s="196"/>
+      <c r="V63" s="196"/>
+      <c r="W63" s="196"/>
+      <c r="X63" s="196"/>
     </row>
     <row r="64" spans="1:61" x14ac:dyDescent="0.25">
-      <c r="A64" s="174"/>
-      <c r="B64" s="174"/>
-      <c r="C64" s="174"/>
-      <c r="D64" s="174"/>
-      <c r="E64" s="174"/>
-      <c r="F64" s="174"/>
-      <c r="G64" s="174"/>
-      <c r="H64" s="174"/>
-      <c r="I64" s="174"/>
-      <c r="J64" s="174"/>
-      <c r="K64" s="174"/>
-      <c r="L64" s="174"/>
-      <c r="M64" s="174"/>
-      <c r="N64" s="174"/>
-      <c r="O64" s="174"/>
-      <c r="P64" s="174"/>
-      <c r="Q64" s="174"/>
-      <c r="R64" s="174"/>
-      <c r="S64" s="174"/>
-      <c r="T64" s="174"/>
-      <c r="U64" s="174"/>
-      <c r="V64" s="174"/>
-      <c r="W64" s="174"/>
-      <c r="X64" s="174"/>
+      <c r="A64" s="196"/>
+      <c r="B64" s="196"/>
+      <c r="C64" s="196"/>
+      <c r="D64" s="196"/>
+      <c r="E64" s="196"/>
+      <c r="F64" s="196"/>
+      <c r="G64" s="196"/>
+      <c r="H64" s="196"/>
+      <c r="I64" s="196"/>
+      <c r="J64" s="196"/>
+      <c r="K64" s="196"/>
+      <c r="L64" s="196"/>
+      <c r="M64" s="196"/>
+      <c r="N64" s="196"/>
+      <c r="O64" s="196"/>
+      <c r="P64" s="196"/>
+      <c r="Q64" s="196"/>
+      <c r="R64" s="196"/>
+      <c r="S64" s="196"/>
+      <c r="T64" s="196"/>
+      <c r="U64" s="196"/>
+      <c r="V64" s="196"/>
+      <c r="W64" s="196"/>
+      <c r="X64" s="196"/>
     </row>
     <row r="65" spans="1:24" x14ac:dyDescent="0.25">
-      <c r="A65" s="174"/>
-      <c r="B65" s="174"/>
-      <c r="C65" s="174"/>
-      <c r="D65" s="174"/>
-      <c r="E65" s="174"/>
-      <c r="F65" s="174"/>
-      <c r="G65" s="174"/>
-      <c r="H65" s="174"/>
-      <c r="I65" s="174"/>
-      <c r="J65" s="174"/>
-      <c r="K65" s="174"/>
-      <c r="L65" s="174"/>
-      <c r="M65" s="174"/>
-      <c r="N65" s="174"/>
-      <c r="O65" s="174"/>
-      <c r="P65" s="174"/>
-      <c r="Q65" s="174"/>
-      <c r="R65" s="174"/>
-      <c r="S65" s="174"/>
-      <c r="T65" s="174"/>
-      <c r="U65" s="174"/>
-      <c r="V65" s="174"/>
-      <c r="W65" s="174"/>
-      <c r="X65" s="174"/>
+      <c r="A65" s="196"/>
+      <c r="B65" s="196"/>
+      <c r="C65" s="196"/>
+      <c r="D65" s="196"/>
+      <c r="E65" s="196"/>
+      <c r="F65" s="196"/>
+      <c r="G65" s="196"/>
+      <c r="H65" s="196"/>
+      <c r="I65" s="196"/>
+      <c r="J65" s="196"/>
+      <c r="K65" s="196"/>
+      <c r="L65" s="196"/>
+      <c r="M65" s="196"/>
+      <c r="N65" s="196"/>
+      <c r="O65" s="196"/>
+      <c r="P65" s="196"/>
+      <c r="Q65" s="196"/>
+      <c r="R65" s="196"/>
+      <c r="S65" s="196"/>
+      <c r="T65" s="196"/>
+      <c r="U65" s="196"/>
+      <c r="V65" s="196"/>
+      <c r="W65" s="196"/>
+      <c r="X65" s="196"/>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -11594,12 +11753,12 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:4" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="A1" s="173" t="s">
+      <c r="A1" s="195" t="s">
         <v>16</v>
       </c>
-      <c r="B1" s="174"/>
-      <c r="C1" s="174"/>
-      <c r="D1" s="174"/>
+      <c r="B1" s="196"/>
+      <c r="C1" s="196"/>
+      <c r="D1" s="196"/>
     </row>
     <row r="3" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="9" t="s">
@@ -11724,18 +11883,18 @@
       </c>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A14" s="182" t="s">
+      <c r="A14" s="204" t="s">
         <v>41</v>
       </c>
-      <c r="B14" s="174"/>
-      <c r="C14" s="174"/>
-      <c r="D14" s="174"/>
+      <c r="B14" s="196"/>
+      <c r="C14" s="196"/>
+      <c r="D14" s="196"/>
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A15" s="174"/>
-      <c r="B15" s="174"/>
-      <c r="C15" s="174"/>
-      <c r="D15" s="174"/>
+      <c r="A15" s="196"/>
+      <c r="B15" s="196"/>
+      <c r="C15" s="196"/>
+      <c r="D15" s="196"/>
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A16" s="161"/>
@@ -11750,6 +11909,210 @@
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{66E88D20-B666-4530-AFCA-447DE0755752}">
+  <dimension ref="A1:D15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="24" customWidth="1"/>
+    <col min="2" max="2" width="14" customWidth="1"/>
+    <col min="3" max="3" width="42" customWidth="1"/>
+    <col min="4" max="4" width="54" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:4" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="A1" s="195" t="s">
+        <v>198</v>
+      </c>
+      <c r="B1" s="196"/>
+      <c r="C1" s="196"/>
+      <c r="D1" s="196"/>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A2" s="197" t="s">
+        <v>197</v>
+      </c>
+      <c r="B2" s="196"/>
+      <c r="C2" s="196"/>
+      <c r="D2" s="196"/>
+    </row>
+    <row r="4" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A4" s="9" t="s">
+        <v>196</v>
+      </c>
+      <c r="B4" s="9" t="s">
+        <v>195</v>
+      </c>
+      <c r="C4" s="9" t="s">
+        <v>194</v>
+      </c>
+      <c r="D4" s="9" t="s">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A5" s="207" t="s">
+        <v>192</v>
+      </c>
+      <c r="B5" s="206" t="s">
+        <v>191</v>
+      </c>
+      <c r="C5" s="205" t="s">
+        <v>190</v>
+      </c>
+      <c r="D5" s="205" t="s">
+        <v>189</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A6" s="207" t="s">
+        <v>188</v>
+      </c>
+      <c r="B6" s="206" t="s">
+        <v>187</v>
+      </c>
+      <c r="C6" s="205" t="s">
+        <v>186</v>
+      </c>
+      <c r="D6" s="205" t="s">
+        <v>185</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A7" s="207" t="s">
+        <v>60</v>
+      </c>
+      <c r="B7" s="206" t="s">
+        <v>173</v>
+      </c>
+      <c r="C7" s="205" t="s">
+        <v>184</v>
+      </c>
+      <c r="D7" s="205" t="s">
+        <v>183</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A8" s="207" t="s">
+        <v>182</v>
+      </c>
+      <c r="B8" s="206" t="s">
+        <v>163</v>
+      </c>
+      <c r="C8" s="205" t="s">
+        <v>181</v>
+      </c>
+      <c r="D8" s="205" t="s">
+        <v>180</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A9" s="207" t="s">
+        <v>58</v>
+      </c>
+      <c r="B9" s="206" t="s">
+        <v>173</v>
+      </c>
+      <c r="C9" s="205" t="s">
+        <v>179</v>
+      </c>
+      <c r="D9" s="205" t="s">
+        <v>178</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10" s="207" t="s">
+        <v>62</v>
+      </c>
+      <c r="B10" s="206" t="s">
+        <v>177</v>
+      </c>
+      <c r="C10" s="205" t="s">
+        <v>176</v>
+      </c>
+      <c r="D10" s="205" t="s">
+        <v>175</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A11" s="207" t="s">
+        <v>174</v>
+      </c>
+      <c r="B11" s="206" t="s">
+        <v>173</v>
+      </c>
+      <c r="C11" s="205" t="s">
+        <v>172</v>
+      </c>
+      <c r="D11" s="205" t="s">
+        <v>171</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A12" s="207" t="s">
+        <v>155</v>
+      </c>
+      <c r="B12" s="206" t="s">
+        <v>163</v>
+      </c>
+      <c r="C12" s="205" t="s">
+        <v>170</v>
+      </c>
+      <c r="D12" s="205" t="s">
+        <v>169</v>
+      </c>
+    </row>
+    <row r="13" spans="1:4" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A13" s="207" t="s">
+        <v>157</v>
+      </c>
+      <c r="B13" s="206" t="s">
+        <v>163</v>
+      </c>
+      <c r="C13" s="205" t="s">
+        <v>168</v>
+      </c>
+      <c r="D13" s="205" t="s">
+        <v>167</v>
+      </c>
+    </row>
+    <row r="14" spans="1:4" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A14" s="207" t="s">
+        <v>159</v>
+      </c>
+      <c r="B14" s="206" t="s">
+        <v>163</v>
+      </c>
+      <c r="C14" s="205" t="s">
+        <v>166</v>
+      </c>
+      <c r="D14" s="205" t="s">
+        <v>165</v>
+      </c>
+    </row>
+    <row r="15" spans="1:4" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A15" s="207" t="s">
+        <v>164</v>
+      </c>
+      <c r="B15" s="206" t="s">
+        <v>163</v>
+      </c>
+      <c r="C15" s="205" t="s">
+        <v>162</v>
+      </c>
+      <c r="D15" s="205" t="s">
+        <v>161</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A1:D1"/>
+    <mergeCell ref="A2:D2"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0500-000000000000}">
   <dimension ref="A1:G27"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -12021,24 +12384,24 @@
       <c r="G24" s="32"/>
     </row>
     <row r="26" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A26" s="182" t="s">
+      <c r="A26" s="204" t="s">
         <v>143</v>
       </c>
-      <c r="B26" s="174"/>
-      <c r="C26" s="174"/>
-      <c r="D26" s="174"/>
-      <c r="E26" s="174"/>
-      <c r="F26" s="174"/>
-      <c r="G26" s="174"/>
+      <c r="B26" s="196"/>
+      <c r="C26" s="196"/>
+      <c r="D26" s="196"/>
+      <c r="E26" s="196"/>
+      <c r="F26" s="196"/>
+      <c r="G26" s="196"/>
     </row>
     <row r="27" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A27" s="174"/>
-      <c r="B27" s="174"/>
-      <c r="C27" s="174"/>
-      <c r="D27" s="174"/>
-      <c r="E27" s="174"/>
-      <c r="F27" s="174"/>
-      <c r="G27" s="174"/>
+      <c r="A27" s="196"/>
+      <c r="B27" s="196"/>
+      <c r="C27" s="196"/>
+      <c r="D27" s="196"/>
+      <c r="E27" s="196"/>
+      <c r="F27" s="196"/>
+      <c r="G27" s="196"/>
     </row>
   </sheetData>
   <mergeCells count="1">

</xml_diff>